<commit_message>
Remove extra KS J links from pesticide and fertilizer manufacturing
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -833,7 +833,7 @@
       </c>
       <c r="K13" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050, 2000, 8010</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050, 2000, 8010</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
     </row>
@@ -16013,54 +16013,54 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">221</t>
+          <t xml:space="preserve">222</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 제조업</t>
+          <t xml:space="preserve">바이오비료 제조업</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">미생물·생물학적 비료 제제 제조</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">221</t>
+          <t xml:space="preserve">223</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 제조업</t>
+          <t xml:space="preserve">바이오사료 제조업</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -16070,61 +16070,61 @@
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">보조사료·사료첨가제 제조분; 단미사료 제외</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">222</t>
+          <t xml:space="preserve">223</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 제조업</t>
+          <t xml:space="preserve">바이오사료 제조업</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 비료 제제 제조</t>
+          <t xml:space="preserve">첨가제 외 바이오사료 제조분</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">222</t>
+          <t xml:space="preserve">223</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 제조업</t>
+          <t xml:space="preserve">바이오사료 제조업</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -16134,29 +16134,29 @@
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">222</t>
+          <t xml:space="preserve">229</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -16166,29 +16166,29 @@
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">생분해성 농업용 필름·용기</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">223</t>
+          <t xml:space="preserve">229</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -16198,29 +16198,29 @@
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">보조사료·사료첨가제 제조분; 단미사료 제외</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">223</t>
+          <t xml:space="preserve">229</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -16230,61 +16230,61 @@
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제 외 바이오사료 제조분</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">223</t>
+          <t xml:space="preserve">231</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 제조업</t>
+          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">생명공학 기반 식품첨가물 제조</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">229</t>
+          <t xml:space="preserve">231</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
+          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -16294,51 +16294,51 @@
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 필름·용기</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">229</t>
+          <t xml:space="preserve">232</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
+          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재</t>
+          <t xml:space="preserve">제어발효 등 바이오 발효식품 제조</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">229</t>
+          <t xml:space="preserve">232</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
+          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
@@ -16365,22 +16365,22 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">231</t>
+          <t xml:space="preserve">233</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
@@ -16390,19 +16390,19 @@
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생명공학 기반 식품첨가물 제조</t>
+          <t xml:space="preserve">법정 건강기능식품 제조</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">231</t>
+          <t xml:space="preserve">233</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
@@ -16429,44 +16429,44 @@
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">232</t>
+          <t xml:space="preserve">234</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">제어발효 등 바이오 발효식품 제조</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">232</t>
+          <t xml:space="preserve">234</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
@@ -16493,44 +16493,44 @@
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">233</t>
+          <t xml:space="preserve">235</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
+          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">법정 건강기능식품 제조</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">233</t>
+          <t xml:space="preserve">235</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
+          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
@@ -16557,12 +16557,12 @@
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">234</t>
+          <t xml:space="preserve">239</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
@@ -16582,19 +16582,19 @@
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 제품</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">234</t>
+          <t xml:space="preserve">239</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
@@ -16621,44 +16621,44 @@
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">235</t>
+          <t xml:space="preserve">240</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">동물용 바이오의약품·백신 제조</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">235</t>
+          <t xml:space="preserve">240</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
@@ -16685,44 +16685,44 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">239</t>
+          <t xml:space="preserve">291</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
+          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 제품</t>
+          <t xml:space="preserve">바이오화장품·향장제품 제조</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">239</t>
+          <t xml:space="preserve">291</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
+          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
@@ -16749,54 +16749,54 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">240</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품·백신 제조</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">240</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -16806,51 +16806,51 @@
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">바이오고분자 생활소재</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">291</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·향장제품 제조</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">291</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
@@ -16877,22 +16877,22 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -16902,29 +16902,29 @@
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">바이오고분자 산업용 제품</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -16934,29 +16934,29 @@
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 생활소재</t>
+          <t xml:space="preserve">그 밖의 바이오화학 제품</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -16966,19 +16966,19 @@
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">바이오환경 제품에 속하는 잔여범위</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
@@ -17005,86 +17005,86 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">7010</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">종자 및 묘목</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 산업용 제품</t>
+          <t xml:space="preserve">취급품목이 종자·묘목일 때의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 제품</t>
+          <t xml:space="preserve">그 밖의 생물자원 취급품목 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
@@ -17094,93 +17094,93 @@
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오환경 제품에 속하는 잔여범위</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">321</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">바이오농약 판매업</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">321</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">바이오농약 판매업</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목이 종자·묘목일 때의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">322</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">바이오비료 판매업</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -17190,19 +17190,19 @@
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생물자원 취급품목 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">322</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">바이오비료 판매업</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
@@ -17229,22 +17229,22 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">321</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 판매업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -17254,157 +17254,157 @@
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">취급품목이 사료첨가제일 때의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">321</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 판매업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">첨가제 외 바이오사료의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">322</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 판매업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">322</t>
+          <t xml:space="preserve">329</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">바이오화학 농자재 취급품목 분야; 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">329</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목이 사료첨가제일 때의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">331</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
@@ -17414,19 +17414,19 @@
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제 외 바이오사료의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">331</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
@@ -17453,22 +17453,22 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">329</t>
+          <t xml:space="preserve">332</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
+          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
@@ -17478,19 +17478,19 @@
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화학 농자재 취급품목 분야; 품목에 따라 재판정</t>
+          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 맞춤형 판매방식 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">329</t>
+          <t xml:space="preserve">332</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
+          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
@@ -17517,22 +17517,22 @@
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">331</t>
+          <t xml:space="preserve">333</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
@@ -17542,19 +17542,19 @@
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">331</t>
+          <t xml:space="preserve">333</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
@@ -17574,29 +17574,29 @@
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 위탁제조 판매만으로 8010 아님</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">332</t>
+          <t xml:space="preserve">339</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -17606,19 +17606,19 @@
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 맞춤형 판매방식 전용 코드 없음</t>
+          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">332</t>
+          <t xml:space="preserve">339</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
@@ -17645,22 +17645,22 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">333</t>
+          <t xml:space="preserve">341</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
@@ -17670,19 +17670,19 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
+          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야; 도매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">333</t>
+          <t xml:space="preserve">341</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
@@ -17702,29 +17702,29 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 위탁제조 판매만으로 8010 아님</t>
+          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">339</t>
+          <t xml:space="preserve">342</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
@@ -17734,19 +17734,19 @@
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
+          <t xml:space="preserve">자기 상표 위탁제조 동물용 의약품의 제품 분야; 판매형태 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">339</t>
+          <t xml:space="preserve">342</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
@@ -17766,125 +17766,125 @@
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분; 제조를 맡기는 발주자는 8010 아님</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">341</t>
+          <t xml:space="preserve">390</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
+          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야; 도매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 처리·보관·배송 서비스 수행분만 대응; 판매품목 확인 전 제품 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">341</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">7010</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">종자 및 묘목</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분</t>
+          <t xml:space="preserve">종자·묘목 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">342</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">7020</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">유전자 변형 생물체</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">자기 상표 위탁제조 동물용 의약품의 제품 분야; 판매형태 전용 코드 없음</t>
+          <t xml:space="preserve">유전자변형 생물체 개발분</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">342</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
@@ -17894,115 +17894,115 @@
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분; 제조를 맡기는 발주자는 8010 아님</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">390</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 처리·보관·배송 서비스 수행분만 대응; 판매품목 확인 전 제품 코드 없음</t>
+          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자·묘목 자체의 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7020</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자 변형 생물체</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자변형 생물체 개발분</t>
+          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
@@ -18029,12 +18029,12 @@
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
@@ -18049,24 +18049,24 @@
       </c>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
@@ -18093,22 +18093,22 @@
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
@@ -18118,29 +18118,29 @@
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
@@ -18150,29 +18150,29 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
@@ -18182,93 +18182,93 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
+          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
@@ -18278,29 +18278,29 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
@@ -18310,61 +18310,61 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
+          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
@@ -18374,29 +18374,29 @@
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -18406,29 +18406,29 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -18438,29 +18438,29 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,29 +18470,29 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
@@ -18502,29 +18502,29 @@
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품용 미생물·효소 소재</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -18534,29 +18534,29 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
+          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
@@ -18566,19 +18566,19 @@
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
+          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
@@ -18605,54 +18605,54 @@
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 소재</t>
+          <t xml:space="preserve">건강기능식품 제품 개발</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18662,61 +18662,61 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
+          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -18726,61 +18726,61 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">발효식품 제품기술 개발</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강기능식품 제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -18790,61 +18790,61 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -18854,19 +18854,19 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효식품 제품기술 개발</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
@@ -18893,12 +18893,12 @@
     <row r="119">
       <c r="A119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
@@ -18918,19 +18918,19 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr">
@@ -18957,54 +18957,54 @@
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">동물용 바이오백신 개발</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E122" s="8" t="inlineStr">
@@ -19014,29 +19014,29 @@
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E123" s="8" t="inlineStr">
@@ -19046,93 +19046,93 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오백신 개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E126" s="8" t="inlineStr">
@@ -19142,93 +19142,93 @@
       </c>
       <c r="F126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E129" s="8" t="inlineStr">
@@ -19238,29 +19238,29 @@
       </c>
       <c r="F129" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E130" s="8" t="inlineStr">
@@ -19270,51 +19270,51 @@
       </c>
       <c r="F130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C132" s="8" t="inlineStr">
@@ -19341,22 +19341,22 @@
     <row r="133">
       <c r="A133" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E133" s="8" t="inlineStr">
@@ -19366,29 +19366,29 @@
       </c>
       <c r="F133" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E134" s="8" t="inlineStr">
@@ -19398,29 +19398,29 @@
       </c>
       <c r="F134" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C135" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E135" s="8" t="inlineStr">
@@ -19430,19 +19430,19 @@
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
@@ -19469,22 +19469,22 @@
     <row r="137">
       <c r="A137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E137" s="8" t="inlineStr">
@@ -19494,29 +19494,29 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E138" s="8" t="inlineStr">
@@ -19526,29 +19526,29 @@
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E139" s="8" t="inlineStr">
@@ -19558,29 +19558,29 @@
       </c>
       <c r="F139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C140" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E140" s="8" t="inlineStr">
@@ -19590,29 +19590,29 @@
       </c>
       <c r="F140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E141" s="8" t="inlineStr">
@@ -19622,29 +19622,29 @@
       </c>
       <c r="F141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E142" s="8" t="inlineStr">
@@ -19654,29 +19654,29 @@
       </c>
       <c r="F142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E143" s="8" t="inlineStr">
@@ -19686,29 +19686,29 @@
       </c>
       <c r="F143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B144" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D144" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E144" s="8" t="inlineStr">
@@ -19718,29 +19718,29 @@
       </c>
       <c r="F144" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">생물학적 폐자원 처리·재활용 제제 또는 시스템 제공분</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B145" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D145" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E145" s="8" t="inlineStr">
@@ -19750,29 +19750,29 @@
       </c>
       <c r="F145" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B146" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C146" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D146" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E146" s="8" t="inlineStr">
@@ -19782,29 +19782,29 @@
       </c>
       <c r="F146" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">그 밖의 바이오환경 서비스; 독립 처리수수료 사업 전체를 직접 포괄하지 않음</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B147" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D147" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E147" s="8" t="inlineStr">
@@ -19814,29 +19814,29 @@
       </c>
       <c r="F147" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B148" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D148" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E148" s="8" t="inlineStr">
@@ -19846,29 +19846,29 @@
       </c>
       <c r="F148" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물학적 폐자원 처리·재활용 제제 또는 시스템 제공분</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B149" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C149" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D149" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E149" s="8" t="inlineStr">
@@ -19878,29 +19878,29 @@
       </c>
       <c r="F149" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B150" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C150" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D150" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E150" s="8" t="inlineStr">
@@ -19910,29 +19910,29 @@
       </c>
       <c r="F150" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오환경 서비스; 독립 처리수수료 사업 전체를 직접 포괄하지 않음</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B151" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D151" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E151" s="8" t="inlineStr">
@@ -19942,29 +19942,29 @@
       </c>
       <c r="F151" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B152" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D152" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E152" s="8" t="inlineStr">
@@ -19973,134 +19973,6 @@
         </is>
       </c>
       <c r="F152" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B153" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C153" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8020</t>
-        </is>
-      </c>
-      <c r="D153" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
-        </is>
-      </c>
-      <c r="E153" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F153" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B154" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C154" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8030</t>
-        </is>
-      </c>
-      <c r="D154" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E154" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F154" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B155" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C155" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8050</t>
-        </is>
-      </c>
-      <c r="D155" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
-        </is>
-      </c>
-      <c r="E155" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F155" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B156" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C156" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D156" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E156" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F156" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Remove extra KS J links from biofeed manufacturing
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -947,7 +947,7 @@
       </c>
       <c r="K15" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050, 3000, 8010</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
     </row>
@@ -16077,22 +16077,22 @@
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">223</t>
+          <t xml:space="preserve">229</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -16102,29 +16102,29 @@
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제 외 바이오사료 제조분</t>
+          <t xml:space="preserve">생분해성 농업용 필름·용기</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">223</t>
+          <t xml:space="preserve">229</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재</t>
         </is>
       </c>
     </row>
@@ -16151,12 +16151,12 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -16166,51 +16166,51 @@
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 필름·용기</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">229</t>
+          <t xml:space="preserve">231</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
+          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재</t>
+          <t xml:space="preserve">생명공학 기반 식품첨가물 제조</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">229</t>
+          <t xml:space="preserve">231</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
+          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
@@ -16237,22 +16237,22 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">231</t>
+          <t xml:space="preserve">232</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
+          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
@@ -16262,19 +16262,19 @@
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생명공학 기반 식품첨가물 제조</t>
+          <t xml:space="preserve">제어발효 등 바이오 발효식품 제조</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">231</t>
+          <t xml:space="preserve">232</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
+          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
@@ -16301,22 +16301,22 @@
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">232</t>
+          <t xml:space="preserve">233</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -16326,19 +16326,19 @@
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">제어발효 등 바이오 발효식품 제조</t>
+          <t xml:space="preserve">법정 건강기능식품 제조</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">232</t>
+          <t xml:space="preserve">233</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
@@ -16365,44 +16365,44 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">233</t>
+          <t xml:space="preserve">234</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">법정 건강기능식품 제조</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">233</t>
+          <t xml:space="preserve">234</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
@@ -16429,12 +16429,12 @@
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">234</t>
+          <t xml:space="preserve">235</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
+          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
@@ -16454,19 +16454,19 @@
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">234</t>
+          <t xml:space="preserve">235</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
+          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
@@ -16493,12 +16493,12 @@
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">235</t>
+          <t xml:space="preserve">239</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
@@ -16518,19 +16518,19 @@
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 제품</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">235</t>
+          <t xml:space="preserve">239</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
@@ -16557,44 +16557,44 @@
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">239</t>
+          <t xml:space="preserve">240</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 제품</t>
+          <t xml:space="preserve">동물용 바이오의약품·백신 제조</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">239</t>
+          <t xml:space="preserve">240</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
@@ -16621,22 +16621,22 @@
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">240</t>
+          <t xml:space="preserve">291</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
+          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -16646,19 +16646,19 @@
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품·백신 제조</t>
+          <t xml:space="preserve">바이오화장품·향장제품 제조</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">240</t>
+          <t xml:space="preserve">291</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
+          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
@@ -16685,12 +16685,12 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">291</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
@@ -16705,34 +16705,34 @@
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·향장제품 제조</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">291</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -16742,7 +16742,7 @@
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">바이오고분자 생활소재</t>
         </is>
       </c>
     </row>
@@ -16759,12 +16759,12 @@
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
@@ -16774,7 +16774,7 @@
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
@@ -16791,12 +16791,12 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -16806,29 +16806,29 @@
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 생활소재</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -16838,29 +16838,29 @@
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">바이오고분자 산업용 제품</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -16870,7 +16870,7 @@
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">그 밖의 바이오화학 제품</t>
         </is>
       </c>
     </row>
@@ -16887,12 +16887,12 @@
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 산업용 제품</t>
+          <t xml:space="preserve">바이오환경 제품에 속하는 잔여범위</t>
         </is>
       </c>
     </row>
@@ -16919,12 +16919,12 @@
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -16934,71 +16934,71 @@
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 제품</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">7010</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">종자 및 묘목</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오환경 제품에 속하는 잔여범위</t>
+          <t xml:space="preserve">취급품목이 종자·묘목일 때의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">그 밖의 생물자원 취급품목 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
@@ -17015,44 +17015,44 @@
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목이 종자·묘목일 때의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">321</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">바이오농약 판매업</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -17062,19 +17062,19 @@
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생물자원 취급품목 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">321</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">바이오농약 판매업</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -17101,12 +17101,12 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">321</t>
+          <t xml:space="preserve">322</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 판매업</t>
+          <t xml:space="preserve">바이오비료 판매업</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
@@ -17126,19 +17126,19 @@
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">321</t>
+          <t xml:space="preserve">322</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 판매업</t>
+          <t xml:space="preserve">바이오비료 판매업</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
@@ -17165,22 +17165,22 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">322</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 판매업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -17190,39 +17190,39 @@
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">취급품목이 사료첨가제일 때의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">322</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 판매업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">첨가제 외 바이오사료의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
@@ -17239,44 +17239,44 @@
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목이 사료첨가제일 때의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">329</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
@@ -17286,19 +17286,19 @@
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제 외 바이오사료의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">바이오화학 농자재 취급품목 분야; 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">329</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
@@ -17325,22 +17325,22 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">329</t>
+          <t xml:space="preserve">331</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
@@ -17350,19 +17350,19 @@
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화학 농자재 취급품목 분야; 품목에 따라 재판정</t>
+          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">329</t>
+          <t xml:space="preserve">331</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
@@ -17389,12 +17389,12 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">331</t>
+          <t xml:space="preserve">332</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
@@ -17414,19 +17414,19 @@
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 맞춤형 판매방식 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">331</t>
+          <t xml:space="preserve">332</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
@@ -17453,22 +17453,22 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">332</t>
+          <t xml:space="preserve">333</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
@@ -17478,19 +17478,19 @@
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 맞춤형 판매방식 전용 코드 없음</t>
+          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">332</t>
+          <t xml:space="preserve">333</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
@@ -17510,19 +17510,19 @@
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 위탁제조 판매만으로 8010 아님</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">333</t>
+          <t xml:space="preserve">339</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
@@ -17549,12 +17549,12 @@
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">333</t>
+          <t xml:space="preserve">339</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
@@ -17574,29 +17574,29 @@
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 위탁제조 판매만으로 8010 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">339</t>
+          <t xml:space="preserve">341</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -17606,19 +17606,19 @@
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
+          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야; 도매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">339</t>
+          <t xml:space="preserve">341</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
@@ -17638,19 +17638,19 @@
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">341</t>
+          <t xml:space="preserve">342</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
@@ -17670,19 +17670,19 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야; 도매업 자체의 대응 아님</t>
+          <t xml:space="preserve">자기 상표 위탁제조 동물용 의약품의 제품 분야; 판매형태 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">341</t>
+          <t xml:space="preserve">342</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
@@ -17702,93 +17702,93 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분</t>
+          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분; 제조를 맡기는 발주자는 8010 아님</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">342</t>
+          <t xml:space="preserve">390</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
+          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">자기 상표 위탁제조 동물용 의약품의 제품 분야; 판매형태 전용 코드 없음</t>
+          <t xml:space="preserve">별도 생물류 처리·보관·배송 서비스 수행분만 대응; 판매품목 확인 전 제품 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">342</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">7010</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">종자 및 묘목</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분; 제조를 맡기는 발주자는 8010 아님</t>
+          <t xml:space="preserve">종자·묘목 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">390</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">7020</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">유전자 변형 생물체</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
@@ -17798,7 +17798,7 @@
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 처리·보관·배송 서비스 수행분만 대응; 판매품목 확인 전 제품 코드 없음</t>
+          <t xml:space="preserve">유전자변형 생물체 개발분</t>
         </is>
       </c>
     </row>
@@ -17815,66 +17815,66 @@
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자·묘목 자체의 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7020</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자 변형 생물체</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자변형 생물체 개발분</t>
+          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
@@ -17901,12 +17901,12 @@
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
@@ -17926,19 +17926,19 @@
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
@@ -17965,12 +17965,12 @@
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
@@ -17985,24 +17985,24 @@
       </c>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
@@ -18029,54 +18029,54 @@
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
+          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -18086,7 +18086,7 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
@@ -18103,76 +18103,76 @@
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
@@ -18182,7 +18182,7 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
@@ -18199,44 +18199,44 @@
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -18246,29 +18246,29 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
@@ -18278,7 +18278,7 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
         </is>
       </c>
     </row>
@@ -18295,12 +18295,12 @@
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
@@ -18310,29 +18310,29 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -18342,29 +18342,29 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
+          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
         </is>
       </c>
     </row>
@@ -18391,12 +18391,12 @@
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -18406,29 +18406,29 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -18438,29 +18438,29 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
+          <t xml:space="preserve">식품용 미생물·효소 소재</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,7 +18470,7 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
         </is>
       </c>
     </row>
@@ -18487,12 +18487,12 @@
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 소재</t>
+          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
         </is>
       </c>
     </row>
@@ -18519,12 +18519,12 @@
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -18534,51 +18534,51 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
+          <t xml:space="preserve">건강기능식품 제품 개발</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
@@ -18605,22 +18605,22 @@
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -18630,29 +18630,29 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강기능식품 제품 개발</t>
+          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18662,7 +18662,7 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">발효식품 제품기술 개발</t>
         </is>
       </c>
     </row>
@@ -18679,44 +18679,44 @@
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -18726,19 +18726,19 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효식품 제품기술 개발</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
@@ -18765,12 +18765,12 @@
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
@@ -18790,19 +18790,19 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
@@ -18829,12 +18829,12 @@
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
@@ -18854,19 +18854,19 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
@@ -18893,54 +18893,54 @@
     <row r="119">
       <c r="A119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
+          <t xml:space="preserve">동물용 바이오백신 개발</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E120" s="8" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="F120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -18967,76 +18967,76 @@
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오백신 개발</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E123" s="8" t="inlineStr">
@@ -19046,7 +19046,7 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -19063,66 +19063,66 @@
       </c>
       <c r="C124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
@@ -19142,19 +19142,19 @@
       </c>
       <c r="F126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
@@ -19169,34 +19169,34 @@
       </c>
       <c r="E127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E128" s="8" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="F128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
@@ -19223,12 +19223,12 @@
       </c>
       <c r="C129" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E129" s="8" t="inlineStr">
@@ -19238,7 +19238,7 @@
       </c>
       <c r="F129" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
@@ -19255,12 +19255,12 @@
       </c>
       <c r="C130" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E130" s="8" t="inlineStr">
@@ -19270,29 +19270,29 @@
       </c>
       <c r="F130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E131" s="8" t="inlineStr">
@@ -19302,29 +19302,29 @@
       </c>
       <c r="F131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C132" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E132" s="8" t="inlineStr">
@@ -19334,7 +19334,7 @@
       </c>
       <c r="F132" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
@@ -19351,12 +19351,12 @@
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E133" s="8" t="inlineStr">
@@ -19366,7 +19366,7 @@
       </c>
       <c r="F133" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
@@ -19383,12 +19383,12 @@
       </c>
       <c r="C134" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E134" s="8" t="inlineStr">
@@ -19398,29 +19398,29 @@
       </c>
       <c r="F134" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C135" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E135" s="8" t="inlineStr">
@@ -19430,29 +19430,29 @@
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E136" s="8" t="inlineStr">
@@ -19462,19 +19462,19 @@
       </c>
       <c r="F136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
@@ -19494,29 +19494,29 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E138" s="8" t="inlineStr">
@@ -19526,29 +19526,29 @@
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E139" s="8" t="inlineStr">
@@ -19558,19 +19558,19 @@
       </c>
       <c r="F139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C140" s="8" t="inlineStr">
@@ -19590,19 +19590,19 @@
       </c>
       <c r="F140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C141" s="8" t="inlineStr">
@@ -19622,29 +19622,29 @@
       </c>
       <c r="F141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E142" s="8" t="inlineStr">
@@ -19654,29 +19654,29 @@
       </c>
       <c r="F142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">생물학적 폐자원 처리·재활용 제제 또는 시스템 제공분</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E143" s="8" t="inlineStr">
@@ -19686,7 +19686,7 @@
       </c>
       <c r="F143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
@@ -19703,12 +19703,12 @@
       </c>
       <c r="C144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D144" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E144" s="8" t="inlineStr">
@@ -19718,29 +19718,29 @@
       </c>
       <c r="F144" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물학적 폐자원 처리·재활용 제제 또는 시스템 제공분</t>
+          <t xml:space="preserve">그 밖의 바이오환경 서비스; 독립 처리수수료 사업 전체를 직접 포괄하지 않음</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B145" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D145" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E145" s="8" t="inlineStr">
@@ -19750,29 +19750,29 @@
       </c>
       <c r="F145" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B146" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C146" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D146" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E146" s="8" t="inlineStr">
@@ -19782,29 +19782,29 @@
       </c>
       <c r="F146" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오환경 서비스; 독립 처리수수료 사업 전체를 직접 포괄하지 않음</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B147" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D147" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E147" s="8" t="inlineStr">
@@ -19814,29 +19814,29 @@
       </c>
       <c r="F147" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B148" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D148" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E148" s="8" t="inlineStr">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="F148" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
@@ -19863,12 +19863,12 @@
       </c>
       <c r="C149" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D149" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E149" s="8" t="inlineStr">
@@ -19878,7 +19878,7 @@
       </c>
       <c r="F149" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
@@ -19895,12 +19895,12 @@
       </c>
       <c r="C150" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D150" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E150" s="8" t="inlineStr">
@@ -19909,70 +19909,6 @@
         </is>
       </c>
       <c r="F150" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B151" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C151" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8050</t>
-        </is>
-      </c>
-      <c r="D151" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
-        </is>
-      </c>
-      <c r="E151" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F151" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B152" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C152" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D152" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E152" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F152" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Remove contract manufacturing link from food additive manufacturing
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -1061,7 +1061,7 @@
       </c>
       <c r="K17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030, 8010</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
     </row>
@@ -16205,32 +16205,32 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">231</t>
+          <t xml:space="preserve">232</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
+          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">제어발효 등 바이오 발효식품 제조</t>
         </is>
       </c>
     </row>
@@ -16247,54 +16247,54 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">제어발효 등 바이오 발효식품 제조</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">232</t>
+          <t xml:space="preserve">233</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">법정 건강기능식품 제조</t>
         </is>
       </c>
     </row>
@@ -16311,44 +16311,44 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">법정 건강기능식품 제조</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">233</t>
+          <t xml:space="preserve">234</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -16358,7 +16358,7 @@
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
@@ -16375,12 +16375,12 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
@@ -16390,29 +16390,29 @@
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">234</t>
+          <t xml:space="preserve">235</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
+          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -16422,7 +16422,7 @@
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
@@ -16439,12 +16439,12 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
@@ -16454,29 +16454,29 @@
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">235</t>
+          <t xml:space="preserve">239</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -16486,7 +16486,7 @@
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 제품</t>
         </is>
       </c>
     </row>
@@ -16503,12 +16503,12 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -16518,39 +16518,39 @@
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 제품</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">239</t>
+          <t xml:space="preserve">240</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">동물용 바이오의약품·백신 제조</t>
         </is>
       </c>
     </row>
@@ -16567,54 +16567,54 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품·백신 제조</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">240</t>
+          <t xml:space="preserve">291</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
+          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">바이오화장품·향장제품 제조</t>
         </is>
       </c>
     </row>
@@ -16631,44 +16631,44 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·향장제품 제조</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">291</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -16678,7 +16678,7 @@
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
@@ -16695,12 +16695,12 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">바이오고분자 생활소재</t>
         </is>
       </c>
     </row>
@@ -16727,12 +16727,12 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -16742,7 +16742,7 @@
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 생활소재</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
@@ -16759,12 +16759,12 @@
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
@@ -16774,29 +16774,29 @@
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -16806,7 +16806,7 @@
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">바이오고분자 산업용 제품</t>
         </is>
       </c>
     </row>
@@ -16823,12 +16823,12 @@
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 산업용 제품</t>
+          <t xml:space="preserve">그 밖의 바이오화학 제품</t>
         </is>
       </c>
     </row>
@@ -16855,12 +16855,12 @@
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -16870,7 +16870,7 @@
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 제품</t>
+          <t xml:space="preserve">바이오환경 제품에 속하는 잔여범위</t>
         </is>
       </c>
     </row>
@@ -16887,12 +16887,12 @@
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -16902,39 +16902,39 @@
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오환경 제품에 속하는 잔여범위</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">7010</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">종자 및 묘목</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">취급품목이 종자·묘목일 때의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
@@ -16951,12 +16951,12 @@
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -16966,7 +16966,7 @@
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목이 종자·묘목일 때의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">그 밖의 생물자원 취급품목 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
@@ -16983,54 +16983,54 @@
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생물자원 취급품목 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">321</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">바이오농약 판매업</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
@@ -17047,54 +17047,54 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">321</t>
+          <t xml:space="preserve">322</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 판매업</t>
+          <t xml:space="preserve">바이오비료 판매업</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
@@ -17111,54 +17111,54 @@
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">322</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 판매업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급품목이 사료첨가제일 때의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
@@ -17175,12 +17175,12 @@
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -17190,7 +17190,7 @@
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목이 사료첨가제일 때의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">첨가제 외 바이오사료의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
@@ -17207,54 +17207,54 @@
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제 외 바이오사료의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">329</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">바이오화학 농자재 취급품목 분야; 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
@@ -17271,54 +17271,54 @@
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화학 농자재 취급품목 분야; 품목에 따라 재판정</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">329</t>
+          <t xml:space="preserve">331</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
@@ -17335,54 +17335,54 @@
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">331</t>
+          <t xml:space="preserve">332</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 맞춤형 판매방식 전용 코드 없음</t>
         </is>
       </c>
     </row>
@@ -17399,54 +17399,54 @@
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 맞춤형 판매방식 전용 코드 없음</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">332</t>
+          <t xml:space="preserve">333</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
         </is>
       </c>
     </row>
@@ -17463,54 +17463,54 @@
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 위탁제조 판매만으로 8010 아님</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">333</t>
+          <t xml:space="preserve">339</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 위탁제조 판매만으로 8010 아님</t>
+          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
         </is>
       </c>
     </row>
@@ -17527,54 +17527,54 @@
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">339</t>
+          <t xml:space="preserve">341</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야; 도매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
@@ -17591,54 +17591,54 @@
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야; 도매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">341</t>
+          <t xml:space="preserve">342</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분</t>
+          <t xml:space="preserve">자기 상표 위탁제조 동물용 의약품의 제품 분야; 판매형태 전용 코드 없음</t>
         </is>
       </c>
     </row>
@@ -17655,34 +17655,34 @@
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">자기 상표 위탁제조 동물용 의약품의 제품 분야; 판매형태 전용 코드 없음</t>
+          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분; 제조를 맡기는 발주자는 8010 아님</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">342</t>
+          <t xml:space="preserve">390</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
+          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
@@ -17702,39 +17702,39 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분; 제조를 맡기는 발주자는 8010 아님</t>
+          <t xml:space="preserve">별도 생물류 처리·보관·배송 서비스 수행분만 대응; 판매품목 확인 전 제품 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">390</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">7010</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">종자 및 묘목</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 처리·보관·배송 서비스 수행분만 대응; 판매품목 확인 전 제품 코드 없음</t>
+          <t xml:space="preserve">종자·묘목 자체의 개발</t>
         </is>
       </c>
     </row>
@@ -17751,22 +17751,22 @@
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">7020</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">유전자 변형 생물체</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자·묘목 자체의 개발</t>
+          <t xml:space="preserve">유전자변형 생물체 개발분</t>
         </is>
       </c>
     </row>
@@ -17783,12 +17783,12 @@
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7020</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자 변형 생물체</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
@@ -17798,39 +17798,39 @@
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자변형 생물체 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
@@ -17847,54 +17847,54 @@
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
@@ -17911,44 +17911,44 @@
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
@@ -17958,7 +17958,7 @@
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
         </is>
       </c>
     </row>
@@ -17975,12 +17975,12 @@
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
@@ -17990,39 +17990,39 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
         </is>
       </c>
     </row>
@@ -18039,22 +18039,22 @@
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
+          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
@@ -18071,12 +18071,12 @@
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -18086,39 +18086,39 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
         </is>
       </c>
     </row>
@@ -18135,22 +18135,22 @@
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
+          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
@@ -18167,12 +18167,12 @@
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
@@ -18182,29 +18182,29 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -18214,7 +18214,7 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
         </is>
       </c>
     </row>
@@ -18231,12 +18231,12 @@
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -18246,7 +18246,7 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
+          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
         </is>
       </c>
     </row>
@@ -18263,12 +18263,12 @@
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
@@ -18278,29 +18278,29 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
         </is>
       </c>
     </row>
@@ -18327,12 +18327,12 @@
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
         </is>
       </c>
     </row>
@@ -18359,12 +18359,12 @@
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
@@ -18374,29 +18374,29 @@
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -18406,7 +18406,7 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품용 미생물·효소 소재</t>
         </is>
       </c>
     </row>
@@ -18423,12 +18423,12 @@
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 소재</t>
+          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
         </is>
       </c>
     </row>
@@ -18455,12 +18455,12 @@
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,7 +18470,7 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
+          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
         </is>
       </c>
     </row>
@@ -18487,12 +18487,12 @@
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
@@ -18502,39 +18502,39 @@
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">건강기능식품 제품 개발</t>
         </is>
       </c>
     </row>
@@ -18551,54 +18551,54 @@
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강기능식품 제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
         </is>
       </c>
     </row>
@@ -18615,22 +18615,22 @@
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
+          <t xml:space="preserve">발효식품 제품기술 개발</t>
         </is>
       </c>
     </row>
@@ -18647,12 +18647,12 @@
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18662,29 +18662,29 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효식품 제품기술 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
@@ -18711,12 +18711,12 @@
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -18726,29 +18726,29 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
@@ -18775,12 +18775,12 @@
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -18790,29 +18790,29 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
@@ -18822,7 +18822,7 @@
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
         </is>
       </c>
     </row>
@@ -18839,12 +18839,12 @@
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -18854,39 +18854,39 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">동물용 바이오백신 개발</t>
         </is>
       </c>
     </row>
@@ -18903,22 +18903,22 @@
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오백신 개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -18935,12 +18935,12 @@
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E120" s="8" t="inlineStr">
@@ -18950,39 +18950,39 @@
       </c>
       <c r="F120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
@@ -18999,22 +18999,22 @@
       </c>
       <c r="C122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -19031,12 +19031,12 @@
       </c>
       <c r="C123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E123" s="8" t="inlineStr">
@@ -19046,39 +19046,39 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
@@ -19095,44 +19095,44 @@
       </c>
       <c r="C125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E126" s="8" t="inlineStr">
@@ -19142,7 +19142,7 @@
       </c>
       <c r="F126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
@@ -19159,12 +19159,12 @@
       </c>
       <c r="C127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E127" s="8" t="inlineStr">
@@ -19174,7 +19174,7 @@
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
@@ -19191,12 +19191,12 @@
       </c>
       <c r="C128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E128" s="8" t="inlineStr">
@@ -19206,7 +19206,7 @@
       </c>
       <c r="F128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
@@ -19223,12 +19223,12 @@
       </c>
       <c r="C129" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E129" s="8" t="inlineStr">
@@ -19238,29 +19238,29 @@
       </c>
       <c r="F129" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E130" s="8" t="inlineStr">
@@ -19270,7 +19270,7 @@
       </c>
       <c r="F130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
@@ -19287,12 +19287,12 @@
       </c>
       <c r="C131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E131" s="8" t="inlineStr">
@@ -19302,7 +19302,7 @@
       </c>
       <c r="F131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
@@ -19319,12 +19319,12 @@
       </c>
       <c r="C132" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E132" s="8" t="inlineStr">
@@ -19334,7 +19334,7 @@
       </c>
       <c r="F132" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
@@ -19351,12 +19351,12 @@
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E133" s="8" t="inlineStr">
@@ -19366,19 +19366,19 @@
       </c>
       <c r="F133" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr">
@@ -19398,7 +19398,7 @@
       </c>
       <c r="F134" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
@@ -19415,12 +19415,12 @@
       </c>
       <c r="C135" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E135" s="8" t="inlineStr">
@@ -19430,29 +19430,29 @@
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E136" s="8" t="inlineStr">
@@ -19462,29 +19462,29 @@
       </c>
       <c r="F136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E137" s="8" t="inlineStr">
@@ -19494,7 +19494,7 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
@@ -19511,12 +19511,12 @@
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E138" s="8" t="inlineStr">
@@ -19526,29 +19526,29 @@
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E139" s="8" t="inlineStr">
@@ -19558,7 +19558,7 @@
       </c>
       <c r="F139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
@@ -19575,12 +19575,12 @@
       </c>
       <c r="C140" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E140" s="8" t="inlineStr">
@@ -19590,29 +19590,29 @@
       </c>
       <c r="F140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E141" s="8" t="inlineStr">
@@ -19622,7 +19622,7 @@
       </c>
       <c r="F141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">생물학적 폐자원 처리·재활용 제제 또는 시스템 제공분</t>
         </is>
       </c>
     </row>
@@ -19639,12 +19639,12 @@
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E142" s="8" t="inlineStr">
@@ -19654,7 +19654,7 @@
       </c>
       <c r="F142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물학적 폐자원 처리·재활용 제제 또는 시스템 제공분</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
@@ -19671,12 +19671,12 @@
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E143" s="8" t="inlineStr">
@@ -19686,19 +19686,19 @@
       </c>
       <c r="F143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">그 밖의 바이오환경 서비스; 독립 처리수수료 사업 전체를 직접 포괄하지 않음</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B144" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C144" s="8" t="inlineStr">
@@ -19718,7 +19718,7 @@
       </c>
       <c r="F144" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오환경 서비스; 독립 처리수수료 사업 전체를 직접 포괄하지 않음</t>
+          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
         </is>
       </c>
     </row>
@@ -19735,12 +19735,12 @@
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D145" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E145" s="8" t="inlineStr">
@@ -19750,29 +19750,29 @@
       </c>
       <c r="F145" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B146" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C146" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D146" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E146" s="8" t="inlineStr">
@@ -19782,7 +19782,7 @@
       </c>
       <c r="F146" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
@@ -19799,12 +19799,12 @@
       </c>
       <c r="C147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D147" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E147" s="8" t="inlineStr">
@@ -19814,7 +19814,7 @@
       </c>
       <c r="F147" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
@@ -19831,12 +19831,12 @@
       </c>
       <c r="C148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D148" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E148" s="8" t="inlineStr">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="F148" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
@@ -19863,12 +19863,12 @@
       </c>
       <c r="C149" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D149" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E149" s="8" t="inlineStr">
@@ -19877,38 +19877,6 @@
         </is>
       </c>
       <c r="F149" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B150" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C150" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D150" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E150" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F150" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Remove contract manufacturing links from food classes
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -1118,7 +1118,7 @@
       </c>
       <c r="K18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040, 8010</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010, 8010</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000, 8010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="K21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000, 8010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="K22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000, 8010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
     </row>
@@ -16237,86 +16237,86 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">232</t>
+          <t xml:space="preserve">233</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">법정 건강기능식품 제조</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">233</t>
+          <t xml:space="preserve">234</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">법정 건강기능식품 제조</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">233</t>
+          <t xml:space="preserve">235</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
+          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -16326,19 +16326,19 @@
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">234</t>
+          <t xml:space="preserve">239</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
@@ -16358,61 +16358,61 @@
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 제품</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">234</t>
+          <t xml:space="preserve">240</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">동물용 바이오의약품·백신 제조</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">235</t>
+          <t xml:space="preserve">240</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -16422,61 +16422,61 @@
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">235</t>
+          <t xml:space="preserve">291</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
+          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">바이오화장품·향장제품 제조</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">239</t>
+          <t xml:space="preserve">291</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
+          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -16486,29 +16486,29 @@
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 제품</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">239</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -16518,61 +16518,61 @@
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">240</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품·백신 제조</t>
+          <t xml:space="preserve">바이오고분자 생활소재</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">240</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -16582,61 +16582,61 @@
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">291</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·향장제품 제조</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">291</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -16646,29 +16646,29 @@
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">바이오고분자 산업용 제품</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -16678,29 +16678,29 @@
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">그 밖의 바이오화학 제품</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
@@ -16710,29 +16710,29 @@
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 생활소재</t>
+          <t xml:space="preserve">바이오환경 제품에 속하는 잔여범위</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8010</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -16742,93 +16742,93 @@
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">7010</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">종자 및 묘목</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">취급품목이 종자·묘목일 때의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 산업용 제품</t>
+          <t xml:space="preserve">그 밖의 생물자원 취급품목 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -16838,61 +16838,61 @@
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 제품</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">321</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">바이오농약 판매업</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오환경 제품에 속하는 잔여범위</t>
+          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">321</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">바이오농약 판매업</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -16902,29 +16902,29 @@
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">322</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">바이오비료 판매업</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -16934,93 +16934,93 @@
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목이 종자·묘목일 때의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">322</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">바이오비료 판매업</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생물자원 취급품목 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급품목이 사료첨가제일 때의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">321</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 판매업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
@@ -17030,19 +17030,19 @@
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">첨가제 외 바이오사료의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">321</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 판매업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
@@ -17069,22 +17069,22 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">322</t>
+          <t xml:space="preserve">329</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
@@ -17094,19 +17094,19 @@
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">바이오화학 농자재 취급품목 분야; 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">322</t>
+          <t xml:space="preserve">329</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
@@ -17133,22 +17133,22 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">331</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -17158,371 +17158,371 @@
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목이 사료첨가제일 때의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 판매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">331</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제 외 바이오사료의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">332</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 맞춤형 판매방식 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">329</t>
+          <t xml:space="preserve">332</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
+          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화학 농자재 취급품목 분야; 품목에 따라 재판정</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">329</t>
+          <t xml:space="preserve">333</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
+          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">331</t>
+          <t xml:space="preserve">333</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 위탁제조 판매만으로 8010 아님</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">331</t>
+          <t xml:space="preserve">339</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">332</t>
+          <t xml:space="preserve">339</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 맞춤형 판매방식 전용 코드 없음</t>
+          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">332</t>
+          <t xml:space="preserve">341</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야; 도매업 자체의 대응 아님</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">333</t>
+          <t xml:space="preserve">341</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
+          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">333</t>
+          <t xml:space="preserve">342</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 위탁제조 판매만으로 8010 아님</t>
+          <t xml:space="preserve">자기 상표 위탁제조 동물용 의약품의 제품 분야; 판매형태 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">339</t>
+          <t xml:space="preserve">342</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
+          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분; 제조를 맡기는 발주자는 8010 아님</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">339</t>
+          <t xml:space="preserve">390</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
@@ -17542,61 +17542,61 @@
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">별도 생물류 처리·보관·배송 서비스 수행분만 대응; 판매품목 확인 전 제품 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">341</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">7010</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">종자 및 묘목</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야; 도매업 자체의 대응 아님</t>
+          <t xml:space="preserve">종자·묘목 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">341</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">7020</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">유전자 변형 생물체</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -17606,93 +17606,93 @@
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분</t>
+          <t xml:space="preserve">유전자변형 생물체 개발분</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">342</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">자기 상표 위탁제조 동물용 의약품의 제품 분야; 판매형태 전용 코드 없음</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">342</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분; 제조를 맡기는 발주자는 8010 아님</t>
+          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">390</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
@@ -17702,29 +17702,29 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 처리·보관·배송 서비스 수행분만 대응; 판매품목 확인 전 제품 코드 없음</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
@@ -17734,29 +17734,29 @@
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자·묘목 자체의 개발</t>
+          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7020</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자 변형 생물체</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
@@ -17766,29 +17766,29 @@
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자변형 생물체 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
@@ -17798,115 +17798,115 @@
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
@@ -17933,54 +17933,54 @@
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
+          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
@@ -17990,61 +17990,61 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
@@ -18054,29 +18054,29 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -18086,61 +18086,61 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
@@ -18150,29 +18150,29 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
@@ -18182,29 +18182,29 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -18214,29 +18214,29 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -18246,29 +18246,29 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
+          <t xml:space="preserve">식품용 미생물·효소 소재</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
@@ -18278,29 +18278,29 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
@@ -18310,29 +18310,29 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
+          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -18342,61 +18342,61 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">건강기능식품 제품 개발</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -18406,61 +18406,61 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 소재</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
+          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,19 +18470,19 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
+          <t xml:space="preserve">발효식품 제품기술 개발</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
@@ -18509,44 +18509,44 @@
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강기능식품 제품 개발</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
@@ -18573,54 +18573,54 @@
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -18630,29 +18630,29 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효식품 제품기술 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18662,29 +18662,29 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
@@ -18694,61 +18694,61 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">동물용 바이오백신 개발</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
@@ -18758,19 +18758,19 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
@@ -18790,61 +18790,61 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -18854,83 +18854,83 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오백신 개발</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr">
@@ -18950,61 +18950,61 @@
       </c>
       <c r="F120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E122" s="8" t="inlineStr">
@@ -19014,29 +19014,29 @@
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E123" s="8" t="inlineStr">
@@ -19046,61 +19046,61 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E125" s="8" t="inlineStr">
@@ -19110,29 +19110,29 @@
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E126" s="8" t="inlineStr">
@@ -19142,29 +19142,29 @@
       </c>
       <c r="F126" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E127" s="8" t="inlineStr">
@@ -19174,29 +19174,29 @@
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E128" s="8" t="inlineStr">
@@ -19206,19 +19206,19 @@
       </c>
       <c r="F128" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
@@ -19238,29 +19238,29 @@
       </c>
       <c r="F129" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E130" s="8" t="inlineStr">
@@ -19270,29 +19270,29 @@
       </c>
       <c r="F130" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E131" s="8" t="inlineStr">
@@ -19302,29 +19302,29 @@
       </c>
       <c r="F131" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C132" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E132" s="8" t="inlineStr">
@@ -19334,29 +19334,29 @@
       </c>
       <c r="F132" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E133" s="8" t="inlineStr">
@@ -19366,29 +19366,29 @@
       </c>
       <c r="F133" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E134" s="8" t="inlineStr">
@@ -19398,19 +19398,19 @@
       </c>
       <c r="F134" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C135" s="8" t="inlineStr">
@@ -19430,29 +19430,29 @@
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E136" s="8" t="inlineStr">
@@ -19462,29 +19462,29 @@
       </c>
       <c r="F136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">생물학적 폐자원 처리·재활용 제제 또는 시스템 제공분</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E137" s="8" t="inlineStr">
@@ -19494,29 +19494,29 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E138" s="8" t="inlineStr">
@@ -19526,29 +19526,29 @@
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">그 밖의 바이오환경 서비스; 독립 처리수수료 사업 전체를 직접 포괄하지 않음</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E139" s="8" t="inlineStr">
@@ -19558,29 +19558,29 @@
       </c>
       <c r="F139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C140" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E140" s="8" t="inlineStr">
@@ -19590,29 +19590,29 @@
       </c>
       <c r="F140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E141" s="8" t="inlineStr">
@@ -19622,29 +19622,29 @@
       </c>
       <c r="F141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물학적 폐자원 처리·재활용 제제 또는 시스템 제공분</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E142" s="8" t="inlineStr">
@@ -19654,29 +19654,29 @@
       </c>
       <c r="F142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E143" s="8" t="inlineStr">
@@ -19686,29 +19686,29 @@
       </c>
       <c r="F143" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오환경 서비스; 독립 처리수수료 사업 전체를 직접 포괄하지 않음</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B144" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D144" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E144" s="8" t="inlineStr">
@@ -19717,166 +19717,6 @@
         </is>
       </c>
       <c r="F144" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">532</t>
-        </is>
-      </c>
-      <c r="B145" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
-        </is>
-      </c>
-      <c r="C145" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4010</t>
-        </is>
-      </c>
-      <c r="D145" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
-        </is>
-      </c>
-      <c r="E145" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F145" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B146" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C146" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8020</t>
-        </is>
-      </c>
-      <c r="D146" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
-        </is>
-      </c>
-      <c r="E146" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F146" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B147" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C147" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8030</t>
-        </is>
-      </c>
-      <c r="D147" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E147" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F147" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B148" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C148" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8050</t>
-        </is>
-      </c>
-      <c r="D148" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
-        </is>
-      </c>
-      <c r="E148" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F148" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B149" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C149" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D149" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E149" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F149" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Keep only KS J 4010 for organic waste treatment
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -3626,7 +3626,7 @@
       </c>
       <c r="K62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030, 4010, 4000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
     </row>
@@ -19447,12 +19447,12 @@
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E136" s="8" t="inlineStr">
@@ -19462,29 +19462,29 @@
       </c>
       <c r="F136" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물학적 폐자원 처리·재활용 제제 또는 시스템 제공분</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E137" s="8" t="inlineStr">
@@ -19494,29 +19494,29 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E138" s="8" t="inlineStr">
@@ -19526,29 +19526,29 @@
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오환경 서비스; 독립 처리수수료 사업 전체를 직접 포괄하지 않음</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E139" s="8" t="inlineStr">
@@ -19558,29 +19558,29 @@
       </c>
       <c r="F139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C140" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E140" s="8" t="inlineStr">
@@ -19590,7 +19590,7 @@
       </c>
       <c r="F140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
@@ -19607,12 +19607,12 @@
       </c>
       <c r="C141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E141" s="8" t="inlineStr">
@@ -19622,7 +19622,7 @@
       </c>
       <c r="F141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
@@ -19639,12 +19639,12 @@
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D142" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E142" s="8" t="inlineStr">
@@ -19653,70 +19653,6 @@
         </is>
       </c>
       <c r="F142" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B143" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C143" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8050</t>
-        </is>
-      </c>
-      <c r="D143" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
-        </is>
-      </c>
-      <c r="E143" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F143" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B144" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C144" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D144" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E144" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F144" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Keep only KS J 4010 for agricultural environment management
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -3683,7 +3683,7 @@
       </c>
       <c r="K63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000, 4010</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
     </row>
@@ -19479,12 +19479,12 @@
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E137" s="8" t="inlineStr">
@@ -19494,29 +19494,29 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물학적 농업환경 관리·개선 서비스가 잔여 바이오환경 범위에 들 때</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E138" s="8" t="inlineStr">
@@ -19526,7 +19526,7 @@
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
@@ -19543,12 +19543,12 @@
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E139" s="8" t="inlineStr">
@@ -19558,7 +19558,7 @@
       </c>
       <c r="F139" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
@@ -19575,12 +19575,12 @@
       </c>
       <c r="C140" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E140" s="8" t="inlineStr">
@@ -19590,7 +19590,7 @@
       </c>
       <c r="F140" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
@@ -19607,12 +19607,12 @@
       </c>
       <c r="C141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D141" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E141" s="8" t="inlineStr">
@@ -19621,38 +19621,6 @@
         </is>
       </c>
       <c r="F141" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B142" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C142" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D142" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E142" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F142" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Exclude KS J links from sales distribution division
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -1629,11 +1629,7 @@
           <t xml:space="preserve">13116, 42230, 42920</t>
         </is>
       </c>
-      <c r="K27" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7010, 7000, 8050</t>
-        </is>
-      </c>
+      <c r="K27" s="10"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1686,11 +1682,7 @@
           <t xml:space="preserve">13113</t>
         </is>
       </c>
-      <c r="K28" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2050, 8050</t>
-        </is>
-      </c>
+      <c r="K28" s="10"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1743,11 +1735,7 @@
           <t xml:space="preserve">13112</t>
         </is>
       </c>
-      <c r="K29" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2050, 8050</t>
-        </is>
-      </c>
+      <c r="K29" s="10"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1800,11 +1788,7 @@
           <t xml:space="preserve">13114</t>
         </is>
       </c>
-      <c r="K30" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3050, 3000, 8050</t>
-        </is>
-      </c>
+      <c r="K30" s="10"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1857,11 +1841,7 @@
           <t xml:space="preserve">13119, 13210</t>
         </is>
       </c>
-      <c r="K31" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2000, 8050</t>
-        </is>
-      </c>
+      <c r="K31" s="10"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1914,11 +1894,7 @@
           <t xml:space="preserve">42363, 43229</t>
         </is>
       </c>
-      <c r="K32" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3010, 8050</t>
-        </is>
-      </c>
+      <c r="K32" s="10"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1971,11 +1947,7 @@
           <t xml:space="preserve">43229</t>
         </is>
       </c>
-      <c r="K33" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3010, 8050</t>
-        </is>
-      </c>
+      <c r="K33" s="10"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2028,11 +2000,7 @@
           <t xml:space="preserve">42390</t>
         </is>
       </c>
-      <c r="K34" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3000, 8050</t>
-        </is>
-      </c>
+      <c r="K34" s="10"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2085,11 +2053,7 @@
           <t xml:space="preserve">42390, 43290</t>
         </is>
       </c>
-      <c r="K35" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3000, 8050</t>
-        </is>
-      </c>
+      <c r="K35" s="10"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2142,11 +2106,7 @@
           <t xml:space="preserve">13115</t>
         </is>
       </c>
-      <c r="K36" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1120, 8050</t>
-        </is>
-      </c>
+      <c r="K36" s="10"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2199,11 +2159,7 @@
           <t xml:space="preserve">13115</t>
         </is>
       </c>
-      <c r="K37" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1120, 8050</t>
-        </is>
-      </c>
+      <c r="K37" s="10"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2256,11 +2212,7 @@
           <t xml:space="preserve">42920</t>
         </is>
       </c>
-      <c r="K38" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8050</t>
-        </is>
-      </c>
+      <c r="K38" s="10"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -16749,12 +16701,12 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
@@ -16769,66 +16721,66 @@
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목이 종자·묘목일 때의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">종자·묘목 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">7020</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">유전자 변형 생물체</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생물자원 취급품목 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">유전자변형 생물체 개발분</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -16838,61 +16790,61 @@
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">321</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 판매업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">321</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 판매업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -16902,61 +16854,61 @@
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">322</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 판매업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">322</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 판매업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -16966,115 +16918,115 @@
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목이 사료첨가제일 때의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제 외 바이오사료의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">329</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -17089,34 +17041,34 @@
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화학 농자재 취급품목 분야; 품목에 따라 재판정</t>
+          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">329</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
@@ -17126,61 +17078,61 @@
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">331</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 판매업 자체의 대응 아님</t>
+          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">331</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -17190,61 +17142,61 @@
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">332</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야; 맞춤형 판매방식 전용 코드 없음</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">332</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -17254,19 +17206,19 @@
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">333</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
@@ -17281,34 +17233,34 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
+          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">333</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
@@ -17318,61 +17270,61 @@
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 위탁제조 판매만으로 8010 아님</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">339</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급 식품의 잔여 제품 분야; 실제 품목이 3010·3030·3040이면 해당 코드 재판정</t>
+          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">339</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
@@ -17382,61 +17334,61 @@
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 보관·배송 서비스 수행분; 단순 재판매·부수 배송 제외</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">341</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야; 도매업 자체의 대응 아님</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">341</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
@@ -17446,61 +17398,61 @@
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분</t>
+          <t xml:space="preserve">식품용 미생물·효소 소재</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">342</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">자기 상표 위탁제조 동물용 의약품의 제품 분야; 판매형태 전용 코드 없음</t>
+          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">342</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -17510,29 +17462,29 @@
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 전문 의약품 보관·배송 서비스 수행분; 제조를 맡기는 발주자는 8010 아님</t>
+          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">390</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
@@ -17542,29 +17494,29 @@
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">별도 생물류 처리·보관·배송 서비스 수행분만 대응; 판매품목 확인 전 제품 코드 없음</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -17574,29 +17526,29 @@
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자·묘목 자체의 개발</t>
+          <t xml:space="preserve">건강기능식품 제품 개발</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7020</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자 변형 생물체</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -17606,83 +17558,83 @@
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자변형 생물체 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">발효식품 제품기술 개발</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
@@ -17709,44 +17661,44 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
@@ -17773,22 +17725,22 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
@@ -17798,19 +17750,19 @@
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
@@ -17837,54 +17789,54 @@
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
@@ -17894,93 +17846,93 @@
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">동물용 바이오백신 개발</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
@@ -17990,61 +17942,61 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
@@ -18054,29 +18006,29 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -18086,61 +18038,61 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
@@ -18150,29 +18102,29 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
@@ -18182,29 +18134,29 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -18214,29 +18166,29 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -18246,29 +18198,29 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 소재</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
@@ -18278,29 +18230,29 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
@@ -18310,29 +18262,29 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -18342,51 +18294,51 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강기능식품 제품 개발</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
@@ -18413,54 +18365,54 @@
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,19 +18422,19 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효식품 제품기술 개발</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
@@ -18502,29 +18454,29 @@
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -18534,29 +18486,29 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
@@ -18566,29 +18518,29 @@
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
@@ -18598,29 +18550,29 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -18630,29 +18582,29 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18662,29 +18614,29 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
@@ -18694,51 +18646,51 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오백신 개발</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
@@ -18758,29 +18710,29 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -18790,837 +18742,37 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F116" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">449</t>
-        </is>
-      </c>
-      <c r="B117" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8030</t>
-        </is>
-      </c>
-      <c r="D117" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F117" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">449</t>
-        </is>
-      </c>
-      <c r="B118" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
-        </is>
-      </c>
-      <c r="C118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8040</t>
-        </is>
-      </c>
-      <c r="D118" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F118" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">451</t>
-        </is>
-      </c>
-      <c r="B119" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
-        </is>
-      </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2040</t>
-        </is>
-      </c>
-      <c r="D119" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
-        </is>
-      </c>
-      <c r="E119" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">핵심</t>
-        </is>
-      </c>
-      <c r="F119" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">451</t>
-        </is>
-      </c>
-      <c r="B120" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8040</t>
-        </is>
-      </c>
-      <c r="D120" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F120" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">452</t>
-        </is>
-      </c>
-      <c r="B121" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
-        </is>
-      </c>
-      <c r="C121" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2040</t>
-        </is>
-      </c>
-      <c r="D121" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
-        </is>
-      </c>
-      <c r="E121" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F121" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">452</t>
-        </is>
-      </c>
-      <c r="B122" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
-        </is>
-      </c>
-      <c r="C122" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2010</t>
-        </is>
-      </c>
-      <c r="D122" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
-        </is>
-      </c>
-      <c r="E122" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F122" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">452</t>
-        </is>
-      </c>
-      <c r="B123" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
-        </is>
-      </c>
-      <c r="C123" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2000</t>
-        </is>
-      </c>
-      <c r="D123" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
-        </is>
-      </c>
-      <c r="E123" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F123" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">452</t>
-        </is>
-      </c>
-      <c r="B124" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
-        </is>
-      </c>
-      <c r="C124" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8040</t>
-        </is>
-      </c>
-      <c r="D124" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E124" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F124" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">461</t>
-        </is>
-      </c>
-      <c r="B125" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
-        </is>
-      </c>
-      <c r="C125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4010</t>
-        </is>
-      </c>
-      <c r="D125" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
-        </is>
-      </c>
-      <c r="E125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F125" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">461</t>
-        </is>
-      </c>
-      <c r="B126" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
-        </is>
-      </c>
-      <c r="C126" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4030</t>
-        </is>
-      </c>
-      <c r="D126" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
-        </is>
-      </c>
-      <c r="E126" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F126" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">461</t>
-        </is>
-      </c>
-      <c r="B127" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
-        </is>
-      </c>
-      <c r="C127" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4000</t>
-        </is>
-      </c>
-      <c r="D127" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
-        </is>
-      </c>
-      <c r="E127" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F127" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">461</t>
-        </is>
-      </c>
-      <c r="B128" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
-        </is>
-      </c>
-      <c r="C128" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8040</t>
-        </is>
-      </c>
-      <c r="D128" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E128" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F128" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">462</t>
-        </is>
-      </c>
-      <c r="B129" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
-        </is>
-      </c>
-      <c r="C129" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8040</t>
-        </is>
-      </c>
-      <c r="D129" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E129" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F129" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">462</t>
-        </is>
-      </c>
-      <c r="B130" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
-        </is>
-      </c>
-      <c r="C130" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D130" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E130" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F130" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">490</t>
-        </is>
-      </c>
-      <c r="B131" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
-        </is>
-      </c>
-      <c r="C131" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8040</t>
-        </is>
-      </c>
-      <c r="D131" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E131" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F131" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">521</t>
-        </is>
-      </c>
-      <c r="B132" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
-        </is>
-      </c>
-      <c r="C132" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8020</t>
-        </is>
-      </c>
-      <c r="D132" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
-        </is>
-      </c>
-      <c r="E132" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F132" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">521</t>
-        </is>
-      </c>
-      <c r="B133" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
-        </is>
-      </c>
-      <c r="C133" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D133" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E133" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F133" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">529</t>
-        </is>
-      </c>
-      <c r="B134" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8020</t>
-        </is>
-      </c>
-      <c r="D134" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
-        </is>
-      </c>
-      <c r="E134" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F134" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">529</t>
-        </is>
-      </c>
-      <c r="B135" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
-        </is>
-      </c>
-      <c r="C135" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D135" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E135" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F135" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">531</t>
-        </is>
-      </c>
-      <c r="B136" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
-        </is>
-      </c>
-      <c r="C136" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4010</t>
-        </is>
-      </c>
-      <c r="D136" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
-        </is>
-      </c>
-      <c r="E136" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F136" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">532</t>
-        </is>
-      </c>
-      <c r="B137" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
-        </is>
-      </c>
-      <c r="C137" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4010</t>
-        </is>
-      </c>
-      <c r="D137" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
-        </is>
-      </c>
-      <c r="E137" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F137" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B138" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C138" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8020</t>
-        </is>
-      </c>
-      <c r="D138" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
-        </is>
-      </c>
-      <c r="E138" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F138" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B139" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C139" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8030</t>
-        </is>
-      </c>
-      <c r="D139" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E139" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F139" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B140" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C140" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8050</t>
-        </is>
-      </c>
-      <c r="D140" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
-        </is>
-      </c>
-      <c r="E140" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F140" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B141" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C141" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D141" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E141" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F141" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Show one KS J product field per sales class
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -1629,7 +1629,11 @@
           <t xml:space="preserve">13116, 42230, 42920</t>
         </is>
       </c>
-      <c r="K27" s="10"/>
+      <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7000</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1682,7 +1686,11 @@
           <t xml:space="preserve">13113</t>
         </is>
       </c>
-      <c r="K28" s="10"/>
+      <c r="K28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2050</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1735,7 +1743,11 @@
           <t xml:space="preserve">13112</t>
         </is>
       </c>
-      <c r="K29" s="10"/>
+      <c r="K29" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2050</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1788,7 +1800,11 @@
           <t xml:space="preserve">13114</t>
         </is>
       </c>
-      <c r="K30" s="10"/>
+      <c r="K30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3050</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1841,7 +1857,11 @@
           <t xml:space="preserve">13119, 13210</t>
         </is>
       </c>
-      <c r="K31" s="10"/>
+      <c r="K31" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2000</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1894,7 +1914,11 @@
           <t xml:space="preserve">42363, 43229</t>
         </is>
       </c>
-      <c r="K32" s="10"/>
+      <c r="K32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3010</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1947,7 +1971,11 @@
           <t xml:space="preserve">43229</t>
         </is>
       </c>
-      <c r="K33" s="10"/>
+      <c r="K33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3010</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2000,7 +2028,11 @@
           <t xml:space="preserve">42390</t>
         </is>
       </c>
-      <c r="K34" s="10"/>
+      <c r="K34" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3000</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2053,7 +2085,11 @@
           <t xml:space="preserve">42390, 43290</t>
         </is>
       </c>
-      <c r="K35" s="10"/>
+      <c r="K35" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3000</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2106,7 +2142,11 @@
           <t xml:space="preserve">13115</t>
         </is>
       </c>
-      <c r="K36" s="10"/>
+      <c r="K36" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1120</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2159,7 +2199,11 @@
           <t xml:space="preserve">13115</t>
         </is>
       </c>
-      <c r="K37" s="10"/>
+      <c r="K37" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1120</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2212,7 +2256,11 @@
           <t xml:space="preserve">42920</t>
         </is>
       </c>
-      <c r="K38" s="10"/>
+      <c r="K38" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2040</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -16701,406 +16749,406 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자·묘목 자체의 개발</t>
+          <t xml:space="preserve">생물자원 취급분의 대표 분야; 가공 소재는 실제 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">321</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">바이오농약 판매업</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7020</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자 변형 생물체</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자변형 생물체 개발분</t>
+          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">322</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">바이오비료 판매업</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">사료첨가제 취급분의 제품 분야; 단미사료 등은 이 코드에 해당하지 않음</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">329</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 취급분의 대표 분야; 실제 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">331</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">332</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">취급품목인 맞춤형 건강기능식품의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">333</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
+          <t xml:space="preserve">그 밖의 바이오식품 취급분의 대표 분야; 식품첨가물 등은 실제 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">339</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 바이오식품 취급분의 대표 분야; 실제 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">341</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
+          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">342</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">자기 상표로 판매하는 동물용 바이오의약품의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">390</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">향장제품·생활제품 취급분의 대표 분야; 동물약국 등 다른 품목은 실제 제품에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">7010</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">종자 및 묘목</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -17110,29 +17158,29 @@
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
+          <t xml:space="preserve">종자·묘목 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">7020</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">유전자 변형 생물체</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -17142,19 +17190,19 @@
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">유전자변형 생물체 개발분</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
@@ -17181,54 +17229,54 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
+          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
@@ -17238,61 +17286,61 @@
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
@@ -17302,29 +17350,29 @@
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
@@ -17334,19 +17382,19 @@
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
+          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
@@ -17373,54 +17421,54 @@
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 소재</t>
+          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
@@ -17430,29 +17478,29 @@
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
+          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -17462,83 +17510,83 @@
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강기능식품 제품 개발</t>
+          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
@@ -17565,54 +17613,54 @@
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
+          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
@@ -17622,19 +17670,19 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효식품 제품기술 개발</t>
+          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
@@ -17661,22 +17709,22 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
@@ -17686,29 +17734,29 @@
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
@@ -17718,29 +17766,29 @@
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
@@ -17750,29 +17798,29 @@
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
@@ -17782,29 +17830,29 @@
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품용 미생물·효소 소재</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
@@ -17814,29 +17862,29 @@
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
+          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
@@ -17846,83 +17894,83 @@
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오백신 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">건강기능식품 제품 개발</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
@@ -17942,29 +17990,29 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
@@ -17974,29 +18022,29 @@
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
+          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
@@ -18006,19 +18054,19 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">발효식품 제품기술 개발</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
@@ -18038,51 +18086,51 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
@@ -18109,22 +18157,22 @@
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
@@ -18134,29 +18182,29 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -18166,29 +18214,29 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -18198,19 +18246,19 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
@@ -18237,54 +18285,54 @@
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">동물용 바이오백신 개발</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -18294,29 +18342,29 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
@@ -18326,61 +18374,61 @@
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -18390,29 +18438,29 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18422,61 +18470,61 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -18486,29 +18534,29 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
@@ -18518,29 +18566,29 @@
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
@@ -18550,29 +18598,29 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -18582,29 +18630,29 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18614,19 +18662,19 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
@@ -18646,29 +18694,29 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">590</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -18678,29 +18726,29 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">590</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
@@ -18710,29 +18758,29 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">590</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -18742,37 +18790,421 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">462</t>
+        </is>
+      </c>
+      <c r="B116" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+        </is>
+      </c>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8040</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
+        </is>
+      </c>
+      <c r="E116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F116" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">462</t>
+        </is>
+      </c>
+      <c r="B117" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8000</t>
+        </is>
+      </c>
+      <c r="D117" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 바이오서비스업</t>
+        </is>
+      </c>
+      <c r="E117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F117" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">490</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8040</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
+        </is>
+      </c>
+      <c r="E118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F118" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">521</t>
+        </is>
+      </c>
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8020</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+        </is>
+      </c>
+      <c r="E119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F119" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">521</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8000</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 바이오서비스업</t>
+        </is>
+      </c>
+      <c r="E120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F120" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">529</t>
+        </is>
+      </c>
+      <c r="B121" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8020</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+        </is>
+      </c>
+      <c r="E121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F121" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">529</t>
+        </is>
+      </c>
+      <c r="B122" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8000</t>
+        </is>
+      </c>
+      <c r="D122" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 바이오서비스업</t>
+        </is>
+      </c>
+      <c r="E122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F122" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">531</t>
+        </is>
+      </c>
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+        </is>
+      </c>
+      <c r="C123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4010</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+        </is>
+      </c>
+      <c r="E123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F123" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">532</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+        </is>
+      </c>
+      <c r="C124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4010</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+        </is>
+      </c>
+      <c r="E124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F124" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">590</t>
         </is>
       </c>
-      <c r="B116" s="10" t="inlineStr">
+      <c r="B125" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
-      <c r="C116" s="8" t="inlineStr">
+      <c r="C125" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8020</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+        </is>
+      </c>
+      <c r="E125" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F125" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">590</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
+        </is>
+      </c>
+      <c r="C126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8030</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+        </is>
+      </c>
+      <c r="E126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F126" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">590</t>
+        </is>
+      </c>
+      <c r="B127" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
+        </is>
+      </c>
+      <c r="C127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8050</t>
+        </is>
+      </c>
+      <c r="D127" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+        </is>
+      </c>
+      <c r="E127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F127" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">590</t>
+        </is>
+      </c>
+      <c r="B128" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
+        </is>
+      </c>
+      <c r="C128" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8000</t>
         </is>
       </c>
-      <c r="D116" s="10" t="inlineStr">
+      <c r="D128" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
-      <c r="E116" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F116" s="10" t="inlineStr">
+      <c r="E128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건부</t>
+        </is>
+      </c>
+      <c r="F128" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Remove KS J 8010 from four manufacturing classes
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -1403,7 +1403,7 @@
       </c>
       <c r="K23" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120, 8010</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K24" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040, 8010</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="K25" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040, 2010, 2000, 8010</t>
+          <t xml:space="preserve">2040, 2010, 2000</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="K26" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010, 2000, 4000, 8010</t>
+          <t xml:space="preserve">2010, 2000, 4000</t>
         </is>
       </c>
     </row>
@@ -16397,44 +16397,44 @@
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">240</t>
+          <t xml:space="preserve">291</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
+          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">바이오화장품·향장제품 제조</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">291</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
@@ -16449,34 +16449,34 @@
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·향장제품 제조</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">291</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -16486,7 +16486,7 @@
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">바이오고분자 생활소재</t>
         </is>
       </c>
     </row>
@@ -16503,12 +16503,12 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -16518,19 +16518,19 @@
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
@@ -16550,19 +16550,19 @@
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 생활소재</t>
+          <t xml:space="preserve">바이오고분자 산업용 제품</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
@@ -16582,29 +16582,29 @@
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">그 밖의 바이오화학 제품</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">292</t>
+          <t xml:space="preserve">299</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
+          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -16614,157 +16614,157 @@
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">바이오환경 제품에 속하는 잔여범위</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">310</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 산업용 제품</t>
+          <t xml:space="preserve">생물자원 취급분의 대표 분야; 가공 소재는 실제 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">321</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">바이오농약 판매업</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 제품</t>
+          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">322</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">바이오비료 판매업</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오환경 제품에 속하는 잔여범위</t>
+          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">299</t>
+          <t xml:space="preserve">323</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
+          <t xml:space="preserve">바이오사료 판매업</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8010</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 위탁 생산ㆍ대행 서비스</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">참고</t>
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">타사 의뢰를 받은 바이오제품 제조 대행</t>
+          <t xml:space="preserve">사료첨가제 취급분의 제품 분야; 단미사료 등은 이 코드에 해당하지 않음</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">310</t>
+          <t xml:space="preserve">329</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
@@ -16774,29 +16774,29 @@
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물자원 취급분의 대표 분야; 가공 소재는 실제 품목에 따라 재판정</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 취급분의 대표 분야; 실제 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">321</t>
+          <t xml:space="preserve">331</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 판매업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -16806,29 +16806,29 @@
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오농약의 제품 분야</t>
+          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">322</t>
+          <t xml:space="preserve">332</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 판매업</t>
+          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -16838,29 +16838,29 @@
       </c>
       <c r="F54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 바이오비료의 제품 분야</t>
+          <t xml:space="preserve">취급품목인 맞춤형 건강기능식품의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">323</t>
+          <t xml:space="preserve">333</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 판매업</t>
+          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -16870,29 +16870,29 @@
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료첨가제 취급분의 제품 분야; 단미사료 등은 이 코드에 해당하지 않음</t>
+          <t xml:space="preserve">그 밖의 바이오식품 취급분의 대표 분야; 식품첨가물 등은 실제 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">329</t>
+          <t xml:space="preserve">339</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
+          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -16902,29 +16902,29 @@
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 취급분의 대표 분야; 실제 품목에 따라 재판정</t>
+          <t xml:space="preserve">그 밖의 바이오식품 취급분의 대표 분야; 실제 품목에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">331</t>
+          <t xml:space="preserve">341</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -16934,29 +16934,29 @@
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 건강기능식품의 제품 분야</t>
+          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">332</t>
+          <t xml:space="preserve">342</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 맞춤형건강기능식품판매업</t>
+          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -16966,29 +16966,29 @@
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 맞춤형 건강기능식품의 제품 분야</t>
+          <t xml:space="preserve">자기 상표로 판매하는 동물용 바이오의약품의 제품 분야</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">333</t>
+          <t xml:space="preserve">390</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
+          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -16998,211 +16998,211 @@
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 취급분의 대표 분야; 식품첨가물 등은 실제 품목에 따라 재판정</t>
+          <t xml:space="preserve">향장제품·생활제품 취급분의 대표 분야; 동물약국 등 다른 품목은 실제 제품에 따라 재판정</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">339</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">7010</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">종자 및 묘목</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 취급분의 대표 분야; 실제 품목에 따라 재판정</t>
+          <t xml:space="preserve">종자·묘목 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">341</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 도매업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">7020</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">유전자 변형 생물체</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">취급품목인 동물용 바이오의약품의 제품 분야</t>
+          <t xml:space="preserve">유전자변형 생물체 개발분</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">342</t>
+          <t xml:space="preserve">411</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 위탁제조판매업</t>
+          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">자기 상표로 판매하는 동물용 바이오의약품의 제품 분야</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">390</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">향장제품·생활제품 취급분의 대표 분야; 동물약국 등 다른 품목은 실제 제품에 따라 재판정</t>
+          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">412</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자 및 묘목</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">종자·묘목 자체의 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7020</t>
+          <t xml:space="preserve">7000</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자 변형 생물체</t>
+          <t xml:space="preserve">기타 바이오자원</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전자변형 생물체 개발분</t>
+          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">411</t>
+          <t xml:space="preserve">413</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
+          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
@@ -17229,12 +17229,12 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
@@ -17249,24 +17249,24 @@
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·균주 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">412</t>
+          <t xml:space="preserve">419</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
@@ -17293,22 +17293,22 @@
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
@@ -17318,29 +17318,29 @@
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">곤충 등 생물자원 자체의 개발</t>
+          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">413</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
@@ -17350,29 +17350,29 @@
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">421</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">바이오농약 연구개발업</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오자원</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
@@ -17382,93 +17382,93 @@
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 살아 있는 생물자원에 한정</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">419</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 방제 제제 개발</t>
+          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
@@ -17478,29 +17478,29 @@
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -17510,61 +17510,61 @@
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
+          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -17574,29 +17574,29 @@
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -17606,29 +17606,29 @@
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
@@ -17638,29 +17638,29 @@
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
@@ -17670,29 +17670,29 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
@@ -17702,29 +17702,29 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품용 미생물·효소 소재</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
@@ -17734,29 +17734,29 @@
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
+          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
@@ -17766,19 +17766,19 @@
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
+          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
@@ -17805,54 +17805,54 @@
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 소재</t>
+          <t xml:space="preserve">건강기능식품 제품 개발</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
@@ -17862,61 +17862,61 @@
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
+          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
@@ -17926,61 +17926,61 @@
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">발효식품 제품기술 개발</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강기능식품 제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
@@ -17990,61 +17990,61 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
@@ -18054,19 +18054,19 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효식품 제품기술 개발</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
@@ -18093,12 +18093,12 @@
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
@@ -18118,19 +18118,19 @@
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
@@ -18157,54 +18157,54 @@
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">동물용 바이오백신 개발</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -18214,29 +18214,29 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -18246,93 +18246,93 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오백신 개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -18342,93 +18342,93 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -18438,29 +18438,29 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,51 +18470,51 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
@@ -18541,22 +18541,22 @@
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
@@ -18566,29 +18566,29 @@
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
@@ -18598,29 +18598,29 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -18630,19 +18630,19 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
@@ -18669,22 +18669,22 @@
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
@@ -18694,29 +18694,29 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -18726,29 +18726,29 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
@@ -18758,29 +18758,29 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -18790,29 +18790,29 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
@@ -18822,29 +18822,29 @@
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -18854,29 +18854,29 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
@@ -18886,29 +18886,29 @@
       </c>
       <c r="F118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
@@ -18918,29 +18918,29 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E120" s="8" t="inlineStr">
@@ -18950,19 +18950,19 @@
       </c>
       <c r="F120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
@@ -18982,29 +18982,29 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E122" s="8" t="inlineStr">
@@ -19014,29 +19014,29 @@
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E123" s="8" t="inlineStr">
@@ -19046,29 +19046,29 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E124" s="8" t="inlineStr">
@@ -19077,134 +19077,6 @@
         </is>
       </c>
       <c r="F124" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B125" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8020</t>
-        </is>
-      </c>
-      <c r="D125" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
-        </is>
-      </c>
-      <c r="E125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F125" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B126" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C126" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8030</t>
-        </is>
-      </c>
-      <c r="D126" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
-        </is>
-      </c>
-      <c r="E126" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F126" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B127" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C127" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8050</t>
-        </is>
-      </c>
-      <c r="D127" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
-        </is>
-      </c>
-      <c r="E127" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F127" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B128" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C128" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D128" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E128" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F128" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Keep KS J 8050 only for sales class 390
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -2258,7 +2258,7 @@
       </c>
       <c r="K38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
     </row>
@@ -16983,22 +16983,22 @@
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">참고</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">향장제품·생활제품 취급분의 대표 분야; 동물약국 등 다른 품목은 실제 제품에 따라 재판정</t>
+          <t xml:space="preserve">그린바이오제품의 별도 가공·처리·보관 서비스를 수행하는 경우에 한정; 판매 자체는 제외</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove KS J 2000 from pesticide and fertilizer R&D
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -2543,7 +2543,7 @@
       </c>
       <c r="K43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050, 2000, 8040</t>
+          <t xml:space="preserve">2050, 8040</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050, 2000, 8040</t>
+          <t xml:space="preserve">2050, 8040</t>
         </is>
       </c>
     </row>
@@ -17335,12 +17335,12 @@
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
@@ -17350,39 +17350,39 @@
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 농약이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">421</t>
+          <t xml:space="preserve">422</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
+          <t xml:space="preserve">바이오비료 연구개발업</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2050</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오농약 및 비료</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
         </is>
       </c>
     </row>
@@ -17399,44 +17399,44 @@
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오농약 및 비료</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물·생물학적 비료 제제 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3050</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">사료 첨가제</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
@@ -17446,29 +17446,29 @@
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생물공정 비료이나 생물학적 제제가 아닌 산출물</t>
+          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">422</t>
+          <t xml:space="preserve">423</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
+          <t xml:space="preserve">바이오사료 연구개발업</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
@@ -17478,7 +17478,7 @@
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
         </is>
       </c>
     </row>
@@ -17495,12 +17495,12 @@
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료 첨가제</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -17510,29 +17510,29 @@
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">사료첨가제 개발분; 단미사료는 제외</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
@@ -17542,29 +17542,29 @@
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
+          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -17574,7 +17574,7 @@
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
         </is>
       </c>
     </row>
@@ -17591,12 +17591,12 @@
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -17606,29 +17606,29 @@
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
@@ -17638,29 +17638,29 @@
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
+          <t xml:space="preserve">식품용 미생물·효소 소재</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
@@ -17670,7 +17670,7 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
         </is>
       </c>
     </row>
@@ -17687,12 +17687,12 @@
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
@@ -17702,7 +17702,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 소재</t>
+          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
         </is>
       </c>
     </row>
@@ -17719,12 +17719,12 @@
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
@@ -17734,51 +17734,51 @@
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
+          <t xml:space="preserve">건강기능식품 제품 개발</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
@@ -17805,22 +17805,22 @@
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
@@ -17830,29 +17830,29 @@
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강기능식품 제품 개발</t>
+          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">발효식품 제품기술 개발</t>
         </is>
       </c>
     </row>
@@ -17879,44 +17879,44 @@
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
@@ -17926,19 +17926,19 @@
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효식품 제품기술 개발</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
@@ -17965,12 +17965,12 @@
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
@@ -17990,19 +17990,19 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
@@ -18029,12 +18029,12 @@
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
@@ -18054,19 +18054,19 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
@@ -18093,54 +18093,54 @@
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
+          <t xml:space="preserve">동물용 바이오백신 개발</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
@@ -18150,7 +18150,7 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -18167,76 +18167,76 @@
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오백신 개발</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -18246,7 +18246,7 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -18263,66 +18263,66 @@
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
@@ -18342,19 +18342,19 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
@@ -18369,34 +18369,34 @@
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -18406,7 +18406,7 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
@@ -18423,12 +18423,12 @@
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
@@ -18455,12 +18455,12 @@
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,29 +18470,29 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
@@ -18502,29 +18502,29 @@
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -18534,7 +18534,7 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
@@ -18551,12 +18551,12 @@
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
@@ -18583,12 +18583,12 @@
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
@@ -18598,29 +18598,29 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -18630,29 +18630,29 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18662,19 +18662,19 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
@@ -18694,29 +18694,29 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -18726,29 +18726,29 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
@@ -18758,19 +18758,19 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
@@ -18790,19 +18790,19 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
@@ -18822,29 +18822,29 @@
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -18854,29 +18854,29 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
@@ -18886,29 +18886,29 @@
       </c>
       <c r="F118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
@@ -18918,29 +18918,29 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E120" s="8" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="F120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
@@ -18967,12 +18967,12 @@
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E121" s="8" t="inlineStr">
@@ -18982,7 +18982,7 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
@@ -18999,12 +18999,12 @@
       </c>
       <c r="C122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E122" s="8" t="inlineStr">
@@ -19013,70 +19013,6 @@
         </is>
       </c>
       <c r="F122" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B123" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C123" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8050</t>
-        </is>
-      </c>
-      <c r="D123" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
-        </is>
-      </c>
-      <c r="E123" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F123" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B124" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C124" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D124" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E124" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F124" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Remove KS J 3000 from feed R&D class
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -2657,7 +2657,7 @@
       </c>
       <c r="K45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3050, 3000, 8040</t>
+          <t xml:space="preserve">3050, 8040</t>
         </is>
       </c>
     </row>
@@ -17463,12 +17463,12 @@
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
@@ -17478,29 +17478,29 @@
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">첨가제가 아닌 바이오사료 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">423</t>
+          <t xml:space="preserve">429</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -17510,7 +17510,7 @@
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
         </is>
       </c>
     </row>
@@ -17527,12 +17527,12 @@
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
@@ -17542,7 +17542,7 @@
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">생분해성 농업용 고분자 자재 개발분</t>
+          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
         </is>
       </c>
     </row>
@@ -17559,12 +17559,12 @@
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -17574,29 +17574,29 @@
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품용 미생물·효소 소재</t>
         </is>
       </c>
     </row>
@@ -17623,12 +17623,12 @@
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
@@ -17638,7 +17638,7 @@
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 소재</t>
+          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
         </is>
       </c>
     </row>
@@ -17655,12 +17655,12 @@
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
@@ -17670,7 +17670,7 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
+          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
         </is>
       </c>
     </row>
@@ -17687,12 +17687,12 @@
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
@@ -17702,39 +17702,39 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">건강기능식품 제품 개발</t>
         </is>
       </c>
     </row>
@@ -17751,54 +17751,54 @@
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강기능식품 제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
         </is>
       </c>
     </row>
@@ -17815,22 +17815,22 @@
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
+          <t xml:space="preserve">발효식품 제품기술 개발</t>
         </is>
       </c>
     </row>
@@ -17847,12 +17847,12 @@
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
@@ -17862,29 +17862,29 @@
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효식품 제품기술 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
@@ -17894,7 +17894,7 @@
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
@@ -17911,12 +17911,12 @@
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
@@ -17926,29 +17926,29 @@
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
@@ -17958,7 +17958,7 @@
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
@@ -17975,12 +17975,12 @@
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
@@ -17990,29 +17990,29 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
@@ -18022,7 +18022,7 @@
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
         </is>
       </c>
     </row>
@@ -18039,12 +18039,12 @@
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
@@ -18054,39 +18054,39 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">동물용 바이오백신 개발</t>
         </is>
       </c>
     </row>
@@ -18103,22 +18103,22 @@
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오백신 개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -18135,12 +18135,12 @@
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
@@ -18150,39 +18150,39 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
@@ -18199,22 +18199,22 @@
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -18231,12 +18231,12 @@
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -18246,39 +18246,39 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
@@ -18295,44 +18295,44 @@
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
@@ -18359,12 +18359,12 @@
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
@@ -18391,12 +18391,12 @@
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -18406,7 +18406,7 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
@@ -18423,12 +18423,12 @@
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -18438,29 +18438,29 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,7 +18470,7 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
@@ -18487,12 +18487,12 @@
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
@@ -18519,12 +18519,12 @@
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -18534,7 +18534,7 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
@@ -18551,12 +18551,12 @@
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
@@ -18566,19 +18566,19 @@
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
@@ -18598,7 +18598,7 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
@@ -18615,12 +18615,12 @@
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -18630,29 +18630,29 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18662,29 +18662,29 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
@@ -18711,12 +18711,12 @@
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -18726,29 +18726,29 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
@@ -18775,12 +18775,12 @@
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -18790,29 +18790,29 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
@@ -18822,19 +18822,19 @@
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
@@ -18854,29 +18854,29 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
@@ -18886,7 +18886,7 @@
       </c>
       <c r="F118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
@@ -18903,12 +18903,12 @@
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
@@ -18935,12 +18935,12 @@
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E120" s="8" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="F120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
@@ -18967,12 +18967,12 @@
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E121" s="8" t="inlineStr">
@@ -18981,38 +18981,6 @@
         </is>
       </c>
       <c r="F121" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B122" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C122" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D122" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E122" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F122" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Remove KS J 2000 from other farm input R&D
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -2714,7 +2714,7 @@
       </c>
       <c r="K46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010, 2000, 8040</t>
+          <t xml:space="preserve">2010, 8040</t>
         </is>
       </c>
     </row>
@@ -17527,12 +17527,12 @@
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
@@ -17542,29 +17542,29 @@
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 농자재 개발분</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429</t>
+          <t xml:space="preserve">431</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -17574,7 +17574,7 @@
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품용 미생물·효소 소재</t>
         </is>
       </c>
     </row>
@@ -17591,12 +17591,12 @@
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3030</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">식품 첨가물</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 소재</t>
+          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
         </is>
       </c>
     </row>
@@ -17623,12 +17623,12 @@
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3030</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품 첨가물</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
@@ -17638,7 +17638,7 @@
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품첨가물로 사용되는 소재</t>
+          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
         </is>
       </c>
     </row>
@@ -17655,12 +17655,12 @@
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
@@ -17670,39 +17670,39 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오식품 원료·중간체</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">431</t>
+          <t xml:space="preserve">432</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
+          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3010</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">건강 기능 식품</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">건강기능식품 제품 개발</t>
         </is>
       </c>
     </row>
@@ -17719,54 +17719,54 @@
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3010</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강 기능 식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">건강기능식품 제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">432</t>
+          <t xml:space="preserve">433</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3020</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">식품용 미생물 및 효소</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
         </is>
       </c>
     </row>
@@ -17783,22 +17783,22 @@
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3020</t>
+          <t xml:space="preserve">3040</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물 및 효소</t>
+          <t xml:space="preserve">발효 식품</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">식품용 미생물·효소 이용기술</t>
+          <t xml:space="preserve">발효식품 제품기술 개발</t>
         </is>
       </c>
     </row>
@@ -17815,12 +17815,12 @@
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3040</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효 식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
@@ -17830,29 +17830,29 @@
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">발효식품 제품기술 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">433</t>
+          <t xml:space="preserve">434</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
+          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
         </is>
       </c>
     </row>
@@ -17879,12 +17879,12 @@
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
@@ -17894,29 +17894,29 @@
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">대체식품 전용 코드가 없어 기타 바이오식품으로 포섭</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">434</t>
+          <t xml:space="preserve">435</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
@@ -17926,7 +17926,7 @@
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
         </is>
       </c>
     </row>
@@ -17943,12 +17943,12 @@
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
@@ -17958,29 +17958,29 @@
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">특수영양·특수의료용도식품 전용 코드가 없음</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">435</t>
+          <t xml:space="preserve">439</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">3000</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오식품</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
         </is>
       </c>
     </row>
@@ -18007,12 +18007,12 @@
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오식품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
@@ -18022,39 +18022,39 @@
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 바이오식품 코드에 속하지 않는 산출물</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">439</t>
+          <t xml:space="preserve">441</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
+          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">동물용 바이오백신 개발</t>
         </is>
       </c>
     </row>
@@ -18071,22 +18071,22 @@
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오백신 개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -18103,12 +18103,12 @@
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
@@ -18118,39 +18118,39 @@
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
@@ -18167,22 +18167,22 @@
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -18199,12 +18199,12 @@
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -18214,39 +18214,39 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
@@ -18263,44 +18263,44 @@
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
@@ -18327,12 +18327,12 @@
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
@@ -18359,12 +18359,12 @@
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
@@ -18391,12 +18391,12 @@
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -18406,29 +18406,29 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
@@ -18455,12 +18455,12 @@
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,7 +18470,7 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
@@ -18487,12 +18487,12 @@
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
@@ -18519,12 +18519,12 @@
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -18534,19 +18534,19 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
@@ -18583,12 +18583,12 @@
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
@@ -18598,29 +18598,29 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -18630,29 +18630,29 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18662,7 +18662,7 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
@@ -18679,12 +18679,12 @@
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
@@ -18694,29 +18694,29 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -18726,7 +18726,7 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
@@ -18743,12 +18743,12 @@
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
@@ -18758,29 +18758,29 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -18790,19 +18790,19 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
@@ -18822,29 +18822,29 @@
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -18854,7 +18854,7 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
@@ -18871,12 +18871,12 @@
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
@@ -18886,7 +18886,7 @@
       </c>
       <c r="F118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
@@ -18903,12 +18903,12 @@
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
@@ -18935,12 +18935,12 @@
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E120" s="8" t="inlineStr">
@@ -18949,38 +18949,6 @@
         </is>
       </c>
       <c r="F120" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B121" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C121" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D121" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E121" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F121" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Remove KS J 8030 from animal vaccine R&D
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -3113,7 +3113,7 @@
       </c>
       <c r="K53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120, 8030, 8040</t>
+          <t xml:space="preserve">1120, 8040</t>
         </is>
       </c>
     </row>
@@ -18071,12 +18071,12 @@
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -18086,39 +18086,39 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">441</t>
+          <t xml:space="preserve">449</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">1120</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">동물용 바이오의약품</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
         </is>
       </c>
     </row>
@@ -18135,22 +18135,22 @@
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 바이오의약품</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">백신 외 동물용 바이오의약품 개발</t>
+          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
         </is>
       </c>
     </row>
@@ -18167,12 +18167,12 @@
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
@@ -18182,39 +18182,39 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
@@ -18231,44 +18231,44 @@
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
@@ -18278,7 +18278,7 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
@@ -18295,12 +18295,12 @@
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
@@ -18327,12 +18327,12 @@
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
@@ -18359,12 +18359,12 @@
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
@@ -18374,29 +18374,29 @@
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -18406,7 +18406,7 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
@@ -18423,12 +18423,12 @@
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
@@ -18455,12 +18455,12 @@
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,7 +18470,7 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
@@ -18487,12 +18487,12 @@
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
@@ -18502,19 +18502,19 @@
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
@@ -18534,7 +18534,7 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
@@ -18551,12 +18551,12 @@
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
@@ -18566,29 +18566,29 @@
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
@@ -18598,29 +18598,29 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -18630,7 +18630,7 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
@@ -18647,12 +18647,12 @@
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18662,29 +18662,29 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
@@ -18711,12 +18711,12 @@
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -18726,29 +18726,29 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
@@ -18758,19 +18758,19 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
@@ -18790,29 +18790,29 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
@@ -18822,7 +18822,7 @@
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
@@ -18839,12 +18839,12 @@
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -18854,7 +18854,7 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
@@ -18871,12 +18871,12 @@
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
@@ -18886,7 +18886,7 @@
       </c>
       <c r="F118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
@@ -18903,12 +18903,12 @@
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
@@ -18917,38 +18917,6 @@
         </is>
       </c>
       <c r="F119" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B120" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D120" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F120" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Remove KS J 8030 from other animal medicine R&D
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -3170,7 +3170,7 @@
       </c>
       <c r="K54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120, 8030, 8040</t>
+          <t xml:space="preserve">1120, 8040</t>
         </is>
       </c>
     </row>
@@ -18135,12 +18135,12 @@
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
@@ -18150,39 +18150,39 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">계약에 따른 비임상 연구개발·효능평가</t>
+          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">449</t>
+          <t xml:space="preserve">451</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">조건부</t>
+          <t xml:space="preserve">핵심</t>
         </is>
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 외부 수탁 연구개발</t>
+          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
         </is>
       </c>
     </row>
@@ -18199,44 +18199,44 @@
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">핵심</t>
+          <t xml:space="preserve">조건부</t>
         </is>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품·인체용 생활화학제품 개발</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">451</t>
+          <t xml:space="preserve">452</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">2040</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -18246,7 +18246,7 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
         </is>
       </c>
     </row>
@@ -18263,12 +18263,12 @@
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2040</t>
+          <t xml:space="preserve">2010</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오화장품 및 생활 화학 제품</t>
+          <t xml:space="preserve">바이오 고분자 제품</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
@@ -18278,7 +18278,7 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">비누·세제 등 바이오 생활화학제품</t>
+          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
         </is>
       </c>
     </row>
@@ -18295,12 +18295,12 @@
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010</t>
+          <t xml:space="preserve">2000</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 고분자 제품</t>
+          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오고분자 기반 포장재·생활소재</t>
+          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
         </is>
       </c>
     </row>
@@ -18327,12 +18327,12 @@
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오화학ㆍ에너지 제품</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -18342,29 +18342,29 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 바이오화학 생활제품</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">452</t>
+          <t xml:space="preserve">461</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
+          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
         </is>
       </c>
     </row>
@@ -18391,12 +18391,12 @@
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">4030</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -18406,7 +18406,7 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 생물학적 환경처리 제제</t>
+          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
         </is>
       </c>
     </row>
@@ -18423,12 +18423,12 @@
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4030</t>
+          <t xml:space="preserve">4000</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리, 자원 재활용 제제 및 시스템</t>
+          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">폐자원 처리·재활용 제제와 시스템</t>
+          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
         </is>
       </c>
     </row>
@@ -18455,12 +18455,12 @@
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오환경 제품 및 서비스</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -18470,19 +18470,19 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경개선 서비스 개발 중 잔여범위</t>
+          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">461</t>
+          <t xml:space="preserve">462</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 연구개발에 한정</t>
+          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
         </is>
       </c>
     </row>
@@ -18519,12 +18519,12 @@
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -18534,29 +18534,29 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">외부 수탁 디지털 기술 연구개발에 한정</t>
+          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">462</t>
+          <t xml:space="preserve">490</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
+          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8040</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">기타 연구개발 서비스</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
@@ -18566,29 +18566,29 @@
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">농업생명정보 서비스가 KS J 바이오서비스 범위에 드는 경우; 전용 코드 없음</t>
+          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">490</t>
+          <t xml:space="preserve">521</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
+          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8040</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 연구개발 서비스</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
@@ -18598,7 +18598,7 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">산출 분야를 특정하지 못한 외부 수탁 연구개발만 대응</t>
+          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
         </is>
       </c>
     </row>
@@ -18615,12 +18615,12 @@
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -18630,29 +18630,29 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질 등 생물학적 분석 결과를 고객에게 제공할 때</t>
+          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">521</t>
+          <t xml:space="preserve">529</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
+          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -18662,7 +18662,7 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">디지털육종 플랫폼이 바이오서비스 잔여범위에 속할 때; 전용 코드 없음</t>
+          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
         </is>
       </c>
     </row>
@@ -18679,12 +18679,12 @@
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
@@ -18694,29 +18694,29 @@
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·대사체 등 생물학적 분석·진단 서비스</t>
+          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">529</t>
+          <t xml:space="preserve">531</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
+          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8000</t>
+          <t xml:space="preserve">4010</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
+          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -18726,19 +18726,19 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그 밖의 생명정보 서비스; 일반 소프트웨어·데이터 판매는 자동 대응하지 않음</t>
+          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">531</t>
+          <t xml:space="preserve">532</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
+          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
@@ -18758,29 +18758,29 @@
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">미생물 등 환경처리용 생물 제제를 함께 제공할 때</t>
+          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">532</t>
+          <t xml:space="preserve">590</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
+          <t xml:space="preserve">기타 그린바이오 서비스업</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4010</t>
+          <t xml:space="preserve">8020</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 처리용 생물 제제 및 시스템</t>
+          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -18790,7 +18790,7 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">환경 정화용 생물 제제·시스템 제공분; 순수 방제대행은 별도 코드 없음</t>
+          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
         </is>
       </c>
     </row>
@@ -18807,12 +18807,12 @@
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8030</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
@@ -18822,7 +18822,7 @@
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
         </is>
       </c>
     </row>
@@ -18839,12 +18839,12 @@
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -18854,7 +18854,7 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
@@ -18871,12 +18871,12 @@
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8050</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
@@ -18885,38 +18885,6 @@
         </is>
       </c>
       <c r="F118" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B119" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D119" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E119" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F119" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Remove KS J 8020 and 8030 from other services
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -3740,7 +3740,7 @@
       </c>
       <c r="K64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020, 8030, 8050, 8000</t>
+          <t xml:space="preserve">8050, 8000</t>
         </is>
       </c>
     </row>
@@ -18775,12 +18775,12 @@
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8020</t>
+          <t xml:space="preserve">8050</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">바이오 분석ㆍ진단 서비스</t>
+          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -18790,7 +18790,7 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">유전체·단백질·대사체의 생물학적 분석·진단 서비스에 해당하는 부분</t>
+          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
         </is>
       </c>
     </row>
@@ -18807,12 +18807,12 @@
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">8030</t>
+          <t xml:space="preserve">8000</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">임상ㆍ비임상 연구개발 서비스</t>
+          <t xml:space="preserve">기타 바이오서비스업</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
@@ -18821,70 +18821,6 @@
         </is>
       </c>
       <c r="F116" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 의약품 비임상 시험의 계약 수탁분</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B117" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8050</t>
-        </is>
-      </c>
-      <c r="D117" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">가공 및 처리ㆍ보관 서비스</t>
-        </is>
-      </c>
-      <c r="E117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F117" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">생물자원의 특화 처리·보관·수송 서비스</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B118" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
-      <c r="C118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8000</t>
-        </is>
-      </c>
-      <c r="D118" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 바이오서비스업</t>
-        </is>
-      </c>
-      <c r="E118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조건부</t>
-        </is>
-      </c>
-      <c r="F118" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">시험·분석으로 포섭되지 않는 인증·검사 등 잔여 바이오서비스</t>
         </is>

</xml_diff>

<commit_message>
Add English definitions to round six classification
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -3802,7 +3802,8 @@
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="58" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="5" max="5" width="110" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3835,6 +3836,11 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">English definition</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">5차 코드</t>
         </is>
       </c>
@@ -3860,7 +3866,8 @@
           <t xml:space="preserve">Green Bio Production</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="10"/>
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
         </is>
@@ -3887,7 +3894,8 @@
           <t xml:space="preserve">Green Bio Seed Production</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="10"/>
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">21</t>
         </is>
@@ -3916,6 +3924,11 @@
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that multiply, collect, or raise seeds to produce seeds to which green-bio has been applied. Seeds include grains, mushroom spawn, seedlings, spores, and vegetative propagules used for propagation or cultivation.</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">210</t>
         </is>
       </c>
@@ -3941,7 +3954,8 @@
           <t xml:space="preserve">Production of Plants for Green Bio Materials</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="10"/>
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">22</t>
         </is>
@@ -3970,6 +3984,11 @@
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that cultivate and produce cannabis (Cannabis sativa L.) for use as a raw material in manufacturing green-bio materials. Cultivation for fiber or seed collection requires a cannabis cultivator permit. Cultivation for cannabidiol or other materials requires a separate legal basis, such as a regulatory sandbox demonstration exemption. Cultivation unrelated to the manufacture of green-bio materials is excluded. Extraction and processing of cannabis-derived materials are classified under 211.</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">221</t>
         </is>
       </c>
@@ -3997,6 +4016,11 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that cultivate and produce plants other than cannabis for use as raw materials in manufacturing green-bio materials, where biotechnology-related techniques have been applied or the plants meet verified green-bio manufacturing specifications. Processing cultivated plants into materials by extraction, drying, milling, or similar methods is classified under 211. Cultivation of ordinary food or ornamental crops is excluded.</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">229</t>
         </is>
       </c>
@@ -4022,7 +4046,8 @@
           <t xml:space="preserve">Green Bio Laboratory Animal Production</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="10"/>
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">23</t>
         </is>
@@ -4051,6 +4076,11 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that breed and multiply laboratory animals used or reared for animal experiments while maintaining their biological identity and reproductive capacity. This class is limited to production that supplies research, development, or testing in green-bio fields such as veterinary medicines, agricultural inputs, and foods. Production supplied solely to fields outside green-bio, such as the development of medicines for human use, is excluded.</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">230</t>
         </is>
       </c>
@@ -4076,7 +4106,8 @@
           <t xml:space="preserve">Other Green Bio Production</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="10"/>
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">29</t>
         </is>
@@ -4105,6 +4136,11 @@
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to culture, multiply, or rear other agricultural biological resources of actual or potential value to agriculture, such as microorganisms and insects, while maintaining their biological identity and reproductive capacity, where they are not classified in the preceding classes. Processing cultured or multiplied biological resources into non-reproductive materials by killing, drying, milling, extraction, or similar methods is classified in the applicable class of Group 21.</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">290</t>
         </is>
       </c>
@@ -4130,7 +4166,8 @@
           <t xml:space="preserve">Green Bio Manufacturing</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="10"/>
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">3</t>
         </is>
@@ -4157,7 +4194,8 @@
           <t xml:space="preserve">Green Bio Material Manufacturing</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="10"/>
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">31</t>
         </is>
@@ -4186,6 +4224,11 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that manufacture green-bio materials, meaning raw materials or intermediate products used to produce green-bio products, by extracting, separating, purifying, fermenting, concentrating, drying, milling, or otherwise processing substances derived from plants or their cell or tissue cultures. Material origin is determined by the output: if the output is a microbial metabolite or microbial biomass, it is classified under 212 even when plant inputs serve as the culture medium or nutrient source. Cultivation of the plants themselves is classified in the applicable class of Group 12.</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">311</t>
         </is>
       </c>
@@ -4213,6 +4256,11 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that culture or ferment microorganisms that are agricultural biological resources of actual or potential value to agriculture, or separate, purify, or process their metabolites or cellular components, to manufacture non-reproductive raw materials or intermediate products used to produce green-bio products. Culturing or multiplying mushroom spawn or microbial strains that retain their biological identity and reproductive capacity is classified under 190.</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">312</t>
         </is>
       </c>
@@ -4240,6 +4288,11 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that dry, mill, extract, separate, purify, or otherwise process insects, as defined in Class 413, or insect-derived substances into green-bio materials used as raw materials or intermediate products for producing green-bio products. Rearing and multiplying live insects is classified under 190.</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">313</t>
         </is>
       </c>
@@ -4267,6 +4320,11 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that manufacture other green-bio materials, meaning raw materials or intermediate products used to produce green-bio products, that are not classified as materials derived from plants, microorganisms, or insects. Materials with two or more origins are included. Manufacture of food additives is classified under 231.</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">319</t>
         </is>
       </c>
@@ -4292,7 +4350,8 @@
           <t xml:space="preserve">Green Bio Agricultural Input Manufacturing</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="10"/>
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">32</t>
         </is>
@@ -4321,6 +4380,11 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that manufacture pesticides used to control crop pests and diseases or regulate crop growth by using living organisms such as microorganisms or insects, or biologically derived substances such as natural substances.</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">321</t>
         </is>
       </c>
@@ -4348,6 +4412,11 @@
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that manufacture fertilizers, including soil improvement materials, used to supply plant nutrients or improve soil by using live microorganisms or their metabolites.</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">322</t>
         </is>
       </c>
@@ -4375,6 +4444,11 @@
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that manufacture animal feed, including single-ingredient feed, compound feed, and supplementary feed, to supply animal nutrition by using living organisms such as microorganisms or insects, biologically derived substances such as natural substances, or fermentation or enzyme technologies. Veterinary medicines are excluded.</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">323</t>
         </is>
       </c>
@@ -4402,6 +4476,11 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that manufacture other green-bio agricultural inputs not classified as biopesticides, biofertilizers, or bio-based animal feed. This includes agricultural films and seedling containers made from biodegradable materials produced using biological resources or microbial fermentation; livestock-facility environmental improvers using microorganisms or natural substances; and crop-growth promoting materials that are neither fertilizers nor pesticides. Seed production is classified under 110, and manufacture of veterinary medicines under 240. Agricultural machinery, facilities, and equipment, and petroleum-derived materials to which green-bio makes no contribution, are excluded.</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">329</t>
         </is>
       </c>
@@ -4427,7 +4506,8 @@
           <t xml:space="preserve">Green Bio Food Manufacturing</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" s="10"/>
+      <c r="F25" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">33</t>
         </is>
@@ -4456,6 +4536,11 @@
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to manufacture food additives used in the manufacture, processing, preparation, or preservation of food for purposes such as sweetening, coloring, bleaching, or preventing oxidation. All biological origins are covered, including enzymes, sweeteners, and preservatives produced by microbial fermentation. Manufacture of raw materials or intermediate products for food manufacture that are not food additives is classified in the applicable class of Group 21.</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">331</t>
         </is>
       </c>
@@ -4483,6 +4568,11 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that manufacture fermented foods by inoculating selected or improved microorganisms or strains, or by directly applying fermentation process control technology. Manufacture of ordinary fermented foods using only spontaneous fermentation is excluded.</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">332</t>
         </is>
       </c>
@@ -4510,6 +4600,11 @@
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to manufacture health functional foods from ingredients or components with functions beneficial to the human body. Ordinary health supplements are excluded.</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">333</t>
         </is>
       </c>
@@ -4537,6 +4632,11 @@
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to manufacture special nutritional foods meeting the nutritional needs of specific population groups, such as infants, older adults, or pregnant women, or foods for special medical purposes intended for the dietary or nutritional management of people with diseases or medical conditions.</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">334</t>
         </is>
       </c>
@@ -4564,6 +4664,11 @@
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that manufacture foods replacing the texture, flavor, nutrition, or function of conventional livestock or fishery products by using biological resources or materials such as plants, microorganisms, insects, and their cell-culture products, or by using biological processes.</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">335</t>
         </is>
       </c>
@@ -4591,6 +4696,11 @@
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that directly use biological resources, biological materials, or biological processes to manufacture other foods not classified in the preceding classes.</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">339</t>
         </is>
       </c>
@@ -4616,7 +4726,8 @@
           <t xml:space="preserve">Green Bio Veterinary Medicine Manufacturing</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="E32" s="10"/>
+      <c r="F32" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">34</t>
         </is>
@@ -4645,6 +4756,11 @@
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to manufacture medicines and pharmaceutical preparations intended solely for animal use.</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">340</t>
         </is>
       </c>
@@ -4670,7 +4786,8 @@
           <t xml:space="preserve">Other Green Bio Product Manufacturing</t>
         </is>
       </c>
-      <c r="E34" s="10" t="inlineStr">
+      <c r="E34" s="10"/>
+      <c r="F34" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">39</t>
         </is>
@@ -4699,6 +4816,11 @@
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that manufacture cosmetics, including functional and customized cosmetics, and personal care products applied directly to the human body, such as body cleansers and oral care products, using green-bio materials derived from microorganisms, insects, natural substances, or similar sources. Household products not applied directly to the human body are classified under 292. Products made by simply mixing natural ingredients are excluded.</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">391</t>
         </is>
       </c>
@@ -4726,6 +4848,11 @@
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that manufacture household goods using green-bio materials derived from microorganisms, insects, natural substances, or similar sources. This includes household chemical products used to clean, wash, deodorize, disinfect, or repel pests in living spaces or on textiles and objects, and consumer goods such as leather substitutes, fibers, packaging, and cushioning made from green-bio materials. Personal care products applied directly to the human body are classified under 291; manufacture at the material stage, such as fabrics or molded forms, is classified in the applicable class of Group 21. Products made by simply mixing natural ingredients are excluded.</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">392</t>
         </is>
       </c>
@@ -4753,6 +4880,11 @@
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that directly use green-bio to manufacture other green-bio products not classified in the preceding classes.</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">399</t>
         </is>
       </c>
@@ -4778,7 +4910,8 @@
           <t xml:space="preserve">Green Bio Sales and Distribution</t>
         </is>
       </c>
-      <c r="E38" s="10" t="inlineStr">
+      <c r="E38" s="10"/>
+      <c r="F38" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">4</t>
         </is>
@@ -4805,7 +4938,8 @@
           <t xml:space="preserve">Green Bio Biological Resource and Material Sales and Distribution</t>
         </is>
       </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="E39" s="10"/>
+      <c r="F39" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">41</t>
         </is>
@@ -4834,6 +4968,11 @@
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that purchase and sell to businesses or consumers living biological resources, including seeds, planting stock, seedlings, mushroom spawn, microbial strains, cell lines, and industrial insects, or green-bio materials such as extracts, fermentation products, and functional ingredients, or broker their trade for a fee or under contract without taking ownership of the goods. Green-bio materials are raw materials or intermediate products used to produce green-bio products. Direct sales of biological resources or materials produced by the seller are classified in the applicable class of Division 1 or 2. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">410</t>
         </is>
       </c>
@@ -4859,7 +4998,8 @@
           <t xml:space="preserve">Green Bio Agricultural Input Sales</t>
         </is>
       </c>
-      <c r="E41" s="10" t="inlineStr">
+      <c r="E41" s="10"/>
+      <c r="F41" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">42</t>
         </is>
@@ -4888,6 +5028,11 @@
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities of a registered pesticide seller that purchases and sells pesticides produced using green-bio to businesses or consumers. Sales businesses dealing only in chemical pesticides are excluded. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">421</t>
         </is>
       </c>
@@ -4915,6 +5060,11 @@
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities of a fertilizer seller that sells fertilizers produced using green-bio. Sales businesses dealing only in ordinary fertilizers for which the application of biotechnology-related techniques cannot be confirmed are excluded. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">422</t>
         </is>
       </c>
@@ -4942,6 +5092,11 @@
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities of a feed seller that sells animal feed produced using green-bio. Sales businesses dealing only in ordinary feed for which the application of biotechnology-related techniques cannot be confirmed are excluded. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">423</t>
         </is>
       </c>
@@ -4969,6 +5124,11 @@
       </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that sell or distribute other green-bio agricultural inputs not covered by the preceding classes. Sales and distribution of seeds are classified under 310, and those of veterinary medicines in the applicable class of Group 34. Sales of agricultural machinery, facilities, and equipment, and businesses dealing only in ordinary agricultural inputs for which the application of biotechnology-related techniques cannot be confirmed, are excluded. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">429</t>
         </is>
       </c>
@@ -4994,7 +5154,8 @@
           <t xml:space="preserve">Green Bio Food Sales</t>
         </is>
       </c>
-      <c r="E46" s="10" t="inlineStr">
+      <c r="E46" s="10"/>
+      <c r="F46" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">43</t>
         </is>
@@ -5023,6 +5184,11 @@
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities of a health functional food seller that sells health functional foods produced using green-bio. Sales by dividing or combining products according to an individual's lifestyle or health status are classified under 332; distribution under the seller's own brand of products manufactured under contract is classified under 333. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">431</t>
         </is>
       </c>
@@ -5050,6 +5216,11 @@
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities of a customized health functional food seller that divides or combines health functional foods produced using green-bio according to an individual's lifestyle, health status, or similar characteristics and sells them. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">432</t>
         </is>
       </c>
@@ -5077,6 +5248,11 @@
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that commission a manufacturer to manufacture or process foods or food additives using green-bio, without manufacturing or processing them directly, and distribute or sell the resulting products under the seller's own brand. Specialized food distribution and sales businesses handling green-bio foods are included. Contract production using raw materials supplied for the seller's own account is classified in the applicable manufacturing class of Division 2. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">433</t>
         </is>
       </c>
@@ -5104,6 +5280,11 @@
       </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that sell or distribute foods and food materials produced using green-bio that are not covered by the preceding classes. This includes wholesale trade in food materials and additives, and food sales businesses handling green-bio foods. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F50" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">439</t>
         </is>
       </c>
@@ -5129,7 +5310,8 @@
           <t xml:space="preserve">Green Bio Veterinary Medicine Sales and Distribution</t>
         </is>
       </c>
-      <c r="E51" s="10" t="inlineStr">
+      <c r="E51" s="10"/>
+      <c r="F51" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">44</t>
         </is>
@@ -5158,6 +5340,11 @@
       </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities of a licensed veterinary medicine wholesaler that purchases veterinary medicines produced using green-bio and sells them to businesses or brokers their trade. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">441</t>
         </is>
       </c>
@@ -5185,6 +5372,11 @@
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities of a veterinary medicine contract-manufacturing seller that commissions the manufacture of green-bio veterinary medicines and distributes or sells them under its own brand. Contract production using raw materials supplied for the seller's own account is classified under 240. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F53" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">442</t>
         </is>
       </c>
@@ -5210,7 +5402,8 @@
           <t xml:space="preserve">Other Green Bio Sales and Distribution</t>
         </is>
       </c>
-      <c r="E54" s="10" t="inlineStr">
+      <c r="E54" s="10"/>
+      <c r="F54" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">49</t>
         </is>
@@ -5239,6 +5432,11 @@
       </c>
       <c r="E55" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that purchase and sell to businesses or consumers other green-bio products produced using green-bio that are not covered by the preceding groups. This includes distribution of green-bio cosmetics, personal care and household products, and retail sales of green-bio veterinary medicines by animal pharmacies. Goods are treated as green-bio goods when they were produced or manufactured through activities in Division 1 or 2. This class applies only when the green-bio portion of the goods handled and the related sales can be distinguished from general merchandise. It excludes general retailers and brokerage platforms whose green-bio goods form only an inseparable part of their product range, as well as simple transportation and storage.</t>
+        </is>
+      </c>
+      <c r="F55" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">490</t>
         </is>
       </c>
@@ -5264,7 +5462,8 @@
           <t xml:space="preserve">Green Bio Research and Development</t>
         </is>
       </c>
-      <c r="E56" s="10" t="inlineStr">
+      <c r="E56" s="10"/>
+      <c r="F56" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
@@ -5291,7 +5490,8 @@
           <t xml:space="preserve">Green Bio Biological Resource Research and Development</t>
         </is>
       </c>
-      <c r="E57" s="10" t="inlineStr">
+      <c r="E57" s="10"/>
+      <c r="F57" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">11</t>
         </is>
@@ -5320,6 +5520,11 @@
       </c>
       <c r="E58" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to breed new seeds or varieties, or research and develop the traits, functions, propagation processes, safety, or uses of grains, mushroom spawn, seedlings, spores, and vegetative propagules used for propagation or cultivation. This includes research and development on the varieties, traits, and safety of genetically modified plants, as well as radiation breeding, polyploid breeding, genomic breeding, and digital breeding.</t>
+        </is>
+      </c>
+      <c r="F58" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">111</t>
         </is>
       </c>
@@ -5347,6 +5552,11 @@
       </c>
       <c r="E59" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to discover or improve living microorganisms, such as strains and starter cultures used in cultivation, animal rearing, or fermentation for food or agricultural input production, or to research and develop their traits, functions, propagation processes, or uses. Research and development of mushroom spawn used as seed is classified under 411. Research and development that uses microorganisms to create agricultural inputs, foods, medicines, or other outputs is classified in the group corresponding to the output, from Groups 42 through 46.</t>
+        </is>
+      </c>
+      <c r="F59" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">112</t>
         </is>
       </c>
@@ -5374,6 +5584,11 @@
       </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to discover or improve living insects used in rearing or propagation, or to research and develop their traits, functions, rearing processes, or uses. This includes the development of superior insect breeding stock. Here, insects include stag beetles, rhinoceros beetles, fireflies, black soldier flies, flower chafers, and bumblebees; all animals classified in class Insecta of phylum Arthropoda under the International Code of Zoological Nomenclature; and arachnids and centipedes. Research and development directed at specific outputs such as feed or food is classified in the group corresponding to the output.</t>
+        </is>
+      </c>
+      <c r="F60" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">113</t>
         </is>
       </c>
@@ -5401,6 +5616,11 @@
       </c>
       <c r="E61" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities not covered by the preceding classes that use green-bio to research and develop other living agricultural biological resources of actual or potential value to agriculture, including their traits, functions, propagation processes, and uses.</t>
+        </is>
+      </c>
+      <c r="F61" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">119</t>
         </is>
       </c>
@@ -5426,7 +5646,8 @@
           <t xml:space="preserve">Green Bio Agricultural Input Research and Development</t>
         </is>
       </c>
-      <c r="E62" s="10" t="inlineStr">
+      <c r="E62" s="10"/>
+      <c r="F62" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">12</t>
         </is>
@@ -5455,6 +5676,11 @@
       </c>
       <c r="E63" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use living organisms such as microorganisms or insects, or biologically derived substances such as natural substances, to research and develop pesticides for crop pest and disease control or growth regulation, including their materials, formulations, production processes, efficacy, and safety.</t>
+        </is>
+      </c>
+      <c r="F63" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">121</t>
         </is>
       </c>
@@ -5482,6 +5708,11 @@
       </c>
       <c r="E64" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use live microorganisms or their metabolites to research and develop fertilizers for plant nutrition or soil improvement, including their materials, formulations, production processes, and efficacy. This includes research and development of microbial preparations for soil improvement, such as soil improvement materials and by-product fertilizers.</t>
+        </is>
+      </c>
+      <c r="F64" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">122</t>
         </is>
       </c>
@@ -5509,6 +5740,11 @@
       </c>
       <c r="E65" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use living organisms such as microorganisms or insects, biologically derived substances such as natural substances, or fermentation or enzyme technologies to research and develop animal feed, including single-ingredient feed, compound feed, and supplementary feed, and its materials, formulations, production processes, or efficacy. Research and development intended for veterinary medicines is classified in Group 44.</t>
+        </is>
+      </c>
+      <c r="F65" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">123</t>
         </is>
       </c>
@@ -5536,6 +5772,11 @@
       </c>
       <c r="E66" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that research and develop other green-bio agricultural inputs not classified as biopesticides, biofertilizers, or bio-based animal feed, including their materials, production processes, or efficacy. This includes agricultural films and seedling containers made from biodegradable materials produced using biological resources or microbial fermentation; livestock-facility environmental improvers using microorganisms or natural substances; and crop-growth promoting materials that are neither fertilizers nor pesticides. Seeds are classified under 411, and veterinary medicines in Group 44. Research and development of agricultural machinery, facilities, and equipment, and petroleum-derived materials to which green-bio makes no contribution, are excluded.</t>
+        </is>
+      </c>
+      <c r="F66" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">129</t>
         </is>
       </c>
@@ -5561,7 +5802,8 @@
           <t xml:space="preserve">Research and Development of Green Bio Food Ingredients and Products</t>
         </is>
       </c>
-      <c r="E67" s="10" t="inlineStr">
+      <c r="E67" s="10"/>
+      <c r="F67" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">13</t>
         </is>
@@ -5590,6 +5832,11 @@
       </c>
       <c r="E68" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that develop natural substances and other materials derived from living organisms such as microorganisms, insects, and plants as raw materials or intermediate products for food manufacture, and research and develop their composition, functions, extraction, separation, purification, standardization, mass production, or uses. Both functional and other food materials are included. Research and development of materials intended for alternative foods is classified under 434; fermentation processes or microbial utilization technologies themselves under 433; and materials intended for cosmetics or household products in Group 45.</t>
+        </is>
+      </c>
+      <c r="F68" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">131</t>
         </is>
       </c>
@@ -5617,6 +5864,11 @@
       </c>
       <c r="E69" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to research and develop the composition, formulation, functionality, safety, or product technology of health functional foods made from ingredients or components with functions beneficial to the human body. Research and development at the raw-material or intermediate-product stage is classified under 431.</t>
+        </is>
+      </c>
+      <c r="F69" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">132</t>
         </is>
       </c>
@@ -5644,6 +5896,11 @@
       </c>
       <c r="E70" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that research and develop technologies for using microorganisms in food manufacture, processing, or fermentation, as well as fermentation processes, enzymes, safety, or product technologies for fermented foods. Discovery or improvement of microbial strains themselves is classified under 412.</t>
+        </is>
+      </c>
+      <c r="F70" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">133</t>
         </is>
       </c>
@@ -5671,6 +5928,11 @@
       </c>
       <c r="E71" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to research and develop foods replacing the texture, flavor, nutrition, or function of conventional livestock or fishery products, including their materials, formulations, structuring processes, safety, and product technologies. This includes research and development of plant- or seaweed-based meat alternatives, cultured meat from animal cells, insect alternative proteins, and microbial-fermentation alternative proteins, regardless of the source material or method.</t>
+        </is>
+      </c>
+      <c r="F71" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">134</t>
         </is>
       </c>
@@ -5698,6 +5960,11 @@
       </c>
       <c r="E72" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to research and develop special nutritional foods meeting the nutritional needs of specific population groups, such as infants, older adults, or pregnant women, or foods for special medical purposes intended for the dietary or nutritional management of people with diseases or medical conditions, including their materials, formulations, and manufacturing processes.</t>
+        </is>
+      </c>
+      <c r="F72" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">135</t>
         </is>
       </c>
@@ -5725,6 +5992,11 @@
       </c>
       <c r="E73" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that research and develop other green-bio foods and food materials not covered by the preceding classes.</t>
+        </is>
+      </c>
+      <c r="F73" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">139</t>
         </is>
       </c>
@@ -5750,7 +6022,8 @@
           <t xml:space="preserve">Green Bio Veterinary Medicine Research and Development</t>
         </is>
       </c>
-      <c r="E74" s="10" t="inlineStr">
+      <c r="E74" s="10"/>
+      <c r="F74" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">14</t>
         </is>
@@ -5779,6 +6052,11 @@
       </c>
       <c r="E75" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to research and develop antigens, immunogens, vaccine strains, vectors, adjuvants, formulations, production processes, efficacy, safety, or administration technologies for medicines intended solely for animal use to prevent infectious animal diseases.</t>
+        </is>
+      </c>
+      <c r="F75" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">141</t>
         </is>
       </c>
@@ -5806,6 +6084,11 @@
       </c>
       <c r="E76" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that research and develop candidate substances, active ingredients, diagnostic agents, therapeutics, formulations, production processes, efficacy, safety, or uses of other green-bio veterinary medicines not classified as veterinary vaccine research and development.</t>
+        </is>
+      </c>
+      <c r="F76" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">149</t>
         </is>
       </c>
@@ -5831,7 +6114,8 @@
           <t xml:space="preserve">Research and Development of Green Bio Cosmetics and Household Products</t>
         </is>
       </c>
-      <c r="E77" s="10" t="inlineStr">
+      <c r="E77" s="10"/>
+      <c r="F77" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">15</t>
         </is>
@@ -5860,6 +6144,11 @@
       </c>
       <c r="E78" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to research and develop cosmetics, including functional and customized cosmetics, and personal care products applied directly to the human body, such as body cleansers and oral care products, as well as materials used to manufacture them, formulations, efficacy, or safety.</t>
+        </is>
+      </c>
+      <c r="F78" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">151</t>
         </is>
       </c>
@@ -5887,6 +6176,11 @@
       </c>
       <c r="E79" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use green-bio to research and develop household goods and the materials, formulations, or efficacy involved in their manufacture. This includes household chemical products for cleaning, washing, deodorizing, antimicrobial treatment, or pest control in living spaces or on textiles and objects, and consumer goods such as leather substitutes, fibers, packaging, and cushioning made from green-bio materials. Personal care products applied directly to the human body are classified under 451; research and development of the materials themselves is classified under 431 or 490.</t>
+        </is>
+      </c>
+      <c r="F79" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">152</t>
         </is>
       </c>
@@ -5912,7 +6206,8 @@
           <t xml:space="preserve">Research and Development of Green Bio Environmental and Digital Services</t>
         </is>
       </c>
-      <c r="E80" s="10" t="inlineStr">
+      <c r="E80" s="10"/>
+      <c r="F80" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">16</t>
         </is>
@@ -5941,6 +6236,11 @@
       </c>
       <c r="E81" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use living biological resources such as insects or microorganisms to research and develop technologies, processes, or preparations for treating organic waste resources; controlling pests and diseases; or managing and improving agricultural environments such as livestock facilities, farmland, and agricultural water. Research and development intended for pesticide preparations is classified under 421; fertilizer or soil-improvement preparations under 422; and discovery or improvement of the biological resources themselves in the applicable class of Group 41. The provision of environmental services itself is classified in the applicable class of Group 53.</t>
+        </is>
+      </c>
+      <c r="F81" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">161</t>
         </is>
       </c>
@@ -5968,6 +6268,11 @@
       </c>
       <c r="E82" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that research and develop technologies for analyzing agricultural bio-resource data, such as genomic and phenotypic data, and digital technologies including digital breeding platforms, software for the green-bio industry, and artificial intelligence models. Research and development that uses molecular markers or genomic analysis to breed varieties themselves is classified under 411; provision of data services itself is classified in the applicable class of Group 52.</t>
+        </is>
+      </c>
+      <c r="F82" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">162</t>
         </is>
       </c>
@@ -5993,7 +6298,8 @@
           <t xml:space="preserve">Other Green Bio Research and Development</t>
         </is>
       </c>
-      <c r="E83" s="10" t="inlineStr">
+      <c r="E83" s="10"/>
+      <c r="F83" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">19</t>
         </is>
@@ -6022,6 +6328,11 @@
       </c>
       <c r="E84" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Other green-bio research and development activities not covered by the preceding groups. This includes research and development of multipurpose materials or platform technologies for which no particular application has been specified. Research and development of data or digital technologies is classified under 462.</t>
+        </is>
+      </c>
+      <c r="F84" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">190</t>
         </is>
       </c>
@@ -6047,7 +6358,8 @@
           <t xml:space="preserve">Green Bio Information, Environmental and Other Services</t>
         </is>
       </c>
-      <c r="E85" s="10" t="inlineStr">
+      <c r="E85" s="10"/>
+      <c r="F85" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">5</t>
         </is>
@@ -6074,7 +6386,8 @@
           <t xml:space="preserve">Green Bio Information and Data Services</t>
         </is>
       </c>
-      <c r="E86" s="10" t="inlineStr">
+      <c r="E86" s="10"/>
+      <c r="F86" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">52</t>
         </is>
@@ -6103,6 +6416,11 @@
       </c>
       <c r="E87" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that provide genomic, marker, or phenotypic analysis and bioinformatics consulting services to support digital breeding by analyzing genomic information and other data on agricultural bio-resources. Services provided by digital breeding consulting and analysis specialist institutions designated by the Ministry of Agriculture, Food and Rural Affairs are included. Research and development that breeds varieties themselves is classified under 411; research and development of analysis technologies or platforms themselves is classified under 462.</t>
+        </is>
+      </c>
+      <c r="F87" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">521</t>
         </is>
       </c>
@@ -6130,6 +6448,11 @@
       </c>
       <c r="E88" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that collect, analyze, process, and provide other data relating to green-bio that are not covered by the preceding class. Operation of bioinformatics databases and platforms is included. Research and development in which data analysis leads to the development of new varieties, materials, products, or technologies is classified in the applicable class of Division 4.</t>
+        </is>
+      </c>
+      <c r="F88" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">529</t>
         </is>
       </c>
@@ -6155,7 +6478,8 @@
           <t xml:space="preserve">Green Bio Environmental Services</t>
         </is>
       </c>
-      <c r="E89" s="10" t="inlineStr">
+      <c r="E89" s="10"/>
+      <c r="F89" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">53</t>
         </is>
@@ -6184,6 +6508,11 @@
       </c>
       <c r="E90" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that apply biotechnology-related techniques to living biological resources such as insects or microorganisms to break down and treat agricultural organic waste resources, including livestock manure and food waste. This class applies when treatment fees are the principal source of revenue. Manufacture of larval feed produced during treatment is classified under 223, and manufacture of fertilizer from insect frass under 222.</t>
+        </is>
+      </c>
+      <c r="F90" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">531</t>
         </is>
       </c>
@@ -6211,6 +6540,11 @@
       </c>
       <c r="E91" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that use living biological resources such as natural enemy insects or microorganisms as the principal means of controlling crop pests and diseases or managing and improving the environment of livestock facilities, farmland, or agricultural water by designing and implementing programs based on biotechnology-related techniques and the organisms' biological characteristics. This includes biological pest control using natural enemies or microorganisms. It excludes contractors that merely apply purchased biopesticides or environmental improvers without biological program design, pest control using only chemical pesticides, and remediation of general industrial wastewater or contaminated soil unrelated to agriculture.</t>
+        </is>
+      </c>
+      <c r="F91" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">532</t>
         </is>
       </c>
@@ -6236,7 +6570,8 @@
           <t xml:space="preserve">Other Green Bio Services</t>
         </is>
       </c>
-      <c r="E92" s="10" t="inlineStr">
+      <c r="E92" s="10"/>
+      <c r="F92" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">59</t>
         </is>
@@ -6265,13 +6600,18 @@
       </c>
       <c r="E93" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Industrial activities that provide other green-bio-related services not covered by the preceding groups. This includes services that use standardized methods to test, inspect, or analyze the quality, composition, functionality, safety, or efficacy of green-bio goods such as seeds, microorganisms, insects, natural substances, foods, and veterinary medicines, including seed testing, microbial identification, genetic or compositional analysis, and contracted nonclinical testing of veterinary medicines; services that inspect, review, and certify whether green-bio goods or their production and manufacturing processes comply with laws, specifications, or standards; and storage or transport services specialized in preserving the identity of biological resources such as seeds and microbial strains. Contract research aimed at developing new varieties, materials, products, or technologies is classified in the applicable class of Division 4; genomic or bioinformatics analysis services supporting digital breeding are classified under 521. Simple transportation and storage are excluded. Education or training about green-bio technologies is also excluded because it conveys knowledge rather than applying biotechnology and belongs to the workforce development support system rather than an industrial activity.</t>
+        </is>
+      </c>
+      <c r="F93" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">590</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Align Green-Bio English spelling with statute
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -305,7 +305,7 @@
       </c>
       <c r="H4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Seed Production</t>
+          <t xml:space="preserve">Green-Bio Seed Production</t>
         </is>
       </c>
       <c r="I4" s="10" t="inlineStr">
@@ -362,7 +362,7 @@
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cannabis Cultivation for Green Bio Materials</t>
+          <t xml:space="preserve">Cannabis Cultivation for Green-Bio Materials</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr">
@@ -419,7 +419,7 @@
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Production of Other Plants for Green Bio Materials</t>
+          <t xml:space="preserve">Production of Other Plants for Green-Bio Materials</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Laboratory Animal Production</t>
+          <t xml:space="preserve">Green-Bio Laboratory Animal Production</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Production</t>
+          <t xml:space="preserve">Other Green-Bio Production</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manufacturing of Green Bio Materials Derived from Plants</t>
+          <t xml:space="preserve">Manufacturing of Green-Bio Materials Derived from Plants</t>
         </is>
       </c>
       <c r="I9" s="10" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manufacturing of Green Bio Materials Derived from Microorganisms</t>
+          <t xml:space="preserve">Manufacturing of Green-Bio Materials Derived from Microorganisms</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manufacturing of Green Bio Materials Derived from Insects</t>
+          <t xml:space="preserve">Manufacturing of Green-Bio Materials Derived from Insects</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Material Manufacturing</t>
+          <t xml:space="preserve">Other Green-Bio Material Manufacturing</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Agricultural Input Manufacturing</t>
+          <t xml:space="preserve">Other Green-Bio Agricultural Input Manufacturing</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Food Additive Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Food Additive Manufacturing</t>
         </is>
       </c>
       <c r="I17" s="10" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Fermented Food Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Fermented Food Manufacturing</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Health Functional Food Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Health Functional Food Manufacturing</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manufacturing of Green Bio Special Nutritional Foods and Foods for Special Medical Purposes</t>
+          <t xml:space="preserve">Manufacturing of Green-Bio Special Nutritional Foods and Foods for Special Medical Purposes</t>
         </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Alternative Food Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Alternative Food Manufacturing</t>
         </is>
       </c>
       <c r="I21" s="10" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Food Manufacturing</t>
+          <t xml:space="preserve">Other Green-Bio Food Manufacturing</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Veterinary Medicine Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Veterinary Medicine Manufacturing</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manufacturing of Green Bio Cosmetics and Personal Care Products</t>
+          <t xml:space="preserve">Manufacturing of Green-Bio Cosmetics and Personal Care Products</t>
         </is>
       </c>
       <c r="I24" s="10" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="H25" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Household Product Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Household Product Manufacturing</t>
         </is>
       </c>
       <c r="I25" s="10" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Product Manufacturing</t>
+          <t xml:space="preserve">Other Green-Bio Product Manufacturing</t>
         </is>
       </c>
       <c r="I26" s="10" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Biological Resource and Material Sales and Distribution</t>
+          <t xml:space="preserve">Green-Bio Biological Resource and Material Sales and Distribution</t>
         </is>
       </c>
       <c r="I27" s="10" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="H31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Agricultural Input Sales</t>
+          <t xml:space="preserve">Other Green-Bio Agricultural Input Sales</t>
         </is>
       </c>
       <c r="I31" s="10" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="H32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Health Functional Food Sales</t>
+          <t xml:space="preserve">Green-Bio Health Functional Food Sales</t>
         </is>
       </c>
       <c r="I32" s="10" t="inlineStr">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="H33" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customized Green Bio Health Functional Food Sales</t>
+          <t xml:space="preserve">Customized Green-Bio Health Functional Food Sales</t>
         </is>
       </c>
       <c r="I33" s="10" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="H34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Specialized Distribution and Sales of Green Bio Foods</t>
+          <t xml:space="preserve">Specialized Distribution and Sales of Green-Bio Foods</t>
         </is>
       </c>
       <c r="I34" s="10" t="inlineStr">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Food Sales</t>
+          <t xml:space="preserve">Other Green-Bio Food Sales</t>
         </is>
       </c>
       <c r="I35" s="10" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Veterinary Medicine Wholesale</t>
+          <t xml:space="preserve">Green-Bio Veterinary Medicine Wholesale</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="H37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sales of Contract-Manufactured Green Bio Veterinary Medicines</t>
+          <t xml:space="preserve">Sales of Contract-Manufactured Green-Bio Veterinary Medicines</t>
         </is>
       </c>
       <c r="I37" s="10" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Sales and Distribution</t>
+          <t xml:space="preserve">Other Green-Bio Sales and Distribution</t>
         </is>
       </c>
       <c r="I38" s="10" t="inlineStr">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="H39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Seed Research and Development</t>
+          <t xml:space="preserve">Green-Bio Seed Research and Development</t>
         </is>
       </c>
       <c r="I39" s="10" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Microorganism Research and Development</t>
+          <t xml:space="preserve">Green-Bio Microorganism Research and Development</t>
         </is>
       </c>
       <c r="I40" s="10" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="H41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Insect Research and Development</t>
+          <t xml:space="preserve">Green-Bio Insect Research and Development</t>
         </is>
       </c>
       <c r="I41" s="10" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Other Green Bio Biological Resources</t>
+          <t xml:space="preserve">Research and Development of Other Green-Bio Biological Resources</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Agricultural Input Research and Development</t>
+          <t xml:space="preserve">Other Green-Bio Agricultural Input Research and Development</t>
         </is>
       </c>
       <c r="I46" s="10" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Food Ingredient Research and Development</t>
+          <t xml:space="preserve">Green-Bio Food Ingredient Research and Development</t>
         </is>
       </c>
       <c r="I47" s="10" t="inlineStr">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Health Functional Food Research and Development</t>
+          <t xml:space="preserve">Green-Bio Health Functional Food Research and Development</t>
         </is>
       </c>
       <c r="I48" s="10" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Green Bio Fermentation and Microbial Technologies for Food</t>
+          <t xml:space="preserve">Research and Development of Green-Bio Fermentation and Microbial Technologies for Food</t>
         </is>
       </c>
       <c r="I49" s="10" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Alternative Food Research and Development</t>
+          <t xml:space="preserve">Green-Bio Alternative Food Research and Development</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Green Bio Special Nutritional Foods and Foods for Special Medical Purposes</t>
+          <t xml:space="preserve">Research and Development of Green-Bio Special Nutritional Foods and Foods for Special Medical Purposes</t>
         </is>
       </c>
       <c r="I51" s="10" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Research and Development of Green Bio Food Ingredients and Products</t>
+          <t xml:space="preserve">Other Research and Development of Green-Bio Food Ingredients and Products</t>
         </is>
       </c>
       <c r="I52" s="10" t="inlineStr">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="H54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Veterinary Medicine Research and Development</t>
+          <t xml:space="preserve">Other Green-Bio Veterinary Medicine Research and Development</t>
         </is>
       </c>
       <c r="I54" s="10" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="H55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Green Bio Cosmetics and Personal Care Products</t>
+          <t xml:space="preserve">Research and Development of Green-Bio Cosmetics and Personal Care Products</t>
         </is>
       </c>
       <c r="I55" s="10" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="H56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Household Product Research and Development</t>
+          <t xml:space="preserve">Green-Bio Household Product Research and Development</t>
         </is>
       </c>
       <c r="I56" s="10" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="H57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Environmental Service Research and Development</t>
+          <t xml:space="preserve">Green-Bio Environmental Service Research and Development</t>
         </is>
       </c>
       <c r="I57" s="10" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Digital Service Research and Development</t>
+          <t xml:space="preserve">Green-Bio Digital Service Research and Development</t>
         </is>
       </c>
       <c r="I58" s="10" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Research and Development</t>
+          <t xml:space="preserve">Other Green-Bio Research and Development</t>
         </is>
       </c>
       <c r="I59" s="10" t="inlineStr">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Digital Breeding Services</t>
+          <t xml:space="preserve">Green-Bio Digital Breeding Services</t>
         </is>
       </c>
       <c r="I60" s="10" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Information and Data Services</t>
+          <t xml:space="preserve">Other Green-Bio Information and Data Services</t>
         </is>
       </c>
       <c r="I61" s="10" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="H62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Organic Waste Resource Treatment</t>
+          <t xml:space="preserve">Green-Bio Organic Waste Resource Treatment</t>
         </is>
       </c>
       <c r="I62" s="10" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="H63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Pest Control and Agricultural Environment Management</t>
+          <t xml:space="preserve">Green-Bio Pest Control and Agricultural Environment Management</t>
         </is>
       </c>
       <c r="I63" s="10" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="H64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Services</t>
+          <t xml:space="preserve">Other Green-Bio Services</t>
         </is>
       </c>
       <c r="I64" s="10" t="inlineStr">
@@ -3809,7 +3809,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Industry Special Classification · Round 6</t>
+          <t xml:space="preserve">Green-Bio Industry Special Classification · Round 6</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Production</t>
+          <t xml:space="preserve">Green-Bio Production</t>
         </is>
       </c>
       <c r="E4" s="10"/>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Seed Production</t>
+          <t xml:space="preserve">Green-Bio Seed Production</t>
         </is>
       </c>
       <c r="E5" s="10"/>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Seed Production</t>
+          <t xml:space="preserve">Green-Bio Seed Production</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Production of Plants for Green Bio Materials</t>
+          <t xml:space="preserve">Production of Plants for Green-Bio Materials</t>
         </is>
       </c>
       <c r="E7" s="10"/>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cannabis Cultivation for Green Bio Materials</t>
+          <t xml:space="preserve">Cannabis Cultivation for Green-Bio Materials</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Production of Other Plants for Green Bio Materials</t>
+          <t xml:space="preserve">Production of Other Plants for Green-Bio Materials</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Laboratory Animal Production</t>
+          <t xml:space="preserve">Green-Bio Laboratory Animal Production</t>
         </is>
       </c>
       <c r="E10" s="10"/>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Laboratory Animal Production</t>
+          <t xml:space="preserve">Green-Bio Laboratory Animal Production</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Production</t>
+          <t xml:space="preserve">Other Green-Bio Production</t>
         </is>
       </c>
       <c r="E12" s="10"/>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Production</t>
+          <t xml:space="preserve">Other Green-Bio Production</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Manufacturing</t>
         </is>
       </c>
       <c r="E14" s="10"/>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Material Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Material Manufacturing</t>
         </is>
       </c>
       <c r="E15" s="10"/>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manufacturing of Green Bio Materials Derived from Plants</t>
+          <t xml:space="preserve">Manufacturing of Green-Bio Materials Derived from Plants</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -4251,7 +4251,7 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manufacturing of Green Bio Materials Derived from Microorganisms</t>
+          <t xml:space="preserve">Manufacturing of Green-Bio Materials Derived from Microorganisms</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manufacturing of Green Bio Materials Derived from Insects</t>
+          <t xml:space="preserve">Manufacturing of Green-Bio Materials Derived from Insects</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -4315,7 +4315,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Material Manufacturing</t>
+          <t xml:space="preserve">Other Green-Bio Material Manufacturing</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Agricultural Input Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Agricultural Input Manufacturing</t>
         </is>
       </c>
       <c r="E20" s="10"/>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Agricultural Input Manufacturing</t>
+          <t xml:space="preserve">Other Green-Bio Agricultural Input Manufacturing</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Food Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Food Manufacturing</t>
         </is>
       </c>
       <c r="E25" s="10"/>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Food Additive Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Food Additive Manufacturing</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
@@ -4563,7 +4563,7 @@
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Fermented Food Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Fermented Food Manufacturing</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Health Functional Food Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Health Functional Food Manufacturing</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manufacturing of Green Bio Special Nutritional Foods and Foods for Special Medical Purposes</t>
+          <t xml:space="preserve">Manufacturing of Green-Bio Special Nutritional Foods and Foods for Special Medical Purposes</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Alternative Food Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Alternative Food Manufacturing</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
@@ -4691,7 +4691,7 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Food Manufacturing</t>
+          <t xml:space="preserve">Other Green-Bio Food Manufacturing</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Veterinary Medicine Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Veterinary Medicine Manufacturing</t>
         </is>
       </c>
       <c r="E32" s="10"/>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Veterinary Medicine Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Veterinary Medicine Manufacturing</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Product Manufacturing</t>
+          <t xml:space="preserve">Other Green-Bio Product Manufacturing</t>
         </is>
       </c>
       <c r="E34" s="10"/>
@@ -4811,7 +4811,7 @@
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manufacturing of Green Bio Cosmetics and Personal Care Products</t>
+          <t xml:space="preserve">Manufacturing of Green-Bio Cosmetics and Personal Care Products</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
@@ -4843,7 +4843,7 @@
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Household Product Manufacturing</t>
+          <t xml:space="preserve">Green-Bio Household Product Manufacturing</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Product Manufacturing</t>
+          <t xml:space="preserve">Other Green-Bio Product Manufacturing</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -4907,7 +4907,7 @@
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Sales and Distribution</t>
+          <t xml:space="preserve">Green-Bio Sales and Distribution</t>
         </is>
       </c>
       <c r="E38" s="10"/>
@@ -4935,7 +4935,7 @@
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Biological Resource and Material Sales and Distribution</t>
+          <t xml:space="preserve">Green-Bio Biological Resource and Material Sales and Distribution</t>
         </is>
       </c>
       <c r="E39" s="10"/>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Biological Resource and Material Sales and Distribution</t>
+          <t xml:space="preserve">Green-Bio Biological Resource and Material Sales and Distribution</t>
         </is>
       </c>
       <c r="E40" s="10" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Agricultural Input Sales</t>
+          <t xml:space="preserve">Green-Bio Agricultural Input Sales</t>
         </is>
       </c>
       <c r="E41" s="10"/>
@@ -5119,7 +5119,7 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Agricultural Input Sales</t>
+          <t xml:space="preserve">Other Green-Bio Agricultural Input Sales</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Food Sales</t>
+          <t xml:space="preserve">Green-Bio Food Sales</t>
         </is>
       </c>
       <c r="E46" s="10"/>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Health Functional Food Sales</t>
+          <t xml:space="preserve">Green-Bio Health Functional Food Sales</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customized Green Bio Health Functional Food Sales</t>
+          <t xml:space="preserve">Customized Green-Bio Health Functional Food Sales</t>
         </is>
       </c>
       <c r="E48" s="10" t="inlineStr">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Specialized Distribution and Sales of Green Bio Foods</t>
+          <t xml:space="preserve">Specialized Distribution and Sales of Green-Bio Foods</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
@@ -5275,7 +5275,7 @@
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Food Sales</t>
+          <t xml:space="preserve">Other Green-Bio Food Sales</t>
         </is>
       </c>
       <c r="E50" s="10" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Veterinary Medicine Sales and Distribution</t>
+          <t xml:space="preserve">Green-Bio Veterinary Medicine Sales and Distribution</t>
         </is>
       </c>
       <c r="E51" s="10"/>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Veterinary Medicine Wholesale</t>
+          <t xml:space="preserve">Green-Bio Veterinary Medicine Wholesale</t>
         </is>
       </c>
       <c r="E52" s="10" t="inlineStr">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sales of Contract-Manufactured Green Bio Veterinary Medicines</t>
+          <t xml:space="preserve">Sales of Contract-Manufactured Green-Bio Veterinary Medicines</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
@@ -5399,7 +5399,7 @@
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Sales and Distribution</t>
+          <t xml:space="preserve">Other Green-Bio Sales and Distribution</t>
         </is>
       </c>
       <c r="E54" s="10"/>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Sales and Distribution</t>
+          <t xml:space="preserve">Other Green-Bio Sales and Distribution</t>
         </is>
       </c>
       <c r="E55" s="10" t="inlineStr">
@@ -5459,7 +5459,7 @@
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Research and Development</t>
+          <t xml:space="preserve">Green-Bio Research and Development</t>
         </is>
       </c>
       <c r="E56" s="10"/>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Biological Resource Research and Development</t>
+          <t xml:space="preserve">Green-Bio Biological Resource Research and Development</t>
         </is>
       </c>
       <c r="E57" s="10"/>
@@ -5515,7 +5515,7 @@
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Seed Research and Development</t>
+          <t xml:space="preserve">Green-Bio Seed Research and Development</t>
         </is>
       </c>
       <c r="E58" s="10" t="inlineStr">
@@ -5547,7 +5547,7 @@
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Microorganism Research and Development</t>
+          <t xml:space="preserve">Green-Bio Microorganism Research and Development</t>
         </is>
       </c>
       <c r="E59" s="10" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Insect Research and Development</t>
+          <t xml:space="preserve">Green-Bio Insect Research and Development</t>
         </is>
       </c>
       <c r="E60" s="10" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Other Green Bio Biological Resources</t>
+          <t xml:space="preserve">Research and Development of Other Green-Bio Biological Resources</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Agricultural Input Research and Development</t>
+          <t xml:space="preserve">Green-Bio Agricultural Input Research and Development</t>
         </is>
       </c>
       <c r="E62" s="10"/>
@@ -5767,7 +5767,7 @@
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Agricultural Input Research and Development</t>
+          <t xml:space="preserve">Other Green-Bio Agricultural Input Research and Development</t>
         </is>
       </c>
       <c r="E66" s="10" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Green Bio Food Ingredients and Products</t>
+          <t xml:space="preserve">Research and Development of Green-Bio Food Ingredients and Products</t>
         </is>
       </c>
       <c r="E67" s="10"/>
@@ -5827,7 +5827,7 @@
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Food Ingredient Research and Development</t>
+          <t xml:space="preserve">Green-Bio Food Ingredient Research and Development</t>
         </is>
       </c>
       <c r="E68" s="10" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Health Functional Food Research and Development</t>
+          <t xml:space="preserve">Green-Bio Health Functional Food Research and Development</t>
         </is>
       </c>
       <c r="E69" s="10" t="inlineStr">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Green Bio Fermentation and Microbial Technologies for Food</t>
+          <t xml:space="preserve">Research and Development of Green-Bio Fermentation and Microbial Technologies for Food</t>
         </is>
       </c>
       <c r="E70" s="10" t="inlineStr">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Alternative Food Research and Development</t>
+          <t xml:space="preserve">Green-Bio Alternative Food Research and Development</t>
         </is>
       </c>
       <c r="E71" s="10" t="inlineStr">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Green Bio Special Nutritional Foods and Foods for Special Medical Purposes</t>
+          <t xml:space="preserve">Research and Development of Green-Bio Special Nutritional Foods and Foods for Special Medical Purposes</t>
         </is>
       </c>
       <c r="E72" s="10" t="inlineStr">
@@ -5987,7 +5987,7 @@
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Research and Development of Green Bio Food Ingredients and Products</t>
+          <t xml:space="preserve">Other Research and Development of Green-Bio Food Ingredients and Products</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Veterinary Medicine Research and Development</t>
+          <t xml:space="preserve">Green-Bio Veterinary Medicine Research and Development</t>
         </is>
       </c>
       <c r="E74" s="10"/>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Veterinary Medicine Research and Development</t>
+          <t xml:space="preserve">Other Green-Bio Veterinary Medicine Research and Development</t>
         </is>
       </c>
       <c r="E76" s="10" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Green Bio Cosmetics and Household Products</t>
+          <t xml:space="preserve">Research and Development of Green-Bio Cosmetics and Household Products</t>
         </is>
       </c>
       <c r="E77" s="10"/>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Green Bio Cosmetics and Personal Care Products</t>
+          <t xml:space="preserve">Research and Development of Green-Bio Cosmetics and Personal Care Products</t>
         </is>
       </c>
       <c r="E78" s="10" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Household Product Research and Development</t>
+          <t xml:space="preserve">Green-Bio Household Product Research and Development</t>
         </is>
       </c>
       <c r="E79" s="10" t="inlineStr">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research and Development of Green Bio Environmental and Digital Services</t>
+          <t xml:space="preserve">Research and Development of Green-Bio Environmental and Digital Services</t>
         </is>
       </c>
       <c r="E80" s="10"/>
@@ -6231,7 +6231,7 @@
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Environmental Service Research and Development</t>
+          <t xml:space="preserve">Green-Bio Environmental Service Research and Development</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Digital Service Research and Development</t>
+          <t xml:space="preserve">Green-Bio Digital Service Research and Development</t>
         </is>
       </c>
       <c r="E82" s="10" t="inlineStr">
@@ -6295,7 +6295,7 @@
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Research and Development</t>
+          <t xml:space="preserve">Other Green-Bio Research and Development</t>
         </is>
       </c>
       <c r="E83" s="10"/>
@@ -6323,7 +6323,7 @@
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Research and Development</t>
+          <t xml:space="preserve">Other Green-Bio Research and Development</t>
         </is>
       </c>
       <c r="E84" s="10" t="inlineStr">
@@ -6355,7 +6355,7 @@
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Information, Environmental and Other Services</t>
+          <t xml:space="preserve">Green-Bio Information, Environmental and Other Services</t>
         </is>
       </c>
       <c r="E85" s="10"/>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Information and Data Services</t>
+          <t xml:space="preserve">Green-Bio Information and Data Services</t>
         </is>
       </c>
       <c r="E86" s="10"/>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Digital Breeding Services</t>
+          <t xml:space="preserve">Green-Bio Digital Breeding Services</t>
         </is>
       </c>
       <c r="E87" s="10" t="inlineStr">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Information and Data Services</t>
+          <t xml:space="preserve">Other Green-Bio Information and Data Services</t>
         </is>
       </c>
       <c r="E88" s="10" t="inlineStr">
@@ -6475,7 +6475,7 @@
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Environmental Services</t>
+          <t xml:space="preserve">Green-Bio Environmental Services</t>
         </is>
       </c>
       <c r="E89" s="10"/>
@@ -6503,7 +6503,7 @@
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Organic Waste Resource Treatment</t>
+          <t xml:space="preserve">Green-Bio Organic Waste Resource Treatment</t>
         </is>
       </c>
       <c r="E90" s="10" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green Bio Pest Control and Agricultural Environment Management</t>
+          <t xml:space="preserve">Green-Bio Pest Control and Agricultural Environment Management</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Services</t>
+          <t xml:space="preserve">Other Green-Bio Services</t>
         </is>
       </c>
       <c r="E92" s="10"/>
@@ -6595,7 +6595,7 @@
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Green Bio Services</t>
+          <t xml:space="preserve">Other Green-Bio Services</t>
         </is>
       </c>
       <c r="E93" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Merge class cells across crosswalk sheet links
</commit_message>
<xml_diff>
--- a/xlsx/그린바이오산업_특수분류표_6차.xlsx
+++ b/xlsx/그린바이오산업_특수분류표_6차.xlsx
@@ -7206,16 +7206,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">110</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 종자 생산업</t>
-        </is>
-      </c>
+      <c r="A5" s="8"/>
+      <c r="B5" s="10"/>
       <c r="C5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">02011</t>
@@ -7272,16 +7264,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A8" s="8"/>
+      <c r="B8" s="10"/>
       <c r="C8" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">01121</t>
@@ -7294,16 +7278,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A9" s="8"/>
+      <c r="B9" s="10"/>
       <c r="C9" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">01122</t>
@@ -7316,16 +7292,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A10" s="8"/>
+      <c r="B10" s="10"/>
       <c r="C10" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">01131</t>
@@ -7338,16 +7306,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A11" s="8"/>
+      <c r="B11" s="10"/>
       <c r="C11" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">01132</t>
@@ -7360,16 +7320,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A12" s="8"/>
+      <c r="B12" s="10"/>
       <c r="C12" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">01140</t>
@@ -7382,16 +7334,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A13" s="8"/>
+      <c r="B13" s="10"/>
       <c r="C13" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">01151</t>
@@ -7404,16 +7348,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A14" s="8"/>
+      <c r="B14" s="10"/>
       <c r="C14" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">01159</t>
@@ -7470,16 +7406,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">190</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생산업</t>
-        </is>
-      </c>
+      <c r="A17" s="8"/>
+      <c r="B17" s="10"/>
       <c r="C17" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21100</t>
@@ -7492,16 +7420,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">190</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생산업</t>
-        </is>
-      </c>
+      <c r="A18" s="8"/>
+      <c r="B18" s="10"/>
       <c r="C18" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">03211</t>
@@ -7514,16 +7434,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">190</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생산업</t>
-        </is>
-      </c>
+      <c r="A19" s="8"/>
+      <c r="B19" s="10"/>
       <c r="C19" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">03212</t>
@@ -7536,16 +7448,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">190</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생산업</t>
-        </is>
-      </c>
+      <c r="A20" s="8"/>
+      <c r="B20" s="10"/>
       <c r="C20" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">03213</t>
@@ -7558,16 +7462,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">190</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생산업</t>
-        </is>
-      </c>
+      <c r="A21" s="8"/>
+      <c r="B21" s="10"/>
       <c r="C21" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10839</t>
@@ -7602,16 +7498,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">211</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A23" s="8"/>
+      <c r="B23" s="10"/>
       <c r="C23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10839</t>
@@ -7624,16 +7512,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">211</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A24" s="8"/>
+      <c r="B24" s="10"/>
       <c r="C24" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">20119</t>
@@ -7668,16 +7548,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">212</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A26" s="8"/>
+      <c r="B26" s="10"/>
       <c r="C26" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">20499</t>
@@ -7690,16 +7562,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">212</t>
-        </is>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A27" s="8"/>
+      <c r="B27" s="10"/>
       <c r="C27" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">20119</t>
@@ -7734,16 +7598,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">213</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 곤충 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A29" s="8"/>
+      <c r="B29" s="10"/>
       <c r="C29" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10839</t>
@@ -7778,16 +7634,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">219</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A31" s="8"/>
+      <c r="B31" s="10"/>
       <c r="C31" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21100</t>
@@ -7800,16 +7648,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">219</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A32" s="8"/>
+      <c r="B32" s="10"/>
       <c r="C32" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">20119</t>
@@ -7822,16 +7662,8 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">219</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A33" s="8"/>
+      <c r="B33" s="10"/>
       <c r="C33" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21220</t>
@@ -7910,16 +7742,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">223</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오사료 제조업</t>
-        </is>
-      </c>
+      <c r="A37" s="8"/>
+      <c r="B37" s="10"/>
       <c r="C37" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10903</t>
@@ -7932,16 +7756,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">223</t>
-        </is>
-      </c>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오사료 제조업</t>
-        </is>
-      </c>
+      <c r="A38" s="8"/>
+      <c r="B38" s="10"/>
       <c r="C38" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10901</t>
@@ -7954,16 +7770,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">223</t>
-        </is>
-      </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오사료 제조업</t>
-        </is>
-      </c>
+      <c r="A39" s="8"/>
+      <c r="B39" s="10"/>
       <c r="C39" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">20119</t>
@@ -7998,16 +7806,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">229</t>
-        </is>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
-        </is>
-      </c>
+      <c r="A41" s="8"/>
+      <c r="B41" s="10"/>
       <c r="C41" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">20499</t>
@@ -8042,16 +7842,8 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">231</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
-        </is>
-      </c>
+      <c r="A43" s="8"/>
+      <c r="B43" s="10"/>
       <c r="C43" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10831</t>
@@ -8064,16 +7856,8 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">231</t>
-        </is>
-      </c>
-      <c r="B44" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
-        </is>
-      </c>
+      <c r="A44" s="8"/>
+      <c r="B44" s="10"/>
       <c r="C44" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10832</t>
@@ -8086,16 +7870,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">231</t>
-        </is>
-      </c>
-      <c r="B45" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품첨가물 제조업</t>
-        </is>
-      </c>
+      <c r="A45" s="8"/>
+      <c r="B45" s="10"/>
       <c r="C45" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">20119</t>
@@ -8130,16 +7906,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A47" s="8"/>
+      <c r="B47" s="10"/>
       <c r="C47" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10302</t>
@@ -8152,16 +7920,8 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A48" s="8"/>
+      <c r="B48" s="10"/>
       <c r="C48" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10309</t>
@@ -8174,16 +7934,8 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A49" s="8"/>
+      <c r="B49" s="10"/>
       <c r="C49" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10421</t>
@@ -8196,16 +7948,8 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A50" s="8"/>
+      <c r="B50" s="10"/>
       <c r="C50" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10422</t>
@@ -8218,16 +7962,8 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B51" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A51" s="8"/>
+      <c r="B51" s="10"/>
       <c r="C51" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10831</t>
@@ -8240,16 +7976,8 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B52" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A52" s="8"/>
+      <c r="B52" s="10"/>
       <c r="C52" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10833</t>
@@ -8262,16 +7990,8 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B53" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A53" s="8"/>
+      <c r="B53" s="10"/>
       <c r="C53" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10839</t>
@@ -8284,16 +8004,8 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B54" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A54" s="8"/>
+      <c r="B54" s="10"/>
       <c r="C54" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">11111</t>
@@ -8306,16 +8018,8 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B55" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A55" s="8"/>
+      <c r="B55" s="10"/>
       <c r="C55" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">11112</t>
@@ -8328,16 +8032,8 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A56" s="8"/>
+      <c r="B56" s="10"/>
       <c r="C56" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">11119</t>
@@ -8350,16 +8046,8 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B57" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A57" s="8"/>
+      <c r="B57" s="10"/>
       <c r="C57" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">11121</t>
@@ -8394,16 +8082,8 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">233</t>
-        </is>
-      </c>
-      <c r="B59" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
-        </is>
-      </c>
+      <c r="A59" s="8"/>
+      <c r="B59" s="10"/>
       <c r="C59" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10895</t>
@@ -8416,16 +8096,8 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">233</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
-        </is>
-      </c>
+      <c r="A60" s="8"/>
+      <c r="B60" s="10"/>
       <c r="C60" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10896</t>
@@ -8460,16 +8132,8 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">234</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
-        </is>
-      </c>
+      <c r="A62" s="8"/>
+      <c r="B62" s="10"/>
       <c r="C62" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10893</t>
@@ -8482,16 +8146,8 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">234</t>
-        </is>
-      </c>
-      <c r="B63" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
-        </is>
-      </c>
+      <c r="A63" s="8"/>
+      <c r="B63" s="10"/>
       <c r="C63" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10701</t>
@@ -8504,16 +8160,8 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">234</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
-        </is>
-      </c>
+      <c r="A64" s="8"/>
+      <c r="B64" s="10"/>
       <c r="C64" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10709</t>
@@ -8526,16 +8174,8 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">234</t>
-        </is>
-      </c>
-      <c r="B65" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
-        </is>
-      </c>
+      <c r="A65" s="8"/>
+      <c r="B65" s="10"/>
       <c r="C65" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10892</t>
@@ -8548,16 +8188,8 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">234</t>
-        </is>
-      </c>
-      <c r="B66" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 제조업</t>
-        </is>
-      </c>
+      <c r="A66" s="8"/>
+      <c r="B66" s="10"/>
       <c r="C66" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10899</t>
@@ -8592,16 +8224,8 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">235</t>
-        </is>
-      </c>
-      <c r="B68" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
-        </is>
-      </c>
+      <c r="A68" s="8"/>
+      <c r="B68" s="10"/>
       <c r="C68" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10519</t>
@@ -8614,16 +8238,8 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">235</t>
-        </is>
-      </c>
-      <c r="B69" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
-        </is>
-      </c>
+      <c r="A69" s="8"/>
+      <c r="B69" s="10"/>
       <c r="C69" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10520</t>
@@ -8636,16 +8252,8 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">235</t>
-        </is>
-      </c>
-      <c r="B70" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
-        </is>
-      </c>
+      <c r="A70" s="8"/>
+      <c r="B70" s="10"/>
       <c r="C70" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10894</t>
@@ -8658,16 +8266,8 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">235</t>
-        </is>
-      </c>
-      <c r="B71" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
-        </is>
-      </c>
+      <c r="A71" s="8"/>
+      <c r="B71" s="10"/>
       <c r="C71" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10899</t>
@@ -8702,16 +8302,8 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">239</t>
-        </is>
-      </c>
-      <c r="B73" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
-        </is>
-      </c>
+      <c r="A73" s="8"/>
+      <c r="B73" s="10"/>
       <c r="C73" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10709</t>
@@ -8724,16 +8316,8 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">239</t>
-        </is>
-      </c>
-      <c r="B74" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
-        </is>
-      </c>
+      <c r="A74" s="8"/>
+      <c r="B74" s="10"/>
       <c r="C74" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10839</t>
@@ -8746,16 +8330,8 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">239</t>
-        </is>
-      </c>
-      <c r="B75" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
-        </is>
-      </c>
+      <c r="A75" s="8"/>
+      <c r="B75" s="10"/>
       <c r="C75" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">10899</t>
@@ -8790,16 +8366,8 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">240</t>
-        </is>
-      </c>
-      <c r="B77" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
-        </is>
-      </c>
+      <c r="A77" s="8"/>
+      <c r="B77" s="10"/>
       <c r="C77" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21100</t>
@@ -8812,16 +8380,8 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">240</t>
-        </is>
-      </c>
-      <c r="B78" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
-        </is>
-      </c>
+      <c r="A78" s="8"/>
+      <c r="B78" s="10"/>
       <c r="C78" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21211</t>
@@ -8856,16 +8416,8 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">291</t>
-        </is>
-      </c>
-      <c r="B80" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 향장제품 제조업</t>
-        </is>
-      </c>
+      <c r="A80" s="8"/>
+      <c r="B80" s="10"/>
       <c r="C80" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">20424</t>
@@ -8900,16 +8452,8 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">292</t>
-        </is>
-      </c>
-      <c r="B82" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
-        </is>
-      </c>
+      <c r="A82" s="8"/>
+      <c r="B82" s="10"/>
       <c r="C82" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">20424</t>
@@ -8922,16 +8466,8 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">292</t>
-        </is>
-      </c>
-      <c r="B83" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
-        </is>
-      </c>
+      <c r="A83" s="8"/>
+      <c r="B83" s="10"/>
       <c r="C83" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">15190</t>
@@ -8966,16 +8502,8 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">299</t>
-        </is>
-      </c>
-      <c r="B85" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
-        </is>
-      </c>
+      <c r="A85" s="8"/>
+      <c r="B85" s="10"/>
       <c r="C85" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">20203</t>
@@ -9010,16 +8538,8 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">310</t>
-        </is>
-      </c>
-      <c r="B87" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
-        </is>
-      </c>
+      <c r="A87" s="8"/>
+      <c r="B87" s="10"/>
       <c r="C87" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">46102</t>
@@ -9120,16 +8640,8 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">329</t>
-        </is>
-      </c>
-      <c r="B92" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
-        </is>
-      </c>
+      <c r="A92" s="8"/>
+      <c r="B92" s="10"/>
       <c r="C92" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">46203</t>
@@ -9164,16 +8676,8 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">331</t>
-        </is>
-      </c>
-      <c r="B94" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
-        </is>
-      </c>
+      <c r="A94" s="8"/>
+      <c r="B94" s="10"/>
       <c r="C94" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">46443</t>
@@ -9230,16 +8734,8 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">333</t>
-        </is>
-      </c>
-      <c r="B97" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품 유통전문판매업</t>
-        </is>
-      </c>
+      <c r="A97" s="8"/>
+      <c r="B97" s="10"/>
       <c r="C97" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">46319</t>
@@ -9274,16 +8770,8 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">339</t>
-        </is>
-      </c>
-      <c r="B99" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
-        </is>
-      </c>
+      <c r="A99" s="8"/>
+      <c r="B99" s="10"/>
       <c r="C99" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">46319</t>
@@ -9296,16 +8784,8 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">339</t>
-        </is>
-      </c>
-      <c r="B100" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
-        </is>
-      </c>
+      <c r="A100" s="8"/>
+      <c r="B100" s="10"/>
       <c r="C100" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">47211</t>
@@ -9318,16 +8798,8 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">339</t>
-        </is>
-      </c>
-      <c r="B101" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
-        </is>
-      </c>
+      <c r="A101" s="8"/>
+      <c r="B101" s="10"/>
       <c r="C101" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">47219</t>
@@ -9406,16 +8878,8 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">390</t>
-        </is>
-      </c>
-      <c r="B105" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
-        </is>
-      </c>
+      <c r="A105" s="8"/>
+      <c r="B105" s="10"/>
       <c r="C105" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">47859</t>
@@ -9428,16 +8892,8 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">390</t>
-        </is>
-      </c>
-      <c r="B106" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 판매·유통업</t>
-        </is>
-      </c>
+      <c r="A106" s="8"/>
+      <c r="B106" s="10"/>
       <c r="C106" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">47999</t>
@@ -9472,16 +8928,8 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">411</t>
-        </is>
-      </c>
-      <c r="B108" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
-        </is>
-      </c>
+      <c r="A108" s="8"/>
+      <c r="B108" s="10"/>
       <c r="C108" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -9494,16 +8942,8 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">411</t>
-        </is>
-      </c>
-      <c r="B109" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
-        </is>
-      </c>
+      <c r="A109" s="8"/>
+      <c r="B109" s="10"/>
       <c r="C109" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -9538,16 +8978,8 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">412</t>
-        </is>
-      </c>
-      <c r="B111" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
-        </is>
-      </c>
+      <c r="A111" s="8"/>
+      <c r="B111" s="10"/>
       <c r="C111" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -9560,16 +8992,8 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">412</t>
-        </is>
-      </c>
-      <c r="B112" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
-        </is>
-      </c>
+      <c r="A112" s="8"/>
+      <c r="B112" s="10"/>
       <c r="C112" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -9604,16 +9028,8 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">413</t>
-        </is>
-      </c>
-      <c r="B114" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
-        </is>
-      </c>
+      <c r="A114" s="8"/>
+      <c r="B114" s="10"/>
       <c r="C114" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -9626,16 +9042,8 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">413</t>
-        </is>
-      </c>
-      <c r="B115" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
-        </is>
-      </c>
+      <c r="A115" s="8"/>
+      <c r="B115" s="10"/>
       <c r="C115" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -9670,16 +9078,8 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">419</t>
-        </is>
-      </c>
-      <c r="B117" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
-        </is>
-      </c>
+      <c r="A117" s="8"/>
+      <c r="B117" s="10"/>
       <c r="C117" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -9692,16 +9092,8 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">419</t>
-        </is>
-      </c>
-      <c r="B118" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
-        </is>
-      </c>
+      <c r="A118" s="8"/>
+      <c r="B118" s="10"/>
       <c r="C118" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -9736,16 +9128,8 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">421</t>
-        </is>
-      </c>
-      <c r="B120" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
-        </is>
-      </c>
+      <c r="A120" s="8"/>
+      <c r="B120" s="10"/>
       <c r="C120" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -9758,16 +9142,8 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">421</t>
-        </is>
-      </c>
-      <c r="B121" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
-        </is>
-      </c>
+      <c r="A121" s="8"/>
+      <c r="B121" s="10"/>
       <c r="C121" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -9802,16 +9178,8 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">422</t>
-        </is>
-      </c>
-      <c r="B123" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
-        </is>
-      </c>
+      <c r="A123" s="8"/>
+      <c r="B123" s="10"/>
       <c r="C123" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -9824,16 +9192,8 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">422</t>
-        </is>
-      </c>
-      <c r="B124" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
-        </is>
-      </c>
+      <c r="A124" s="8"/>
+      <c r="B124" s="10"/>
       <c r="C124" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -9868,16 +9228,8 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">423</t>
-        </is>
-      </c>
-      <c r="B126" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
-        </is>
-      </c>
+      <c r="A126" s="8"/>
+      <c r="B126" s="10"/>
       <c r="C126" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -9890,16 +9242,8 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">423</t>
-        </is>
-      </c>
-      <c r="B127" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
-        </is>
-      </c>
+      <c r="A127" s="8"/>
+      <c r="B127" s="10"/>
       <c r="C127" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -9934,16 +9278,8 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">429</t>
-        </is>
-      </c>
-      <c r="B129" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
-        </is>
-      </c>
+      <c r="A129" s="8"/>
+      <c r="B129" s="10"/>
       <c r="C129" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -9956,16 +9292,8 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">429</t>
-        </is>
-      </c>
-      <c r="B130" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
-        </is>
-      </c>
+      <c r="A130" s="8"/>
+      <c r="B130" s="10"/>
       <c r="C130" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -10000,16 +9328,8 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">431</t>
-        </is>
-      </c>
-      <c r="B132" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
-        </is>
-      </c>
+      <c r="A132" s="8"/>
+      <c r="B132" s="10"/>
       <c r="C132" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70112</t>
@@ -10022,16 +9342,8 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">431</t>
-        </is>
-      </c>
-      <c r="B133" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
-        </is>
-      </c>
+      <c r="A133" s="8"/>
+      <c r="B133" s="10"/>
       <c r="C133" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -10066,16 +9378,8 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">432</t>
-        </is>
-      </c>
-      <c r="B135" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A135" s="8"/>
+      <c r="B135" s="10"/>
       <c r="C135" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70112</t>
@@ -10088,16 +9392,8 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">432</t>
-        </is>
-      </c>
-      <c r="B136" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A136" s="8"/>
+      <c r="B136" s="10"/>
       <c r="C136" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -10132,16 +9428,8 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">433</t>
-        </is>
-      </c>
-      <c r="B138" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
-        </is>
-      </c>
+      <c r="A138" s="8"/>
+      <c r="B138" s="10"/>
       <c r="C138" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70112</t>
@@ -10154,16 +9442,8 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">433</t>
-        </is>
-      </c>
-      <c r="B139" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
-        </is>
-      </c>
+      <c r="A139" s="8"/>
+      <c r="B139" s="10"/>
       <c r="C139" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -10198,16 +9478,8 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">434</t>
-        </is>
-      </c>
-      <c r="B141" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A141" s="8"/>
+      <c r="B141" s="10"/>
       <c r="C141" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70112</t>
@@ -10220,16 +9492,8 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">434</t>
-        </is>
-      </c>
-      <c r="B142" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A142" s="8"/>
+      <c r="B142" s="10"/>
       <c r="C142" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -10264,16 +9528,8 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">435</t>
-        </is>
-      </c>
-      <c r="B144" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A144" s="8"/>
+      <c r="B144" s="10"/>
       <c r="C144" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70112</t>
@@ -10286,16 +9542,8 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">435</t>
-        </is>
-      </c>
-      <c r="B145" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A145" s="8"/>
+      <c r="B145" s="10"/>
       <c r="C145" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -10330,16 +9578,8 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">439</t>
-        </is>
-      </c>
-      <c r="B147" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A147" s="8"/>
+      <c r="B147" s="10"/>
       <c r="C147" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70112</t>
@@ -10352,16 +9592,8 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">439</t>
-        </is>
-      </c>
-      <c r="B148" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A148" s="8"/>
+      <c r="B148" s="10"/>
       <c r="C148" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -10396,16 +9628,8 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">441</t>
-        </is>
-      </c>
-      <c r="B150" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
-        </is>
-      </c>
+      <c r="A150" s="8"/>
+      <c r="B150" s="10"/>
       <c r="C150" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70112</t>
@@ -10418,16 +9642,8 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">441</t>
-        </is>
-      </c>
-      <c r="B151" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
-        </is>
-      </c>
+      <c r="A151" s="8"/>
+      <c r="B151" s="10"/>
       <c r="C151" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -10462,16 +9678,8 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">449</t>
-        </is>
-      </c>
-      <c r="B153" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A153" s="8"/>
+      <c r="B153" s="10"/>
       <c r="C153" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70112</t>
@@ -10484,16 +9692,8 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">449</t>
-        </is>
-      </c>
-      <c r="B154" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A154" s="8"/>
+      <c r="B154" s="10"/>
       <c r="C154" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -10528,16 +9728,8 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">451</t>
-        </is>
-      </c>
-      <c r="B156" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A156" s="8"/>
+      <c r="B156" s="10"/>
       <c r="C156" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -10572,16 +9764,8 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">452</t>
-        </is>
-      </c>
-      <c r="B158" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A158" s="8"/>
+      <c r="B158" s="10"/>
       <c r="C158" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -10616,16 +9800,8 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">461</t>
-        </is>
-      </c>
-      <c r="B160" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
-        </is>
-      </c>
+      <c r="A160" s="8"/>
+      <c r="B160" s="10"/>
       <c r="C160" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -10660,16 +9836,8 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">462</t>
-        </is>
-      </c>
-      <c r="B162" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
-        </is>
-      </c>
+      <c r="A162" s="8"/>
+      <c r="B162" s="10"/>
       <c r="C162" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70111</t>
@@ -10704,16 +9872,8 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">490</t>
-        </is>
-      </c>
-      <c r="B164" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
-        </is>
-      </c>
+      <c r="A164" s="8"/>
+      <c r="B164" s="10"/>
       <c r="C164" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70112</t>
@@ -10726,16 +9886,8 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">490</t>
-        </is>
-      </c>
-      <c r="B165" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
-        </is>
-      </c>
+      <c r="A165" s="8"/>
+      <c r="B165" s="10"/>
       <c r="C165" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">70130</t>
@@ -10770,16 +9922,8 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">521</t>
-        </is>
-      </c>
-      <c r="B167" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
-        </is>
-      </c>
+      <c r="A167" s="8"/>
+      <c r="B167" s="10"/>
       <c r="C167" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">63111</t>
@@ -10814,16 +9958,8 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">529</t>
-        </is>
-      </c>
-      <c r="B169" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
-        </is>
-      </c>
+      <c r="A169" s="8"/>
+      <c r="B169" s="10"/>
       <c r="C169" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">63991</t>
@@ -10836,16 +9972,8 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">529</t>
-        </is>
-      </c>
-      <c r="B170" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
-        </is>
-      </c>
+      <c r="A170" s="8"/>
+      <c r="B170" s="10"/>
       <c r="C170" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">62010</t>
@@ -10858,16 +9986,8 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">529</t>
-        </is>
-      </c>
-      <c r="B171" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
-        </is>
-      </c>
+      <c r="A171" s="8"/>
+      <c r="B171" s="10"/>
       <c r="C171" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">58222</t>
@@ -10902,16 +10022,8 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">531</t>
-        </is>
-      </c>
-      <c r="B173" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
-        </is>
-      </c>
+      <c r="A173" s="8"/>
+      <c r="B173" s="10"/>
       <c r="C173" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">38210</t>
@@ -10946,16 +10058,8 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">532</t>
-        </is>
-      </c>
-      <c r="B175" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
-        </is>
-      </c>
+      <c r="A175" s="8"/>
+      <c r="B175" s="10"/>
       <c r="C175" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">01411</t>
@@ -10990,16 +10094,8 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B177" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
+      <c r="A177" s="8"/>
+      <c r="B177" s="10"/>
       <c r="C177" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">72911</t>
@@ -11012,16 +10108,8 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B178" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
+      <c r="A178" s="8"/>
+      <c r="B178" s="10"/>
       <c r="C178" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">72919</t>
@@ -11034,16 +10122,8 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B179" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
+      <c r="A179" s="8"/>
+      <c r="B179" s="10"/>
       <c r="C179" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">52109</t>
@@ -11056,16 +10136,8 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B180" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
+      <c r="A180" s="8"/>
+      <c r="B180" s="10"/>
       <c r="C180" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">52101</t>
@@ -11078,8 +10150,110 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="103">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A7:A14"/>
+    <mergeCell ref="B7:B14"/>
+    <mergeCell ref="A16:A21"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="A36:A39"/>
+    <mergeCell ref="B36:B39"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="A46:A57"/>
+    <mergeCell ref="B46:B57"/>
+    <mergeCell ref="A58:A60"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="A61:A66"/>
+    <mergeCell ref="B61:B66"/>
+    <mergeCell ref="A67:A71"/>
+    <mergeCell ref="B67:B71"/>
+    <mergeCell ref="A72:A75"/>
+    <mergeCell ref="B72:B75"/>
+    <mergeCell ref="A76:A78"/>
+    <mergeCell ref="B76:B78"/>
+    <mergeCell ref="A79:A80"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="A81:A83"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="A86:A87"/>
+    <mergeCell ref="B86:B87"/>
+    <mergeCell ref="A91:A92"/>
+    <mergeCell ref="B91:B92"/>
+    <mergeCell ref="A93:A94"/>
+    <mergeCell ref="B93:B94"/>
+    <mergeCell ref="A96:A97"/>
+    <mergeCell ref="B96:B97"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="B104:B106"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="B107:B109"/>
+    <mergeCell ref="A110:A112"/>
+    <mergeCell ref="B110:B112"/>
+    <mergeCell ref="A113:A115"/>
+    <mergeCell ref="B113:B115"/>
+    <mergeCell ref="A116:A118"/>
+    <mergeCell ref="B116:B118"/>
+    <mergeCell ref="A119:A121"/>
+    <mergeCell ref="B119:B121"/>
+    <mergeCell ref="A122:A124"/>
+    <mergeCell ref="B122:B124"/>
+    <mergeCell ref="A125:A127"/>
+    <mergeCell ref="B125:B127"/>
+    <mergeCell ref="A128:A130"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="A131:A133"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="A134:A136"/>
+    <mergeCell ref="B134:B136"/>
+    <mergeCell ref="A137:A139"/>
+    <mergeCell ref="B137:B139"/>
+    <mergeCell ref="A140:A142"/>
+    <mergeCell ref="B140:B142"/>
+    <mergeCell ref="A143:A145"/>
+    <mergeCell ref="B143:B145"/>
+    <mergeCell ref="A146:A148"/>
+    <mergeCell ref="B146:B148"/>
+    <mergeCell ref="A149:A151"/>
+    <mergeCell ref="B149:B151"/>
+    <mergeCell ref="A152:A154"/>
+    <mergeCell ref="B152:B154"/>
+    <mergeCell ref="A155:A156"/>
+    <mergeCell ref="B155:B156"/>
+    <mergeCell ref="A157:A158"/>
+    <mergeCell ref="B157:B158"/>
+    <mergeCell ref="A159:A160"/>
+    <mergeCell ref="B159:B160"/>
+    <mergeCell ref="A161:A162"/>
+    <mergeCell ref="B161:B162"/>
+    <mergeCell ref="A163:A165"/>
+    <mergeCell ref="B163:B165"/>
+    <mergeCell ref="A166:A167"/>
+    <mergeCell ref="B166:B167"/>
+    <mergeCell ref="A168:A171"/>
+    <mergeCell ref="B168:B171"/>
+    <mergeCell ref="A172:A173"/>
+    <mergeCell ref="B172:B173"/>
+    <mergeCell ref="A174:A175"/>
+    <mergeCell ref="B174:B175"/>
+    <mergeCell ref="A176:A180"/>
+    <mergeCell ref="B176:B180"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11147,16 +10321,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">110</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 종자 생산업</t>
-        </is>
-      </c>
+      <c r="A5" s="8"/>
+      <c r="B5" s="10"/>
       <c r="C5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21250</t>
@@ -11191,16 +10357,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">121</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 소재용 대마 재배업</t>
-        </is>
-      </c>
+      <c r="A7" s="8"/>
+      <c r="B7" s="10"/>
       <c r="C7" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21290</t>
@@ -11235,16 +10393,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A9" s="8"/>
+      <c r="B9" s="10"/>
       <c r="C9" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21151</t>
@@ -11257,16 +10407,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A10" s="8"/>
+      <c r="B10" s="10"/>
       <c r="C10" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21152</t>
@@ -11279,16 +10421,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A11" s="8"/>
+      <c r="B11" s="10"/>
       <c r="C11" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21190</t>
@@ -11301,16 +10435,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A12" s="8"/>
+      <c r="B12" s="10"/>
       <c r="C12" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21242</t>
@@ -11323,16 +10449,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">129</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재용 식물 생산업</t>
-        </is>
-      </c>
+      <c r="A13" s="8"/>
+      <c r="B13" s="10"/>
       <c r="C13" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">21290</t>
@@ -11389,16 +10507,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">190</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생산업</t>
-        </is>
-      </c>
+      <c r="A16" s="8"/>
+      <c r="B16" s="10"/>
       <c r="C16" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">22620</t>
@@ -11411,16 +10521,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">190</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생산업</t>
-        </is>
-      </c>
+      <c r="A17" s="8"/>
+      <c r="B17" s="10"/>
       <c r="C17" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">22690</t>
@@ -11433,16 +10535,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">190</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생산업</t>
-        </is>
-      </c>
+      <c r="A18" s="8"/>
+      <c r="B18" s="10"/>
       <c r="C18" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">22900</t>
@@ -11455,16 +10549,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">190</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생산업</t>
-        </is>
-      </c>
+      <c r="A19" s="8"/>
+      <c r="B19" s="10"/>
       <c r="C19" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">31164</t>
@@ -11499,16 +10585,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">211</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A21" s="8"/>
+      <c r="B21" s="10"/>
       <c r="C21" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">33910</t>
@@ -11543,16 +10621,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">212</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A23" s="8"/>
+      <c r="B23" s="10"/>
       <c r="C23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">31169</t>
@@ -11675,16 +10745,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">223</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오사료 제조업</t>
-        </is>
-      </c>
+      <c r="A29" s="8"/>
+      <c r="B29" s="10"/>
       <c r="C29" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">11162</t>
@@ -11697,16 +10759,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">223</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오사료 제조업</t>
-        </is>
-      </c>
+      <c r="A30" s="8"/>
+      <c r="B30" s="10"/>
       <c r="C30" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">11163</t>
@@ -11741,16 +10795,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">229</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
-        </is>
-      </c>
+      <c r="A32" s="8"/>
+      <c r="B32" s="10"/>
       <c r="C32" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">11199</t>
@@ -11807,16 +10853,8 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A35" s="8"/>
+      <c r="B35" s="10"/>
       <c r="C35" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">31163</t>
@@ -11829,16 +10867,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A36" s="8"/>
+      <c r="B36" s="10"/>
       <c r="C36" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">31211</t>
@@ -11851,16 +10881,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A37" s="8"/>
+      <c r="B37" s="10"/>
       <c r="C37" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">31212</t>
@@ -11873,16 +10895,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A38" s="8"/>
+      <c r="B38" s="10"/>
       <c r="C38" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">31219</t>
@@ -11895,16 +10909,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">232</t>
-        </is>
-      </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 발효식품 제조업</t>
-        </is>
-      </c>
+      <c r="A39" s="8"/>
+      <c r="B39" s="10"/>
       <c r="C39" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">31221</t>
@@ -11939,16 +10945,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">233</t>
-        </is>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
-        </is>
-      </c>
+      <c r="A41" s="8"/>
+      <c r="B41" s="10"/>
       <c r="C41" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">31182</t>
@@ -11961,16 +10959,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">233</t>
-        </is>
-      </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 제조업</t>
-        </is>
-      </c>
+      <c r="A42" s="8"/>
+      <c r="B42" s="10"/>
       <c r="C42" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">31183</t>
@@ -12027,16 +11017,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">235</t>
-        </is>
-      </c>
-      <c r="B45" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 대체식품 제조업</t>
-        </is>
-      </c>
+      <c r="A45" s="8"/>
+      <c r="B45" s="10"/>
       <c r="C45" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">31199</t>
@@ -12071,16 +11053,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">239</t>
-        </is>
-      </c>
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품 제조업</t>
-        </is>
-      </c>
+      <c r="A47" s="8"/>
+      <c r="B47" s="10"/>
       <c r="C47" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">33200</t>
@@ -12115,16 +11089,8 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">240</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 동물용 의약품 제조업</t>
-        </is>
-      </c>
+      <c r="A49" s="8"/>
+      <c r="B49" s="10"/>
       <c r="C49" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">11172</t>
@@ -12203,16 +11169,8 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">299</t>
-        </is>
-      </c>
-      <c r="B53" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
-        </is>
-      </c>
+      <c r="A53" s="8"/>
+      <c r="B53" s="10"/>
       <c r="C53" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">33940</t>
@@ -12247,16 +11205,8 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">310</t>
-        </is>
-      </c>
-      <c r="B55" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
-        </is>
-      </c>
+      <c r="A55" s="8"/>
+      <c r="B55" s="10"/>
       <c r="C55" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">42230</t>
@@ -12269,16 +11219,8 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">310</t>
-        </is>
-      </c>
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생물자원·소재 판매·유통업</t>
-        </is>
-      </c>
+      <c r="A56" s="8"/>
+      <c r="B56" s="10"/>
       <c r="C56" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">42920</t>
@@ -12379,16 +11321,8 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">329</t>
-        </is>
-      </c>
-      <c r="B61" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 판매업</t>
-        </is>
-      </c>
+      <c r="A61" s="8"/>
+      <c r="B61" s="10"/>
       <c r="C61" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">13210</t>
@@ -12423,16 +11357,8 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">331</t>
-        </is>
-      </c>
-      <c r="B63" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 건강기능식품판매업</t>
-        </is>
-      </c>
+      <c r="A63" s="8"/>
+      <c r="B63" s="10"/>
       <c r="C63" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">43229</t>
@@ -12511,16 +11437,8 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">339</t>
-        </is>
-      </c>
-      <c r="B67" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품 판매업</t>
-        </is>
-      </c>
+      <c r="A67" s="8"/>
+      <c r="B67" s="10"/>
       <c r="C67" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">43290</t>
@@ -12621,16 +11539,8 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">411</t>
-        </is>
-      </c>
-      <c r="B72" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
-        </is>
-      </c>
+      <c r="A72" s="8"/>
+      <c r="B72" s="10"/>
       <c r="C72" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -12665,16 +11575,8 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">412</t>
-        </is>
-      </c>
-      <c r="B74" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
-        </is>
-      </c>
+      <c r="A74" s="8"/>
+      <c r="B74" s="10"/>
       <c r="C74" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -12709,16 +11611,8 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">413</t>
-        </is>
-      </c>
-      <c r="B76" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
-        </is>
-      </c>
+      <c r="A76" s="8"/>
+      <c r="B76" s="10"/>
       <c r="C76" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -12753,16 +11647,8 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">419</t>
-        </is>
-      </c>
-      <c r="B78" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
-        </is>
-      </c>
+      <c r="A78" s="8"/>
+      <c r="B78" s="10"/>
       <c r="C78" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -12797,16 +11683,8 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">421</t>
-        </is>
-      </c>
-      <c r="B80" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
-        </is>
-      </c>
+      <c r="A80" s="8"/>
+      <c r="B80" s="10"/>
       <c r="C80" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -12841,16 +11719,8 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">422</t>
-        </is>
-      </c>
-      <c r="B82" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
-        </is>
-      </c>
+      <c r="A82" s="8"/>
+      <c r="B82" s="10"/>
       <c r="C82" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -12885,16 +11755,8 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">423</t>
-        </is>
-      </c>
-      <c r="B84" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
-        </is>
-      </c>
+      <c r="A84" s="8"/>
+      <c r="B84" s="10"/>
       <c r="C84" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -12929,16 +11791,8 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">429</t>
-        </is>
-      </c>
-      <c r="B86" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
-        </is>
-      </c>
+      <c r="A86" s="8"/>
+      <c r="B86" s="10"/>
       <c r="C86" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -12973,16 +11827,8 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">431</t>
-        </is>
-      </c>
-      <c r="B88" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
-        </is>
-      </c>
+      <c r="A88" s="8"/>
+      <c r="B88" s="10"/>
       <c r="C88" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13017,16 +11863,8 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">432</t>
-        </is>
-      </c>
-      <c r="B90" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A90" s="8"/>
+      <c r="B90" s="10"/>
       <c r="C90" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13061,16 +11899,8 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">433</t>
-        </is>
-      </c>
-      <c r="B92" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
-        </is>
-      </c>
+      <c r="A92" s="8"/>
+      <c r="B92" s="10"/>
       <c r="C92" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13105,16 +11935,8 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">434</t>
-        </is>
-      </c>
-      <c r="B94" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A94" s="8"/>
+      <c r="B94" s="10"/>
       <c r="C94" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13149,16 +11971,8 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">435</t>
-        </is>
-      </c>
-      <c r="B96" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A96" s="8"/>
+      <c r="B96" s="10"/>
       <c r="C96" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13193,16 +12007,8 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">439</t>
-        </is>
-      </c>
-      <c r="B98" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A98" s="8"/>
+      <c r="B98" s="10"/>
       <c r="C98" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13237,16 +12043,8 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">441</t>
-        </is>
-      </c>
-      <c r="B100" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
-        </is>
-      </c>
+      <c r="A100" s="8"/>
+      <c r="B100" s="10"/>
       <c r="C100" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13281,16 +12079,8 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">449</t>
-        </is>
-      </c>
-      <c r="B102" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A102" s="8"/>
+      <c r="B102" s="10"/>
       <c r="C102" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13325,16 +12115,8 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">451</t>
-        </is>
-      </c>
-      <c r="B104" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A104" s="8"/>
+      <c r="B104" s="10"/>
       <c r="C104" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13369,16 +12151,8 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">452</t>
-        </is>
-      </c>
-      <c r="B106" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A106" s="8"/>
+      <c r="B106" s="10"/>
       <c r="C106" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13413,16 +12187,8 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">461</t>
-        </is>
-      </c>
-      <c r="B108" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
-        </is>
-      </c>
+      <c r="A108" s="8"/>
+      <c r="B108" s="10"/>
       <c r="C108" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13457,16 +12223,8 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">462</t>
-        </is>
-      </c>
-      <c r="B110" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
-        </is>
-      </c>
+      <c r="A110" s="8"/>
+      <c r="B110" s="10"/>
       <c r="C110" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13501,16 +12259,8 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">490</t>
-        </is>
-      </c>
-      <c r="B112" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 연구개발업</t>
-        </is>
-      </c>
+      <c r="A112" s="8"/>
+      <c r="B112" s="10"/>
       <c r="C112" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">82112</t>
@@ -13545,16 +12295,8 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">521</t>
-        </is>
-      </c>
-      <c r="B114" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
-        </is>
-      </c>
+      <c r="A114" s="8"/>
+      <c r="B114" s="10"/>
       <c r="C114" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">84202</t>
@@ -13589,16 +12331,8 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">529</t>
-        </is>
-      </c>
-      <c r="B116" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
-        </is>
-      </c>
+      <c r="A116" s="8"/>
+      <c r="B116" s="10"/>
       <c r="C116" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">84202</t>
@@ -13633,16 +12367,8 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">531</t>
-        </is>
-      </c>
-      <c r="B118" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 유기성 폐자원 처리업</t>
-        </is>
-      </c>
+      <c r="A118" s="8"/>
+      <c r="B118" s="10"/>
       <c r="C118" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">89120</t>
@@ -13677,16 +12403,8 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">532</t>
-        </is>
-      </c>
-      <c r="B120" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 방제·농업환경 관리업</t>
-        </is>
-      </c>
+      <c r="A120" s="8"/>
+      <c r="B120" s="10"/>
       <c r="C120" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">24299</t>
@@ -13721,16 +12439,8 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B122" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
+      <c r="A122" s="8"/>
+      <c r="B122" s="10"/>
       <c r="C122" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">89409</t>
@@ -13743,8 +12453,96 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="89">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A8:A13"/>
+    <mergeCell ref="B8:B13"/>
+    <mergeCell ref="A15:A19"/>
+    <mergeCell ref="B15:B19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="A34:A39"/>
+    <mergeCell ref="B34:B39"/>
+    <mergeCell ref="A40:A42"/>
+    <mergeCell ref="B40:B42"/>
+    <mergeCell ref="A44:A45"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="A48:A49"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="A52:A53"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="B54:B56"/>
+    <mergeCell ref="A60:A61"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="A62:A63"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="A71:A72"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="A73:A74"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="A75:A76"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="A79:A80"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="A83:A84"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="A85:A86"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="A87:A88"/>
+    <mergeCell ref="B87:B88"/>
+    <mergeCell ref="A89:A90"/>
+    <mergeCell ref="B89:B90"/>
+    <mergeCell ref="A91:A92"/>
+    <mergeCell ref="B91:B92"/>
+    <mergeCell ref="A93:A94"/>
+    <mergeCell ref="B93:B94"/>
+    <mergeCell ref="A95:A96"/>
+    <mergeCell ref="B95:B96"/>
+    <mergeCell ref="A97:A98"/>
+    <mergeCell ref="B97:B98"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="B99:B100"/>
+    <mergeCell ref="A101:A102"/>
+    <mergeCell ref="B101:B102"/>
+    <mergeCell ref="A103:A104"/>
+    <mergeCell ref="B103:B104"/>
+    <mergeCell ref="A105:A106"/>
+    <mergeCell ref="B105:B106"/>
+    <mergeCell ref="A107:A108"/>
+    <mergeCell ref="B107:B108"/>
+    <mergeCell ref="A109:A110"/>
+    <mergeCell ref="B109:B110"/>
+    <mergeCell ref="A111:A112"/>
+    <mergeCell ref="B111:B112"/>
+    <mergeCell ref="A113:A114"/>
+    <mergeCell ref="B113:B114"/>
+    <mergeCell ref="A115:A116"/>
+    <mergeCell ref="B115:B116"/>
+    <mergeCell ref="A117:A118"/>
+    <mergeCell ref="B117:B118"/>
+    <mergeCell ref="A119:A120"/>
+    <mergeCell ref="B119:B120"/>
+    <mergeCell ref="A121:A122"/>
+    <mergeCell ref="B121:B122"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13812,16 +12610,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">110</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 종자 생산업</t>
-        </is>
-      </c>
+      <c r="A5" s="8"/>
+      <c r="B5" s="10"/>
       <c r="C5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">7020</t>
@@ -13922,16 +12712,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">190</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생산업</t>
-        </is>
-      </c>
+      <c r="A10" s="8"/>
+      <c r="B10" s="10"/>
       <c r="C10" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3020</t>
@@ -13966,16 +12748,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">211</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A12" s="8"/>
+      <c r="B12" s="10"/>
       <c r="C12" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">2000</t>
@@ -13988,16 +12762,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">211</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A13" s="8"/>
+      <c r="B13" s="10"/>
       <c r="C13" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3030</t>
@@ -14010,16 +12776,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">211</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A14" s="8"/>
+      <c r="B14" s="10"/>
       <c r="C14" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3000</t>
@@ -14032,16 +12790,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">211</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A15" s="8"/>
+      <c r="B15" s="10"/>
       <c r="C15" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8010</t>
@@ -14076,16 +12826,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">212</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A17" s="8"/>
+      <c r="B17" s="10"/>
       <c r="C17" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3020</t>
@@ -14098,16 +12840,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">212</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A18" s="8"/>
+      <c r="B18" s="10"/>
       <c r="C18" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3030</t>
@@ -14120,16 +12854,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">212</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A19" s="8"/>
+      <c r="B19" s="10"/>
       <c r="C19" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">2000</t>
@@ -14142,16 +12868,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">212</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A20" s="8"/>
+      <c r="B20" s="10"/>
       <c r="C20" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8010</t>
@@ -14186,16 +12904,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">213</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 곤충 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A22" s="8"/>
+      <c r="B22" s="10"/>
       <c r="C22" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3050</t>
@@ -14208,16 +12918,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">213</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 곤충 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A23" s="8"/>
+      <c r="B23" s="10"/>
       <c r="C23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">2000</t>
@@ -14230,16 +12932,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">213</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 곤충 유래 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A24" s="8"/>
+      <c r="B24" s="10"/>
       <c r="C24" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8010</t>
@@ -14274,16 +12968,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">219</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A26" s="8"/>
+      <c r="B26" s="10"/>
       <c r="C26" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3000</t>
@@ -14296,16 +12982,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">219</t>
-        </is>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 소재 제조업</t>
-        </is>
-      </c>
+      <c r="A27" s="8"/>
+      <c r="B27" s="10"/>
       <c r="C27" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8010</t>
@@ -14406,16 +13084,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">229</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
-        </is>
-      </c>
+      <c r="A32" s="8"/>
+      <c r="B32" s="10"/>
       <c r="C32" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">2000</t>
@@ -14428,16 +13098,8 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">229</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 제조업</t>
-        </is>
-      </c>
+      <c r="A33" s="8"/>
+      <c r="B33" s="10"/>
       <c r="C33" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8010</t>
@@ -14648,16 +13310,8 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">292</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
-        </is>
-      </c>
+      <c r="A43" s="8"/>
+      <c r="B43" s="10"/>
       <c r="C43" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">2010</t>
@@ -14670,16 +13324,8 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">292</t>
-        </is>
-      </c>
-      <c r="B44" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 제조업</t>
-        </is>
-      </c>
+      <c r="A44" s="8"/>
+      <c r="B44" s="10"/>
       <c r="C44" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">2000</t>
@@ -14714,16 +13360,8 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">299</t>
-        </is>
-      </c>
-      <c r="B46" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
-        </is>
-      </c>
+      <c r="A46" s="8"/>
+      <c r="B46" s="10"/>
       <c r="C46" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">2000</t>
@@ -14736,16 +13374,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">299</t>
-        </is>
-      </c>
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그 외 기타 그린바이오 제품 제조업</t>
-        </is>
-      </c>
+      <c r="A47" s="8"/>
+      <c r="B47" s="10"/>
       <c r="C47" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">4000</t>
@@ -15044,16 +13674,8 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">411</t>
-        </is>
-      </c>
-      <c r="B61" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
-        </is>
-      </c>
+      <c r="A61" s="8"/>
+      <c r="B61" s="10"/>
       <c r="C61" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">7020</t>
@@ -15066,16 +13688,8 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">411</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 종자 연구개발업</t>
-        </is>
-      </c>
+      <c r="A62" s="8"/>
+      <c r="B62" s="10"/>
       <c r="C62" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15110,16 +13724,8 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">412</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 미생물 연구개발업</t>
-        </is>
-      </c>
+      <c r="A64" s="8"/>
+      <c r="B64" s="10"/>
       <c r="C64" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15154,16 +13760,8 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">413</t>
-        </is>
-      </c>
-      <c r="B66" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 곤충 연구개발업</t>
-        </is>
-      </c>
+      <c r="A66" s="8"/>
+      <c r="B66" s="10"/>
       <c r="C66" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15198,16 +13796,8 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">419</t>
-        </is>
-      </c>
-      <c r="B68" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 생물자원 연구개발업</t>
-        </is>
-      </c>
+      <c r="A68" s="8"/>
+      <c r="B68" s="10"/>
       <c r="C68" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15242,16 +13832,8 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">421</t>
-        </is>
-      </c>
-      <c r="B70" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오농약 연구개발업</t>
-        </is>
-      </c>
+      <c r="A70" s="8"/>
+      <c r="B70" s="10"/>
       <c r="C70" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15286,16 +13868,8 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">422</t>
-        </is>
-      </c>
-      <c r="B72" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오비료 연구개발업</t>
-        </is>
-      </c>
+      <c r="A72" s="8"/>
+      <c r="B72" s="10"/>
       <c r="C72" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15330,16 +13904,8 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">423</t>
-        </is>
-      </c>
-      <c r="B74" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">바이오사료 연구개발업</t>
-        </is>
-      </c>
+      <c r="A74" s="8"/>
+      <c r="B74" s="10"/>
       <c r="C74" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15374,16 +13940,8 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">429</t>
-        </is>
-      </c>
-      <c r="B76" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 농자재 연구개발업</t>
-        </is>
-      </c>
+      <c r="A76" s="8"/>
+      <c r="B76" s="10"/>
       <c r="C76" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15418,16 +13976,8 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">431</t>
-        </is>
-      </c>
-      <c r="B78" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
-        </is>
-      </c>
+      <c r="A78" s="8"/>
+      <c r="B78" s="10"/>
       <c r="C78" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3030</t>
@@ -15440,16 +13990,8 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">431</t>
-        </is>
-      </c>
-      <c r="B79" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
-        </is>
-      </c>
+      <c r="A79" s="8"/>
+      <c r="B79" s="10"/>
       <c r="C79" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3000</t>
@@ -15462,16 +14004,8 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">431</t>
-        </is>
-      </c>
-      <c r="B80" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 소재 연구개발업</t>
-        </is>
-      </c>
+      <c r="A80" s="8"/>
+      <c r="B80" s="10"/>
       <c r="C80" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15506,16 +14040,8 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">432</t>
-        </is>
-      </c>
-      <c r="B82" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 건강기능식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A82" s="8"/>
+      <c r="B82" s="10"/>
       <c r="C82" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15550,16 +14076,8 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">433</t>
-        </is>
-      </c>
-      <c r="B84" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
-        </is>
-      </c>
+      <c r="A84" s="8"/>
+      <c r="B84" s="10"/>
       <c r="C84" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3040</t>
@@ -15572,16 +14090,8 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">433</t>
-        </is>
-      </c>
-      <c r="B85" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 식품용 발효·미생물 기술 연구개발업</t>
-        </is>
-      </c>
+      <c r="A85" s="8"/>
+      <c r="B85" s="10"/>
       <c r="C85" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15616,16 +14126,8 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">434</t>
-        </is>
-      </c>
-      <c r="B87" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 대체식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A87" s="8"/>
+      <c r="B87" s="10"/>
       <c r="C87" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15660,16 +14162,8 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">435</t>
-        </is>
-      </c>
-      <c r="B89" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 특수영양·특수의료용도식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A89" s="8"/>
+      <c r="B89" s="10"/>
       <c r="C89" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15704,16 +14198,8 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">439</t>
-        </is>
-      </c>
-      <c r="B91" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 식품소재·식품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A91" s="8"/>
+      <c r="B91" s="10"/>
       <c r="C91" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15748,16 +14234,8 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">441</t>
-        </is>
-      </c>
-      <c r="B93" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동물용 바이오 백신 연구개발업</t>
-        </is>
-      </c>
+      <c r="A93" s="8"/>
+      <c r="B93" s="10"/>
       <c r="C93" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15792,16 +14270,8 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">449</t>
-        </is>
-      </c>
-      <c r="B95" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 동물용 의약품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A95" s="8"/>
+      <c r="B95" s="10"/>
       <c r="C95" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15836,16 +14306,8 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">451</t>
-        </is>
-      </c>
-      <c r="B97" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 향장제품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A97" s="8"/>
+      <c r="B97" s="10"/>
       <c r="C97" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15880,16 +14342,8 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">452</t>
-        </is>
-      </c>
-      <c r="B99" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A99" s="8"/>
+      <c r="B99" s="10"/>
       <c r="C99" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">2010</t>
@@ -15902,16 +14356,8 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">452</t>
-        </is>
-      </c>
-      <c r="B100" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A100" s="8"/>
+      <c r="B100" s="10"/>
       <c r="C100" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">2000</t>
@@ -15924,16 +14370,8 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">452</t>
-        </is>
-      </c>
-      <c r="B101" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 생활제품 연구개발업</t>
-        </is>
-      </c>
+      <c r="A101" s="8"/>
+      <c r="B101" s="10"/>
       <c r="C101" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -15968,16 +14406,8 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">461</t>
-        </is>
-      </c>
-      <c r="B103" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
-        </is>
-      </c>
+      <c r="A103" s="8"/>
+      <c r="B103" s="10"/>
       <c r="C103" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">4030</t>
@@ -15990,16 +14420,8 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">461</t>
-        </is>
-      </c>
-      <c r="B104" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
-        </is>
-      </c>
+      <c r="A104" s="8"/>
+      <c r="B104" s="10"/>
       <c r="C104" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">4000</t>
@@ -16012,16 +14434,8 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">461</t>
-        </is>
-      </c>
-      <c r="B105" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 환경서비스 연구개발업</t>
-        </is>
-      </c>
+      <c r="A105" s="8"/>
+      <c r="B105" s="10"/>
       <c r="C105" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8040</t>
@@ -16056,16 +14470,8 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">462</t>
-        </is>
-      </c>
-      <c r="B107" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 디지털서비스 연구개발업</t>
-        </is>
-      </c>
+      <c r="A107" s="8"/>
+      <c r="B107" s="10"/>
       <c r="C107" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8000</t>
@@ -16122,16 +14528,8 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">521</t>
-        </is>
-      </c>
-      <c r="B110" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">그린바이오 디지털육종 서비스업</t>
-        </is>
-      </c>
+      <c r="A110" s="8"/>
+      <c r="B110" s="10"/>
       <c r="C110" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8000</t>
@@ -16166,16 +14564,8 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">529</t>
-        </is>
-      </c>
-      <c r="B112" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 정보·데이터 서비스업</t>
-        </is>
-      </c>
+      <c r="A112" s="8"/>
+      <c r="B112" s="10"/>
       <c r="C112" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8000</t>
@@ -16254,16 +14644,8 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">590</t>
-        </is>
-      </c>
-      <c r="B116" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">기타 그린바이오 서비스업</t>
-        </is>
-      </c>
+      <c r="A116" s="8"/>
+      <c r="B116" s="10"/>
       <c r="C116" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">8000</t>
@@ -16276,8 +14658,72 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="65">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="A11:A15"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="A16:A20"/>
+    <mergeCell ref="B16:B20"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="A45:A47"/>
+    <mergeCell ref="B45:B47"/>
+    <mergeCell ref="A60:A62"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="A63:A64"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="A67:A68"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="A71:A72"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="A73:A74"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="A75:A76"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="A77:A80"/>
+    <mergeCell ref="B77:B80"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="B83:B85"/>
+    <mergeCell ref="A86:A87"/>
+    <mergeCell ref="B86:B87"/>
+    <mergeCell ref="A88:A89"/>
+    <mergeCell ref="B88:B89"/>
+    <mergeCell ref="A90:A91"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="A92:A93"/>
+    <mergeCell ref="B92:B93"/>
+    <mergeCell ref="A94:A95"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="A96:A97"/>
+    <mergeCell ref="B96:B97"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="A106:A107"/>
+    <mergeCell ref="B106:B107"/>
+    <mergeCell ref="A109:A110"/>
+    <mergeCell ref="B109:B110"/>
+    <mergeCell ref="A111:A112"/>
+    <mergeCell ref="B111:B112"/>
+    <mergeCell ref="A115:A116"/>
+    <mergeCell ref="B115:B116"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>